<commit_message>
Update: Ranking Data (13:48:16)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{926B95D7-CC23-4DE5-A4BC-195092CE60C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F542E15C-E41B-42BC-A313-B3BC98B569DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{0B284692-EF3A-4E3C-97E3-D2D5B039E418}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{0B431DE2-6DC2-485E-9BAF-6CB2F22AD1E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,6 +63,24 @@
     <t>진행된 경기 수</t>
   </si>
   <si>
+    <t>M008</t>
+  </si>
+  <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>Voor</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>첼시</t>
+  </si>
+  <si>
     <t>M017</t>
   </si>
   <si>
@@ -72,24 +90,6 @@
     <t>바이에른 뮌헨</t>
   </si>
   <si>
-    <t>Voor</t>
-  </si>
-  <si>
-    <t>17시즌</t>
-  </si>
-  <si>
-    <t>첼시</t>
-  </si>
-  <si>
-    <t>M008</t>
-  </si>
-  <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
     <t>대회종류</t>
   </si>
   <si>
@@ -120,6 +120,18 @@
     <t>1부리그</t>
   </si>
   <si>
+    <t>M015</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
     <t>M005</t>
   </si>
   <si>
@@ -127,18 +139,6 @@
   </si>
   <si>
     <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>M015</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
   </si>
   <si>
     <t>UEFA_B조</t>
@@ -731,7 +731,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87714EE8-F9C0-4E86-B6AA-D2C94CB42EDB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18A54BA4-1AB0-44D6-8321-B9770961B7FC}">
   <dimension ref="A1:Y29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -769,16 +769,16 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>1172.8479166666666</v>
+        <v>1030.9075</v>
       </c>
       <c r="E2">
-        <v>1211.8679166666666</v>
+        <v>1254.1175000000001</v>
       </c>
       <c r="F2">
-        <v>39.019999999999982</v>
+        <v>223.21000000000004</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="T2" t="s">
         <v>10</v>
@@ -801,16 +801,16 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>1030.9075</v>
+        <v>1172.8479166666666</v>
       </c>
       <c r="E3">
-        <v>1199.7375000000002</v>
+        <v>1211.8679166666666</v>
       </c>
       <c r="F3">
-        <v>168.83000000000015</v>
+        <v>39.019999999999982</v>
       </c>
       <c r="G3">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="T3" t="s">
         <v>16</v>
@@ -883,16 +883,16 @@
         <v>28</v>
       </c>
       <c r="D5">
-        <v>1050.1424999999999</v>
+        <v>1101.9679166666665</v>
       </c>
       <c r="E5">
-        <v>1104.5225</v>
+        <v>1097.2279166666665</v>
       </c>
       <c r="F5">
-        <v>54.380000000000109</v>
+        <v>-4.7400000000000091</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="T5" t="s">
         <v>29</v>
@@ -924,16 +924,16 @@
         <v>32</v>
       </c>
       <c r="D6">
-        <v>1101.9679166666665</v>
+        <v>1050.1424999999999</v>
       </c>
       <c r="E6">
-        <v>1097.2279166666665</v>
+        <v>1077.3425</v>
       </c>
       <c r="F6">
-        <v>-4.7400000000000091</v>
+        <v>27.200000000000045</v>
       </c>
       <c r="G6">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="T6" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
Update: Ranking Data (13:56:03)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F542E15C-E41B-42BC-A313-B3BC98B569DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E1CBFE3-FAC2-47E9-94D5-C3A0CCDAB6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{0B431DE2-6DC2-485E-9BAF-6CB2F22AD1E3}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{2FA9493D-59FE-4535-98AB-DFC0BEFCC6EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,6 +63,24 @@
     <t>진행된 경기 수</t>
   </si>
   <si>
+    <t>M017</t>
+  </si>
+  <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>Voor</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>첼시</t>
+  </si>
+  <si>
     <t>M008</t>
   </si>
   <si>
@@ -72,24 +90,6 @@
     <t>AS 로마</t>
   </si>
   <si>
-    <t>Voor</t>
-  </si>
-  <si>
-    <t>17시즌</t>
-  </si>
-  <si>
-    <t>첼시</t>
-  </si>
-  <si>
-    <t>M017</t>
-  </si>
-  <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
     <t>대회종류</t>
   </si>
   <si>
@@ -120,6 +120,18 @@
     <t>1부리그</t>
   </si>
   <si>
+    <t>M005</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
     <t>M015</t>
   </si>
   <si>
@@ -129,18 +141,6 @@
     <t>마인츠</t>
   </si>
   <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>M005</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
     <t>UEFA_B조</t>
   </si>
   <si>
@@ -156,6 +156,12 @@
     <t>UEFA Tournament</t>
   </si>
   <si>
+    <t>M001</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>M002</t>
   </si>
   <si>
@@ -163,12 +169,6 @@
   </si>
   <si>
     <t>프랑크푸르트</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>M001</t>
   </si>
   <si>
     <t>M011</t>
@@ -731,7 +731,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18A54BA4-1AB0-44D6-8321-B9770961B7FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{500F0083-F3E4-4900-9273-A9A22FF32C5D}">
   <dimension ref="A1:Y29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -769,16 +769,16 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>1030.9075</v>
+        <v>1172.8479166666666</v>
       </c>
       <c r="E2">
-        <v>1254.1175000000001</v>
+        <v>1211.8679166666666</v>
       </c>
       <c r="F2">
-        <v>223.21000000000004</v>
+        <v>39.019999999999982</v>
       </c>
       <c r="G2">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="T2" t="s">
         <v>10</v>
@@ -801,16 +801,16 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>1172.8479166666666</v>
+        <v>1030.9075</v>
       </c>
       <c r="E3">
-        <v>1211.8679166666666</v>
+        <v>1129.8975</v>
       </c>
       <c r="F3">
-        <v>39.019999999999982</v>
+        <v>98.990000000000009</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="T3" t="s">
         <v>16</v>
@@ -857,10 +857,10 @@
         <v>25</v>
       </c>
       <c r="U4">
-        <v>-34.92</v>
+        <v>0</v>
       </c>
       <c r="V4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W4">
         <v>0</v>
@@ -869,7 +869,7 @@
         <v>0</v>
       </c>
       <c r="Y4">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
@@ -883,16 +883,16 @@
         <v>28</v>
       </c>
       <c r="D5">
-        <v>1101.9679166666665</v>
+        <v>1050.1424999999999</v>
       </c>
       <c r="E5">
-        <v>1097.2279166666665</v>
+        <v>1104.5225</v>
       </c>
       <c r="F5">
-        <v>-4.7400000000000091</v>
+        <v>54.380000000000109</v>
       </c>
       <c r="G5">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="T5" t="s">
         <v>29</v>
@@ -924,16 +924,16 @@
         <v>32</v>
       </c>
       <c r="D6">
-        <v>1050.1424999999999</v>
+        <v>1101.9679166666665</v>
       </c>
       <c r="E6">
-        <v>1077.3425</v>
+        <v>1097.2279166666665</v>
       </c>
       <c r="F6">
-        <v>27.200000000000045</v>
+        <v>-4.7400000000000091</v>
       </c>
       <c r="G6">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="T6" t="s">
         <v>33</v>
@@ -1000,31 +1000,31 @@
         <v>38</v>
       </c>
       <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <v>1097.9099999999999</v>
+      </c>
+      <c r="E8">
+        <v>1062.04</v>
+      </c>
+      <c r="F8">
+        <v>-35.869999999999891</v>
+      </c>
+      <c r="G8">
+        <v>5</v>
+      </c>
+      <c r="T8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8">
-        <v>1123.425</v>
-      </c>
-      <c r="E8">
-        <v>1059.5549999999998</v>
-      </c>
-      <c r="F8">
-        <v>-63.870000000000118</v>
-      </c>
-      <c r="G8">
-        <v>9</v>
-      </c>
-      <c r="T8" t="s">
-        <v>41</v>
-      </c>
       <c r="U8">
-        <v>-70.790000000000006</v>
+        <v>-35.870000000000005</v>
       </c>
       <c r="V8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W8">
         <v>1</v>
@@ -1033,30 +1033,30 @@
         <v>1</v>
       </c>
       <c r="Y8">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
         <v>42</v>
       </c>
-      <c r="B9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
       <c r="D9">
-        <v>1097.9099999999999</v>
+        <v>1123.425</v>
       </c>
       <c r="E9">
-        <v>1027.1199999999999</v>
+        <v>1059.5549999999998</v>
       </c>
       <c r="F9">
-        <v>-70.789999999999964</v>
+        <v>-63.870000000000118</v>
       </c>
       <c r="G9">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (18:55:37)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E1CBFE3-FAC2-47E9-94D5-C3A0CCDAB6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFBA1361-C99F-417F-AE4F-751EBC3529D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{2FA9493D-59FE-4535-98AB-DFC0BEFCC6EA}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{1E2322A8-7595-4683-8184-CC75217B2796}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -108,6 +108,18 @@
     <t>패</t>
   </si>
   <si>
+    <t>M005</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
     <t>M009</t>
   </si>
   <si>
@@ -117,21 +129,27 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>M005</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
     <t>FA컵</t>
   </si>
   <si>
+    <t>M001</t>
+  </si>
+  <si>
+    <t>UEFA_B조</t>
+  </si>
+  <si>
+    <t>M006</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
     <t>M015</t>
   </si>
   <si>
@@ -141,27 +159,18 @@
     <t>마인츠</t>
   </si>
   <si>
-    <t>UEFA_B조</t>
-  </si>
-  <si>
-    <t>M006</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>M001</t>
-  </si>
-  <si>
     <t>전체 합계</t>
   </si>
   <si>
+    <t>M004</t>
+  </si>
+  <si>
+    <t>킹왕두</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
     <t>M002</t>
   </si>
   <si>
@@ -171,6 +180,15 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
+    <t>M021</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
     <t>M011</t>
   </si>
   <si>
@@ -180,15 +198,6 @@
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
-    <t>M004</t>
-  </si>
-  <si>
-    <t>킹왕두</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
     <t>M003</t>
   </si>
   <si>
@@ -198,15 +207,6 @@
     <t>인테르</t>
   </si>
   <si>
-    <t>M021</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>M014</t>
   </si>
   <si>
@@ -216,6 +216,15 @@
     <t>AS 모나코</t>
   </si>
   <si>
+    <t>M012</t>
+  </si>
+  <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
     <t>M010</t>
   </si>
   <si>
@@ -225,6 +234,15 @@
     <t>라치오</t>
   </si>
   <si>
+    <t>M027</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
     <t>M024</t>
   </si>
   <si>
@@ -234,13 +252,13 @@
     <t>셀틱 FC</t>
   </si>
   <si>
-    <t>M027</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
+    <t>M013</t>
+  </si>
+  <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
   </si>
   <si>
     <t>M030</t>
@@ -252,13 +270,58 @@
     <t>RC 셀타 비고</t>
   </si>
   <si>
-    <t>M013</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
+    <t>M028</t>
+  </si>
+  <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>M023</t>
+  </si>
+  <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
+  </si>
+  <si>
+    <t>M029</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>M025</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>M031</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>M026</t>
+  </si>
+  <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
   </si>
   <si>
     <t>M007</t>
@@ -268,69 +331,6 @@
   </si>
   <si>
     <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>M025</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>M012</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
-  </si>
-  <si>
-    <t>M023</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>M029</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>M028</t>
-  </si>
-  <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
-    <t>M031</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
-    <t>M026</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
   </si>
   <si>
     <t>M020</t>
@@ -731,7 +731,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{500F0083-F3E4-4900-9273-A9A22FF32C5D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEE2389-40DF-4AA8-B946-1D1B9B60827B}">
   <dimension ref="A1:Y29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -769,13 +769,13 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>1172.8479166666666</v>
+        <v>1110.1612500000001</v>
       </c>
       <c r="E2">
-        <v>1211.8679166666666</v>
+        <v>1149.50125</v>
       </c>
       <c r="F2">
-        <v>39.019999999999982</v>
+        <v>39.339999999999918</v>
       </c>
       <c r="G2">
         <v>4</v>
@@ -801,13 +801,13 @@
         <v>15</v>
       </c>
       <c r="D3">
-        <v>1030.9075</v>
+        <v>1031.54</v>
       </c>
       <c r="E3">
-        <v>1129.8975</v>
+        <v>1119.26</v>
       </c>
       <c r="F3">
-        <v>98.990000000000009</v>
+        <v>87.720000000000027</v>
       </c>
       <c r="G3">
         <v>11</v>
@@ -842,16 +842,16 @@
         <v>24</v>
       </c>
       <c r="D4">
-        <v>1071.9875</v>
+        <v>1050.075</v>
       </c>
       <c r="E4">
-        <v>1110.3074999999999</v>
+        <v>1098.0450000000001</v>
       </c>
       <c r="F4">
-        <v>38.319999999999936</v>
+        <v>47.970000000000027</v>
       </c>
       <c r="G4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="T4" t="s">
         <v>25</v>
@@ -883,22 +883,22 @@
         <v>28</v>
       </c>
       <c r="D5">
-        <v>1050.1424999999999</v>
+        <v>1039.04</v>
       </c>
       <c r="E5">
-        <v>1104.5225</v>
+        <v>1090.8799999999999</v>
       </c>
       <c r="F5">
-        <v>54.380000000000109</v>
+        <v>51.839999999999918</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="T5" t="s">
         <v>29</v>
       </c>
       <c r="U5">
-        <v>18.89</v>
+        <v>14.25</v>
       </c>
       <c r="V5">
         <v>1</v>
@@ -918,28 +918,28 @@
         <v>30</v>
       </c>
       <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>1124.6424999999999</v>
+      </c>
+      <c r="E6">
+        <v>1088.2524999999998</v>
+      </c>
+      <c r="F6">
+        <v>-36.3900000000001</v>
+      </c>
+      <c r="G6">
+        <v>5</v>
+      </c>
+      <c r="T6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6">
-        <v>1101.9679166666665</v>
-      </c>
-      <c r="E6">
-        <v>1097.2279166666665</v>
-      </c>
-      <c r="F6">
-        <v>-4.7400000000000091</v>
-      </c>
-      <c r="G6">
-        <v>18</v>
-      </c>
-      <c r="T6" t="s">
-        <v>33</v>
-      </c>
       <c r="U6">
-        <v>-54.760000000000005</v>
+        <v>-50.64</v>
       </c>
       <c r="V6">
         <v>4</v>
@@ -956,28 +956,28 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s">
         <v>34</v>
       </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
       <c r="D7">
-        <v>1023.9974999999999</v>
+        <v>1045.2150000000001</v>
       </c>
       <c r="E7">
-        <v>1065.5074999999999</v>
+        <v>1084.575</v>
       </c>
       <c r="F7">
-        <v>41.509999999999991</v>
+        <v>39.3599999999999</v>
       </c>
       <c r="G7">
         <v>5</v>
       </c>
       <c r="T7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="U7">
         <v>0</v>
@@ -997,31 +997,31 @@
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
         <v>38</v>
       </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
       <c r="D8">
-        <v>1097.9099999999999</v>
+        <v>1038.8812499999999</v>
       </c>
       <c r="E8">
-        <v>1062.04</v>
+        <v>1052.4512499999998</v>
       </c>
       <c r="F8">
-        <v>-35.869999999999891</v>
+        <v>13.569999999999936</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="T8" t="s">
         <v>39</v>
       </c>
       <c r="U8">
-        <v>-35.870000000000005</v>
+        <v>-36.39</v>
       </c>
       <c r="V8">
         <v>5</v>
@@ -1047,16 +1047,16 @@
         <v>42</v>
       </c>
       <c r="D9">
-        <v>1123.425</v>
+        <v>1055.5475000000001</v>
       </c>
       <c r="E9">
-        <v>1059.5549999999998</v>
+        <v>1028.7475000000002</v>
       </c>
       <c r="F9">
-        <v>-63.870000000000118</v>
+        <v>-26.799999999999955</v>
       </c>
       <c r="G9">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">
@@ -1070,16 +1070,16 @@
         <v>45</v>
       </c>
       <c r="D10">
-        <v>1008.0675000000001</v>
+        <v>1038.22</v>
       </c>
       <c r="E10">
-        <v>1020.1375000000002</v>
+        <v>1019.84</v>
       </c>
       <c r="F10">
-        <v>12.07000000000005</v>
+        <v>-18.379999999999995</v>
       </c>
       <c r="G10">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
@@ -1093,16 +1093,16 @@
         <v>48</v>
       </c>
       <c r="D11">
-        <v>1050.5300000000002</v>
+        <v>1001.55125</v>
       </c>
       <c r="E11">
-        <v>1017.0500000000002</v>
+        <v>1001.55125</v>
       </c>
       <c r="F11">
-        <v>-33.480000000000018</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.3">
@@ -1116,16 +1116,16 @@
         <v>51</v>
       </c>
       <c r="D12">
-        <v>1050.0379166666667</v>
+        <v>993.26</v>
       </c>
       <c r="E12">
-        <v>1002.5179166666667</v>
+        <v>1000.7</v>
       </c>
       <c r="F12">
-        <v>-47.519999999999982</v>
+        <v>7.4400000000000546</v>
       </c>
       <c r="G12">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
@@ -1139,16 +1139,16 @@
         <v>54</v>
       </c>
       <c r="D13">
-        <v>993.23791666666671</v>
+        <v>1030.00125</v>
       </c>
       <c r="E13">
-        <v>993.23791666666671</v>
+        <v>999.64125000000001</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>-30.360000000000014</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
@@ -1162,13 +1162,13 @@
         <v>57</v>
       </c>
       <c r="D14">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E14">
-        <v>967.42965909090901</v>
+        <v>985.96090909090901</v>
       </c>
       <c r="F14">
-        <v>57.639999999999986</v>
+        <v>50.159999999999968</v>
       </c>
       <c r="G14">
         <v>11</v>
@@ -1185,16 +1185,16 @@
         <v>60</v>
       </c>
       <c r="D15">
-        <v>1013.63</v>
+        <v>970.9425</v>
       </c>
       <c r="E15">
-        <v>965.14</v>
+        <v>970.9425</v>
       </c>
       <c r="F15">
-        <v>-48.490000000000009</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.3">
@@ -1208,16 +1208,16 @@
         <v>63</v>
       </c>
       <c r="D16">
-        <v>909.78965909090903</v>
+        <v>1007.8275000000001</v>
       </c>
       <c r="E16">
-        <v>960.36965909090895</v>
+        <v>967.49750000000006</v>
       </c>
       <c r="F16">
-        <v>50.579999999999927</v>
+        <v>-40.330000000000041</v>
       </c>
       <c r="G16">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1231,16 +1231,16 @@
         <v>66</v>
       </c>
       <c r="D17">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E17">
-        <v>944.60965909090908</v>
+        <v>959.55090909090904</v>
       </c>
       <c r="F17">
-        <v>34.82000000000005</v>
+        <v>23.75</v>
       </c>
       <c r="G17">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1254,16 +1254,16 @@
         <v>69</v>
       </c>
       <c r="D18">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E18">
-        <v>925.00965909090905</v>
+        <v>955.31090909090904</v>
       </c>
       <c r="F18">
-        <v>15.220000000000027</v>
+        <v>19.509999999999991</v>
       </c>
       <c r="G18">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1277,13 +1277,13 @@
         <v>72</v>
       </c>
       <c r="D19">
-        <v>937.65291666666667</v>
+        <v>955.46125000000006</v>
       </c>
       <c r="E19">
-        <v>922.9929166666667</v>
+        <v>946.26125000000002</v>
       </c>
       <c r="F19">
-        <v>-14.659999999999968</v>
+        <v>-9.2000000000000455</v>
       </c>
       <c r="G19">
         <v>6</v>
@@ -1300,16 +1300,16 @@
         <v>75</v>
       </c>
       <c r="D20">
-        <v>933.4425</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E20">
-        <v>911.16250000000002</v>
+        <v>938.98090909090899</v>
       </c>
       <c r="F20">
-        <v>-22.279999999999973</v>
+        <v>3.17999999999995</v>
       </c>
       <c r="G20">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1323,16 +1323,16 @@
         <v>78</v>
       </c>
       <c r="D21">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E21">
-        <v>909.80965909090901</v>
+        <v>935.970909090909</v>
       </c>
       <c r="F21">
-        <v>1.999999999998181E-2</v>
+        <v>0.16999999999995907</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1346,10 +1346,10 @@
         <v>81</v>
       </c>
       <c r="D22">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E22">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1369,10 +1369,10 @@
         <v>84</v>
       </c>
       <c r="D23">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E23">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1392,16 +1392,16 @@
         <v>87</v>
       </c>
       <c r="D24">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E24">
-        <v>909.78965909090903</v>
+        <v>935.20090909090902</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>-0.60000000000002274</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1415,16 +1415,16 @@
         <v>90</v>
       </c>
       <c r="D25">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E25">
-        <v>909.78965909090903</v>
+        <v>930.53090909090906</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>-5.2699999999999818</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1438,16 +1438,16 @@
         <v>93</v>
       </c>
       <c r="D26">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E26">
-        <v>904.82965909090899</v>
+        <v>929.77090909090907</v>
       </c>
       <c r="F26">
-        <v>-4.9600000000000364</v>
+        <v>-6.0299999999999727</v>
       </c>
       <c r="G26">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1461,16 +1461,16 @@
         <v>96</v>
       </c>
       <c r="D27">
-        <v>909.78965909090903</v>
+        <v>982.40249999999992</v>
       </c>
       <c r="E27">
-        <v>900.38965909090905</v>
+        <v>929.50249999999994</v>
       </c>
       <c r="F27">
-        <v>-9.3999999999999773</v>
+        <v>-52.899999999999977</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1484,16 +1484,16 @@
         <v>99</v>
       </c>
       <c r="D28">
-        <v>911.98791666666671</v>
+        <v>944.29124999999999</v>
       </c>
       <c r="E28">
-        <v>883.9979166666667</v>
+        <v>919.02125000000001</v>
       </c>
       <c r="F28">
-        <v>-27.990000000000009</v>
+        <v>-25.269999999999982</v>
       </c>
       <c r="G28">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1507,13 +1507,13 @@
         <v>102</v>
       </c>
       <c r="D29">
-        <v>909.78965909090903</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E29">
-        <v>861.78965909090903</v>
+        <v>891.18090909090904</v>
       </c>
       <c r="F29">
-        <v>-48</v>
+        <v>-44.620000000000005</v>
       </c>
       <c r="G29">
         <v>3</v>

</xml_diff>

<commit_message>
Update: Ranking Data (19:26:12)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFBA1361-C99F-417F-AE4F-751EBC3529D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8AC273F-3F3E-44EA-973B-140D4B292B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{1E2322A8-7595-4683-8184-CC75217B2796}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{E7E6E5DF-5D9E-4CA4-B6B9-20C5672ECCB7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -72,70 +72,70 @@
     <t>바이에른 뮌헨</t>
   </si>
   <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>M008</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
+    <t>승</t>
+  </si>
+  <si>
+    <t>무</t>
+  </si>
+  <si>
+    <t>패</t>
+  </si>
+  <si>
+    <t>M005</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
+    <t>M009</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>M001</t>
+  </si>
+  <si>
     <t>Voor</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>첼시</t>
   </si>
   <si>
-    <t>M008</t>
-  </si>
-  <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>승</t>
-  </si>
-  <si>
-    <t>무</t>
-  </si>
-  <si>
-    <t>패</t>
-  </si>
-  <si>
-    <t>M005</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>M009</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>M001</t>
-  </si>
-  <si>
-    <t>UEFA_B조</t>
+    <t>UEFA_A조</t>
   </si>
   <si>
     <t>M006</t>
@@ -180,6 +180,15 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
+    <t>M011</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
     <t>M021</t>
   </si>
   <si>
@@ -189,15 +198,6 @@
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>M011</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
     <t>M003</t>
   </si>
   <si>
@@ -216,6 +216,51 @@
     <t>AS 모나코</t>
   </si>
   <si>
+    <t>M027</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>M010</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>M028</t>
+  </si>
+  <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>M013</t>
+  </si>
+  <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
+    <t>M024</t>
+  </si>
+  <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
     <t>M012</t>
   </si>
   <si>
@@ -225,40 +270,31 @@
     <t>함부르크SV</t>
   </si>
   <si>
-    <t>M010</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>M027</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>M024</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
-    <t>M013</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
+    <t>M023</t>
+  </si>
+  <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
+  </si>
+  <si>
+    <t>M029</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>M025</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
   </si>
   <si>
     <t>M030</t>
@@ -270,40 +306,13 @@
     <t>RC 셀타 비고</t>
   </si>
   <si>
-    <t>M028</t>
-  </si>
-  <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
-    <t>M023</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>M029</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>M025</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
+    <t>M007</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
   </si>
   <si>
     <t>M031</t>
@@ -322,15 +331,6 @@
   </si>
   <si>
     <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>M007</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
   </si>
   <si>
     <t>M020</t>
@@ -731,11 +731,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEE2389-40DF-4AA8-B946-1D1B9B60827B}">
-  <dimension ref="A1:Y29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D33C20C-3036-4A76-A781-E575993374F4}">
+  <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -758,7 +758,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -780,66 +780,66 @@
       <c r="G2">
         <v>4</v>
       </c>
-      <c r="T2" t="s">
+      <c r="I2" t="s">
         <v>10</v>
       </c>
-      <c r="V2" t="s">
+      <c r="K2" t="s">
         <v>11</v>
       </c>
-      <c r="W2" t="s">
+      <c r="L2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>1031.54</v>
       </c>
       <c r="E3">
-        <v>1119.26</v>
+        <v>1119.54</v>
       </c>
       <c r="F3">
-        <v>87.720000000000027</v>
+        <v>88</v>
       </c>
       <c r="G3">
         <v>11</v>
       </c>
-      <c r="T3" t="s">
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+      <c r="K3" t="s">
         <v>16</v>
       </c>
-      <c r="U3" t="s">
+      <c r="L3" t="s">
         <v>17</v>
       </c>
-      <c r="V3" t="s">
+      <c r="M3" t="s">
         <v>18</v>
       </c>
-      <c r="W3" t="s">
+      <c r="N3" t="s">
         <v>19</v>
       </c>
-      <c r="X3" t="s">
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
       </c>
       <c r="D4">
         <v>1050.075</v>
@@ -853,75 +853,75 @@
       <c r="G4">
         <v>4</v>
       </c>
-      <c r="T4" t="s">
+      <c r="I4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J4">
+        <v>57.1</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>2</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
         <v>25</v>
       </c>
-      <c r="U4">
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
-        <v>0</v>
-      </c>
-      <c r="Y4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
       </c>
       <c r="D5">
         <v>1039.04</v>
       </c>
       <c r="E5">
-        <v>1090.8799999999999</v>
+        <v>1090.82</v>
       </c>
       <c r="F5">
-        <v>51.839999999999918</v>
+        <v>51.779999999999973</v>
       </c>
       <c r="G5">
         <v>8</v>
       </c>
-      <c r="T5" t="s">
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5">
+        <v>17.93</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" t="s">
         <v>29</v>
       </c>
-      <c r="U5">
-        <v>14.25</v>
-      </c>
-      <c r="V5">
-        <v>1</v>
-      </c>
-      <c r="W5">
-        <v>1</v>
-      </c>
-      <c r="X5">
-        <v>0</v>
-      </c>
-      <c r="Y5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C6" t="s">
         <v>30</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
       </c>
       <c r="D6">
         <v>1124.6424999999999</v>
@@ -935,26 +935,26 @@
       <c r="G6">
         <v>5</v>
       </c>
-      <c r="T6" t="s">
+      <c r="I6" t="s">
         <v>31</v>
       </c>
-      <c r="U6">
-        <v>-50.64</v>
-      </c>
-      <c r="V6">
+      <c r="J6">
+        <v>12.969999999999999</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
         <v>4</v>
       </c>
-      <c r="W6">
+      <c r="M6">
         <v>0</v>
       </c>
-      <c r="X6">
-        <v>1</v>
-      </c>
-      <c r="Y6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="N6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -968,34 +968,34 @@
         <v>1045.2150000000001</v>
       </c>
       <c r="E7">
-        <v>1084.575</v>
+        <v>1084.4150000000002</v>
       </c>
       <c r="F7">
-        <v>39.3599999999999</v>
+        <v>39.200000000000045</v>
       </c>
       <c r="G7">
         <v>5</v>
       </c>
-      <c r="T7" t="s">
+      <c r="I7" t="s">
         <v>35</v>
       </c>
-      <c r="U7">
+      <c r="J7">
         <v>0</v>
       </c>
-      <c r="V7">
+      <c r="K7">
         <v>0</v>
       </c>
-      <c r="W7">
+      <c r="L7">
         <v>0</v>
       </c>
-      <c r="X7">
+      <c r="M7">
         <v>0</v>
       </c>
-      <c r="Y7">
+      <c r="N7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1009,34 +1009,34 @@
         <v>1038.8812499999999</v>
       </c>
       <c r="E8">
-        <v>1052.4512499999998</v>
+        <v>1056.81125</v>
       </c>
       <c r="F8">
-        <v>13.569999999999936</v>
+        <v>17.930000000000064</v>
       </c>
       <c r="G8">
         <v>18</v>
       </c>
-      <c r="T8" t="s">
+      <c r="I8" t="s">
         <v>39</v>
       </c>
-      <c r="U8">
-        <v>-36.39</v>
-      </c>
-      <c r="V8">
-        <v>5</v>
-      </c>
-      <c r="W8">
-        <v>1</v>
-      </c>
-      <c r="X8">
-        <v>1</v>
-      </c>
-      <c r="Y8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="J8">
+        <v>88</v>
+      </c>
+      <c r="K8">
+        <v>11</v>
+      </c>
+      <c r="L8">
+        <v>7</v>
+      </c>
+      <c r="M8">
+        <v>2</v>
+      </c>
+      <c r="N8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -1050,16 +1050,16 @@
         <v>1055.5475000000001</v>
       </c>
       <c r="E9">
-        <v>1028.7475000000002</v>
+        <v>1028.7775000000001</v>
       </c>
       <c r="F9">
-        <v>-26.799999999999955</v>
+        <v>-26.769999999999982</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -1073,16 +1073,16 @@
         <v>1038.22</v>
       </c>
       <c r="E10">
-        <v>1019.84</v>
+        <v>1019.7900000000001</v>
       </c>
       <c r="F10">
-        <v>-18.379999999999995</v>
+        <v>-18.42999999999995</v>
       </c>
       <c r="G10">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>46</v>
       </c>
@@ -1093,19 +1093,19 @@
         <v>48</v>
       </c>
       <c r="D11">
-        <v>1001.55125</v>
+        <v>993.26</v>
       </c>
       <c r="E11">
-        <v>1001.55125</v>
+        <v>1012.97</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>19.710000000000036</v>
       </c>
       <c r="G11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>49</v>
       </c>
@@ -1116,19 +1116,19 @@
         <v>51</v>
       </c>
       <c r="D12">
-        <v>993.26</v>
+        <v>1001.55125</v>
       </c>
       <c r="E12">
-        <v>1000.7</v>
+        <v>1001.55125</v>
       </c>
       <c r="F12">
-        <v>7.4400000000000546</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -1142,16 +1142,16 @@
         <v>1030.00125</v>
       </c>
       <c r="E13">
-        <v>999.64125000000001</v>
+        <v>998.44125000000008</v>
       </c>
       <c r="F13">
-        <v>-30.360000000000014</v>
+        <v>-31.559999999999945</v>
       </c>
       <c r="G13">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1165,16 +1165,16 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E14">
-        <v>985.96090909090901</v>
+        <v>991.20090909090902</v>
       </c>
       <c r="F14">
-        <v>50.159999999999968</v>
+        <v>55.399999999999977</v>
       </c>
       <c r="G14">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>58</v>
       </c>
@@ -1185,19 +1185,19 @@
         <v>60</v>
       </c>
       <c r="D15">
-        <v>970.9425</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E15">
-        <v>970.9425</v>
+        <v>979.00090909090909</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>43.200000000000045</v>
       </c>
       <c r="G15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>61</v>
       </c>
@@ -1234,13 +1234,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E17">
-        <v>959.55090909090904</v>
+        <v>958.09090909090901</v>
       </c>
       <c r="F17">
-        <v>23.75</v>
+        <v>22.289999999999964</v>
       </c>
       <c r="G17">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1254,16 +1254,16 @@
         <v>69</v>
       </c>
       <c r="D18">
-        <v>935.80090909090904</v>
+        <v>955.46125000000006</v>
       </c>
       <c r="E18">
-        <v>955.31090909090904</v>
+        <v>956.69125000000008</v>
       </c>
       <c r="F18">
-        <v>19.509999999999991</v>
+        <v>1.2300000000000182</v>
       </c>
       <c r="G18">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1277,16 +1277,16 @@
         <v>72</v>
       </c>
       <c r="D19">
-        <v>955.46125000000006</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E19">
-        <v>946.26125000000002</v>
+        <v>955.31090909090904</v>
       </c>
       <c r="F19">
-        <v>-9.2000000000000455</v>
+        <v>19.509999999999991</v>
       </c>
       <c r="G19">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1300,16 +1300,16 @@
         <v>75</v>
       </c>
       <c r="D20">
-        <v>935.80090909090904</v>
+        <v>970.9425</v>
       </c>
       <c r="E20">
-        <v>938.98090909090899</v>
+        <v>954.35249999999996</v>
       </c>
       <c r="F20">
-        <v>3.17999999999995</v>
+        <v>-16.590000000000032</v>
       </c>
       <c r="G20">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1326,13 +1326,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E21">
-        <v>935.970909090909</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="F21">
-        <v>0.16999999999995907</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1372,13 +1372,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E23">
-        <v>935.80090909090904</v>
+        <v>933.23090909090899</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>-2.57000000000005</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -1395,13 +1395,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E24">
-        <v>935.20090909090902</v>
+        <v>929.470909090909</v>
       </c>
       <c r="F24">
-        <v>-0.60000000000002274</v>
+        <v>-6.3300000000000409</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1415,16 +1415,16 @@
         <v>90</v>
       </c>
       <c r="D25">
-        <v>935.80090909090904</v>
+        <v>982.40249999999992</v>
       </c>
       <c r="E25">
-        <v>930.53090909090906</v>
+        <v>928.94249999999988</v>
       </c>
       <c r="F25">
-        <v>-5.2699999999999818</v>
+        <v>-53.460000000000036</v>
       </c>
       <c r="G25">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1441,13 +1441,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E26">
-        <v>929.77090909090907</v>
+        <v>916.09090909090901</v>
       </c>
       <c r="F26">
-        <v>-6.0299999999999727</v>
+        <v>-19.710000000000036</v>
       </c>
       <c r="G26">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1461,16 +1461,16 @@
         <v>96</v>
       </c>
       <c r="D27">
-        <v>982.40249999999992</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E27">
-        <v>929.50249999999994</v>
+        <v>912.18090909090904</v>
       </c>
       <c r="F27">
-        <v>-52.899999999999977</v>
+        <v>-23.620000000000005</v>
       </c>
       <c r="G27">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1487,10 +1487,10 @@
         <v>944.29124999999999</v>
       </c>
       <c r="E28">
-        <v>919.02125000000001</v>
+        <v>908.15125</v>
       </c>
       <c r="F28">
-        <v>-25.269999999999982</v>
+        <v>-36.139999999999986</v>
       </c>
       <c r="G28">
         <v>25</v>
@@ -1510,10 +1510,10 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E29">
-        <v>891.18090909090904</v>
+        <v>892.88090909090909</v>
       </c>
       <c r="F29">
-        <v>-44.620000000000005</v>
+        <v>-42.919999999999959</v>
       </c>
       <c r="G29">
         <v>3</v>

</xml_diff>

<commit_message>
Update: Ranking Data (07:29:13)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8AC273F-3F3E-44EA-973B-140D4B292B6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEF99447-5796-4C8A-98FA-6E9E7C1AD323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{E7E6E5DF-5D9E-4CA4-B6B9-20C5672ECCB7}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{89A005C2-DE1A-4625-A69F-C8B9F99BD438}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -81,25 +81,37 @@
     <t>AS 로마</t>
   </si>
   <si>
+    <t>M001</t>
+  </si>
+  <si>
+    <t>Voor</t>
+  </si>
+  <si>
+    <t>첼시</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
+    <t>승</t>
+  </si>
+  <si>
+    <t>무</t>
+  </si>
+  <si>
+    <t>패</t>
+  </si>
+  <si>
     <t>M008</t>
   </si>
   <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>승</t>
-  </si>
-  <si>
-    <t>무</t>
-  </si>
-  <si>
-    <t>패</t>
+    <t>1부리그</t>
   </si>
   <si>
     <t>M005</t>
@@ -111,7 +123,7 @@
     <t>AC 밀란</t>
   </si>
   <si>
-    <t>1부리그</t>
+    <t>FA컵</t>
   </si>
   <si>
     <t>M009</t>
@@ -123,18 +135,6 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>M001</t>
-  </si>
-  <si>
-    <t>Voor</t>
-  </si>
-  <si>
-    <t>첼시</t>
-  </si>
-  <si>
     <t>UEFA_A조</t>
   </si>
   <si>
@@ -198,6 +198,15 @@
     <t>SSC 나폴리</t>
   </si>
   <si>
+    <t>M028</t>
+  </si>
+  <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
     <t>M003</t>
   </si>
   <si>
@@ -207,6 +216,15 @@
     <t>인테르</t>
   </si>
   <si>
+    <t>M027</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
     <t>M014</t>
   </si>
   <si>
@@ -216,15 +234,6 @@
     <t>AS 모나코</t>
   </si>
   <si>
-    <t>M027</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
     <t>M010</t>
   </si>
   <si>
@@ -234,13 +243,49 @@
     <t>라치오</t>
   </si>
   <si>
-    <t>M028</t>
-  </si>
-  <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
+    <t>M012</t>
+  </si>
+  <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>M024</t>
+  </si>
+  <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>M030</t>
+  </si>
+  <si>
+    <t>스페인전도사</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
+    <t>M029</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>M025</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
   </si>
   <si>
     <t>M013</t>
@@ -252,22 +297,31 @@
     <t>경남 FC</t>
   </si>
   <si>
-    <t>M024</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
-    <t>M012</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
+    <t>M031</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>M026</t>
+  </si>
+  <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>M007</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
   </si>
   <si>
     <t>M023</t>
@@ -277,60 +331,6 @@
   </si>
   <si>
     <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>M029</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>M025</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>M030</t>
-  </si>
-  <si>
-    <t>스페인전도사</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
-  </si>
-  <si>
-    <t>M007</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>M031</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
-    <t>M026</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
   </si>
   <si>
     <t>M020</t>
@@ -731,7 +731,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D33C20C-3036-4A76-A781-E575993374F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A7087EC-CDAB-4A93-B765-F8B69F14006C}">
   <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -795,63 +795,63 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>1031.54</v>
+        <v>1124.6424999999999</v>
       </c>
       <c r="E3">
-        <v>1119.54</v>
+        <v>1129.0625</v>
       </c>
       <c r="F3">
-        <v>88</v>
+        <v>4.4200000000000728</v>
       </c>
       <c r="G3">
         <v>11</v>
       </c>
       <c r="I3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="L3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="N3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D4">
-        <v>1050.075</v>
+        <v>1031.54</v>
       </c>
       <c r="E4">
-        <v>1098.0450000000001</v>
+        <v>1119.54</v>
       </c>
       <c r="F4">
-        <v>47.970000000000027</v>
+        <v>88</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="I4" t="s">
         <v>23</v>
@@ -883,16 +883,16 @@
         <v>26</v>
       </c>
       <c r="D5">
-        <v>1039.04</v>
+        <v>1050.075</v>
       </c>
       <c r="E5">
-        <v>1090.82</v>
+        <v>1092.385</v>
       </c>
       <c r="F5">
-        <v>51.779999999999973</v>
+        <v>42.309999999999945</v>
       </c>
       <c r="G5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I5" t="s">
         <v>27</v>
@@ -924,16 +924,16 @@
         <v>30</v>
       </c>
       <c r="D6">
-        <v>1124.6424999999999</v>
+        <v>1039.04</v>
       </c>
       <c r="E6">
-        <v>1088.2524999999998</v>
+        <v>1090.82</v>
       </c>
       <c r="F6">
-        <v>-36.3900000000001</v>
+        <v>51.779999999999973</v>
       </c>
       <c r="G6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I6" t="s">
         <v>31</v>
@@ -1096,13 +1096,13 @@
         <v>993.26</v>
       </c>
       <c r="E11">
-        <v>1012.97</v>
+        <v>1006.55</v>
       </c>
       <c r="F11">
-        <v>19.710000000000036</v>
+        <v>13.289999999999964</v>
       </c>
       <c r="G11">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1139,16 +1139,16 @@
         <v>54</v>
       </c>
       <c r="D13">
-        <v>1030.00125</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E13">
-        <v>998.44125000000008</v>
+        <v>999.04090909090905</v>
       </c>
       <c r="F13">
-        <v>-31.559999999999945</v>
+        <v>63.240000000000009</v>
       </c>
       <c r="G13">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -1162,16 +1162,16 @@
         <v>57</v>
       </c>
       <c r="D14">
-        <v>935.80090909090904</v>
+        <v>1030.00125</v>
       </c>
       <c r="E14">
-        <v>991.20090909090902</v>
+        <v>998.44125000000008</v>
       </c>
       <c r="F14">
-        <v>55.399999999999977</v>
+        <v>-31.559999999999945</v>
       </c>
       <c r="G14">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1188,13 +1188,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E15">
-        <v>979.00090909090909</v>
+        <v>976.26090909090908</v>
       </c>
       <c r="F15">
-        <v>43.200000000000045</v>
+        <v>40.460000000000036</v>
       </c>
       <c r="G15">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -1208,16 +1208,16 @@
         <v>63</v>
       </c>
       <c r="D16">
-        <v>1007.8275000000001</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E16">
-        <v>967.49750000000006</v>
+        <v>971.24090909090899</v>
       </c>
       <c r="F16">
-        <v>-40.330000000000041</v>
+        <v>35.439999999999941</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1231,16 +1231,16 @@
         <v>66</v>
       </c>
       <c r="D17">
-        <v>935.80090909090904</v>
+        <v>1007.8275000000001</v>
       </c>
       <c r="E17">
-        <v>958.09090909090901</v>
+        <v>967.49750000000006</v>
       </c>
       <c r="F17">
-        <v>22.289999999999964</v>
+        <v>-40.330000000000041</v>
       </c>
       <c r="G17">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1254,16 +1254,16 @@
         <v>69</v>
       </c>
       <c r="D18">
-        <v>955.46125000000006</v>
+        <v>970.9425</v>
       </c>
       <c r="E18">
-        <v>956.69125000000008</v>
+        <v>958.61249999999995</v>
       </c>
       <c r="F18">
-        <v>1.2300000000000182</v>
+        <v>-12.330000000000041</v>
       </c>
       <c r="G18">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1300,16 +1300,16 @@
         <v>75</v>
       </c>
       <c r="D20">
-        <v>970.9425</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E20">
-        <v>954.35249999999996</v>
+        <v>948.55090909090904</v>
       </c>
       <c r="F20">
-        <v>-16.590000000000032</v>
+        <v>12.75</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1349,13 +1349,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E22">
-        <v>935.80090909090904</v>
+        <v>933.23090909090899</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>-2.57000000000005</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -1369,16 +1369,16 @@
         <v>84</v>
       </c>
       <c r="D23">
-        <v>935.80090909090904</v>
+        <v>955.46125000000006</v>
       </c>
       <c r="E23">
-        <v>933.23090909090899</v>
+        <v>928.02125000000001</v>
       </c>
       <c r="F23">
-        <v>-2.57000000000005</v>
+        <v>-27.440000000000055</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -1395,13 +1395,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E24">
-        <v>929.470909090909</v>
+        <v>926.50090909090909</v>
       </c>
       <c r="F24">
-        <v>-6.3300000000000409</v>
+        <v>-9.2999999999999545</v>
       </c>
       <c r="G24">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1415,16 +1415,16 @@
         <v>90</v>
       </c>
       <c r="D25">
-        <v>982.40249999999992</v>
+        <v>935.80090909090904</v>
       </c>
       <c r="E25">
-        <v>928.94249999999988</v>
+        <v>918.03090909090906</v>
       </c>
       <c r="F25">
-        <v>-53.460000000000036</v>
+        <v>-17.769999999999982</v>
       </c>
       <c r="G25">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1438,16 +1438,16 @@
         <v>93</v>
       </c>
       <c r="D26">
-        <v>935.80090909090904</v>
+        <v>982.40249999999992</v>
       </c>
       <c r="E26">
-        <v>916.09090909090901</v>
+        <v>913.26249999999993</v>
       </c>
       <c r="F26">
-        <v>-19.710000000000036</v>
+        <v>-69.139999999999986</v>
       </c>
       <c r="G26">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1464,13 +1464,13 @@
         <v>935.80090909090904</v>
       </c>
       <c r="E27">
-        <v>912.18090909090904</v>
+        <v>906.38090909090909</v>
       </c>
       <c r="F27">
-        <v>-23.620000000000005</v>
+        <v>-29.419999999999959</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1487,10 +1487,10 @@
         <v>944.29124999999999</v>
       </c>
       <c r="E28">
-        <v>908.15125</v>
+        <v>902.21124999999995</v>
       </c>
       <c r="F28">
-        <v>-36.139999999999986</v>
+        <v>-42.080000000000041</v>
       </c>
       <c r="G28">
         <v>25</v>

</xml_diff>

<commit_message>
Update: Ranking Data (12:50:44)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E0CB50F-7544-4FB3-A343-190C9CB2D659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{20541DAA-3827-4C35-A8E5-C1149149BDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{CFB5E9A9-399B-418B-BA05-9F1BFDF5E835}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{1D6FC72D-549F-4B7E-ADBB-74BD5CDCA9FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -637,7 +637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55D72402-01E0-4A9B-8ECC-48C409EB3897}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27269916-11CE-4374-A763-F555C98AE6E6}">
   <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -710,13 +710,13 @@
         <v>11</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I3" t="s">
         <v>12</v>
@@ -751,13 +751,13 @@
         <v>11</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I4" t="s">
         <v>17</v>
@@ -792,13 +792,13 @@
         <v>7</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="s">
         <v>20</v>
@@ -833,13 +833,13 @@
         <v>8</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I6" t="s">
         <v>23</v>
@@ -874,13 +874,13 @@
         <v>5</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="s">
         <v>26</v>
@@ -915,13 +915,13 @@
         <v>18</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I8" t="s">
         <v>29</v>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -979,13 +979,13 @@
         <v>9</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -1002,13 +1002,13 @@
         <v>17</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
@@ -1025,13 +1025,13 @@
         <v>10</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
@@ -1071,13 +1071,13 @@
         <v>10</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -1094,13 +1094,13 @@
         <v>19</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -1117,13 +1117,13 @@
         <v>15</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -1146,7 +1146,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1163,13 +1163,13 @@
         <v>12</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1186,13 +1186,13 @@
         <v>5</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -1209,13 +1209,13 @@
         <v>15</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1258,10 +1258,10 @@
         <v>0</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -1278,13 +1278,13 @@
         <v>8</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
@@ -1301,13 +1301,13 @@
         <v>11</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
@@ -1324,13 +1324,13 @@
         <v>6</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
@@ -1347,13 +1347,13 @@
         <v>15</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
@@ -1370,13 +1370,13 @@
         <v>7</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1393,13 +1393,13 @@
         <v>25</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1416,13 +1416,13 @@
         <v>7</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (12:56:53)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9739824-D27D-4CBD-A35C-C04F261A063E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5099787-44CE-41DB-8C2E-BA2E004333EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{697255EC-1792-4332-BFEA-978B4652329A}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{E082C765-AD56-4ACF-949A-3EA4052F1488}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -637,7 +637,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5F6BDFB-6BCC-4E9D-975D-FB459EA8E28B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBF8066C-7588-4994-881C-DFA5CBAE000B}">
   <dimension ref="A1:N29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (13:11:46)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5099787-44CE-41DB-8C2E-BA2E004333EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{146BC381-758B-4001-A4FC-07199FCCEE5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{E082C765-AD56-4ACF-949A-3EA4052F1488}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{802C15E6-4013-4621-A12C-AA6050C6B086}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,11 +39,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="73">
   <si>
     <t>17th ELO</t>
   </si>
   <si>
+    <t>±</t>
+  </si>
+  <si>
     <t>닉네임</t>
   </si>
   <si>
@@ -92,7 +95,7 @@
     <t>AS 로마</t>
   </si>
   <si>
-    <t>1부리그</t>
+    <t/>
   </si>
   <si>
     <t>검정소</t>
@@ -110,7 +113,7 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>UEFA_B조</t>
+    <t>Error</t>
   </si>
   <si>
     <t>은안</t>
@@ -637,11 +640,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBF8066C-7588-4994-881C-DFA5CBAE000B}">
-  <dimension ref="A1:N29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B99E414-5FC5-4213-8CC6-0B71983C795C}">
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -663,22 +666,25 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1149.50125</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
+      <c r="B2">
+        <v>39.339999999999918</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2">
-        <v>4</v>
+      <c r="D2" t="s">
+        <v>9</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -686,40 +692,43 @@
       <c r="G2">
         <v>0</v>
       </c>
-      <c r="I2" t="s">
-        <v>9</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
         <v>10</v>
       </c>
       <c r="L2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M2" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1129.0725</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
+      <c r="B3">
+        <v>4.4300000000000637</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>11</v>
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="I3" t="s">
-        <v>12</v>
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
       </c>
       <c r="J3" t="s">
         <v>13</v>
@@ -728,7 +737,7 @@
         <v>14</v>
       </c>
       <c r="L3" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -736,34 +745,37 @@
       <c r="N3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1119.54</v>
       </c>
-      <c r="B4" t="s">
-        <v>15</v>
+      <c r="B4">
+        <v>88</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="D4">
-        <v>11</v>
+      <c r="D4" t="s">
+        <v>17</v>
       </c>
       <c r="E4">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>2</v>
-      </c>
-      <c r="I4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
+        <v>18</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -777,40 +789,43 @@
       <c r="N4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>1092.395</v>
       </c>
-      <c r="B5" t="s">
-        <v>18</v>
+      <c r="B5">
+        <v>42.319999999999936</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
       </c>
-      <c r="D5">
-        <v>7</v>
+      <c r="D5" t="s">
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5">
-        <v>14.25</v>
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
       </c>
       <c r="K5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -818,75 +833,81 @@
       <c r="N5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>1090.82</v>
       </c>
-      <c r="B6" t="s">
-        <v>21</v>
+      <c r="B6">
+        <v>51.779999999999973</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="D6">
-        <v>8</v>
+      <c r="D6" t="s">
+        <v>23</v>
       </c>
       <c r="E6">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="I6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J6">
-        <v>-9.8199999999999985</v>
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
+        <v>24</v>
       </c>
       <c r="K6">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>1084.4150000000002</v>
       </c>
-      <c r="B7" t="s">
-        <v>24</v>
+      <c r="B7">
+        <v>39.200000000000045</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="D7">
-        <v>5</v>
+      <c r="D7" t="s">
+        <v>26</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="J7" t="s">
+        <v>27</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -900,60 +921,66 @@
       <c r="N7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="O7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1056.81125</v>
       </c>
-      <c r="B8" t="s">
-        <v>27</v>
+      <c r="B8">
+        <v>17.930000000000064</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
       </c>
-      <c r="D8">
-        <v>18</v>
+      <c r="D8" t="s">
+        <v>29</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>3</v>
-      </c>
-      <c r="I8" t="s">
-        <v>29</v>
-      </c>
-      <c r="J8">
-        <v>4.4300000000000015</v>
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s">
+        <v>30</v>
       </c>
       <c r="K8">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>1028.7775000000001</v>
       </c>
-      <c r="B9" t="s">
-        <v>30</v>
+      <c r="B9">
+        <v>-26.769999999999982</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
       </c>
-      <c r="D9">
-        <v>2</v>
+      <c r="D9" t="s">
+        <v>32</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -962,90 +989,102 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1019.7900000000001</v>
       </c>
-      <c r="B10" t="s">
-        <v>32</v>
+      <c r="B10">
+        <v>-18.42999999999995</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
       </c>
-      <c r="D10">
-        <v>9</v>
+      <c r="D10" t="s">
+        <v>34</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1006.7609090909091</v>
       </c>
-      <c r="B11" t="s">
-        <v>34</v>
+      <c r="B11">
+        <v>70.960000000000036</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
       </c>
-      <c r="D11">
-        <v>17</v>
+      <c r="D11" t="s">
+        <v>36</v>
       </c>
       <c r="E11">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1006.55</v>
       </c>
-      <c r="B12" t="s">
-        <v>36</v>
+      <c r="B12">
+        <v>13.289999999999964</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
       </c>
-      <c r="D12">
-        <v>10</v>
+      <c r="D12" t="s">
+        <v>38</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1001.55125</v>
       </c>
-      <c r="B13" t="s">
-        <v>38</v>
+      <c r="B13">
+        <v>0</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
       </c>
-      <c r="D13">
-        <v>0</v>
+      <c r="D13" t="s">
+        <v>40</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -1056,88 +1095,100 @@
       <c r="G13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>998.44125000000008</v>
       </c>
-      <c r="B14" t="s">
-        <v>40</v>
+      <c r="B14">
+        <v>-31.559999999999945</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
       </c>
-      <c r="D14">
-        <v>10</v>
+      <c r="D14" t="s">
+        <v>42</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>976.28090909090906</v>
       </c>
-      <c r="B15" t="s">
-        <v>42</v>
+      <c r="B15">
+        <v>40.480000000000018</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
       </c>
-      <c r="D15">
-        <v>19</v>
+      <c r="D15" t="s">
+        <v>44</v>
       </c>
       <c r="E15">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>973.00090909090909</v>
       </c>
-      <c r="B16" t="s">
-        <v>44</v>
+      <c r="B16">
+        <v>37.200000000000045</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
       </c>
-      <c r="D16">
-        <v>15</v>
+      <c r="D16" t="s">
+        <v>46</v>
       </c>
       <c r="E16">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>967.49750000000006</v>
       </c>
-      <c r="B17" t="s">
-        <v>46</v>
+      <c r="B17">
+        <v>-40.330000000000041</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
       </c>
-      <c r="D17">
-        <v>3</v>
+      <c r="D17" t="s">
+        <v>48</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1146,90 +1197,102 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>955.31090909090904</v>
       </c>
-      <c r="B18" t="s">
-        <v>48</v>
+      <c r="B18">
+        <v>19.509999999999991</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
       </c>
-      <c r="D18">
-        <v>12</v>
+      <c r="D18" t="s">
+        <v>50</v>
       </c>
       <c r="E18">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>951.13250000000005</v>
       </c>
-      <c r="B19" t="s">
-        <v>50</v>
+      <c r="B19">
+        <v>-19.809999999999945</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
       </c>
-      <c r="D19">
-        <v>5</v>
+      <c r="D19" t="s">
+        <v>52</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>948.55090909090904</v>
       </c>
-      <c r="B20" t="s">
-        <v>52</v>
+      <c r="B20">
+        <v>12.75</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
       </c>
-      <c r="D20">
-        <v>15</v>
+      <c r="D20" t="s">
+        <v>54</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>935.80090909090904</v>
       </c>
-      <c r="B21" t="s">
-        <v>54</v>
+      <c r="B21">
+        <v>0</v>
       </c>
       <c r="C21" t="s">
         <v>55</v>
       </c>
-      <c r="D21">
-        <v>0</v>
+      <c r="D21" t="s">
+        <v>56</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1240,189 +1303,216 @@
       <c r="G21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>933.23090909090899</v>
       </c>
-      <c r="B22" t="s">
-        <v>56</v>
+      <c r="B22">
+        <v>-2.57000000000005</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
       </c>
-      <c r="D22">
-        <v>2</v>
+      <c r="D22" t="s">
+        <v>58</v>
       </c>
       <c r="E22">
         <v>0</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>928.66125000000011</v>
       </c>
-      <c r="B23" t="s">
-        <v>58</v>
+      <c r="B23">
+        <v>-26.799999999999955</v>
       </c>
       <c r="C23" t="s">
         <v>59</v>
       </c>
-      <c r="D23">
-        <v>8</v>
+      <c r="D23" t="s">
+        <v>60</v>
       </c>
       <c r="E23">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>926.50090909090909</v>
       </c>
-      <c r="B24" t="s">
-        <v>60</v>
+      <c r="B24">
+        <v>-9.2999999999999545</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
       </c>
-      <c r="D24">
-        <v>11</v>
+      <c r="D24" t="s">
+        <v>62</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>918.03090909090906</v>
       </c>
-      <c r="B25" t="s">
-        <v>62</v>
+      <c r="B25">
+        <v>-17.769999999999982</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
       </c>
-      <c r="D25">
-        <v>6</v>
+      <c r="D25" t="s">
+        <v>64</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>913.26249999999993</v>
       </c>
-      <c r="B26" t="s">
-        <v>64</v>
+      <c r="B26">
+        <v>-69.139999999999986</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
       </c>
-      <c r="D26">
-        <v>15</v>
+      <c r="D26" t="s">
+        <v>66</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>906.470909090909</v>
       </c>
-      <c r="B27" t="s">
-        <v>66</v>
+      <c r="B27">
+        <v>-29.330000000000041</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
       </c>
-      <c r="D27">
-        <v>7</v>
+      <c r="D27" t="s">
+        <v>68</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
       <c r="G27">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>902.18124999999998</v>
       </c>
-      <c r="B28" t="s">
-        <v>68</v>
+      <c r="B28">
+        <v>-42.110000000000014</v>
       </c>
       <c r="C28" t="s">
         <v>69</v>
       </c>
-      <c r="D28">
-        <v>25</v>
+      <c r="D28" t="s">
+        <v>70</v>
       </c>
       <c r="E28">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>892.01090909090908</v>
       </c>
-      <c r="B29" t="s">
-        <v>70</v>
+      <c r="B29">
+        <v>-43.789999999999964</v>
       </c>
       <c r="C29" t="s">
         <v>71</v>
       </c>
-      <c r="D29">
-        <v>7</v>
+      <c r="D29" t="s">
+        <v>72</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29">
         <v>0</v>
       </c>
       <c r="G29">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (13:14:36)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3329B15-2375-469A-8FD5-6FB2AB0E6201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{908F79E1-9056-4231-A405-68714E605DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{DB802FCF-0934-4D86-9DCC-A8B5AD1A7B5D}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{5020C1BC-B932-4CAB-A188-0DC4C59BA1F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF05942E-B1BC-4ECF-B94F-53DD3197788A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4378D927-4E13-4370-A034-8495D1ACE3F1}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -684,10 +684,10 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -719,16 +719,16 @@
         <v>12</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J3" t="s">
         <v>13</v>
@@ -763,16 +763,16 @@
         <v>17</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" t="s">
         <v>18</v>
@@ -807,16 +807,16 @@
         <v>20</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
@@ -851,16 +851,16 @@
         <v>23</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6">
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" t="s">
         <v>24</v>
@@ -895,16 +895,16 @@
         <v>26</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="s">
         <v>27</v>
@@ -939,16 +939,16 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J8" t="s">
         <v>30</v>
@@ -983,7 +983,7 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -992,7 +992,7 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -1009,16 +1009,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
@@ -1035,16 +1035,16 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
@@ -1061,16 +1061,16 @@
         <v>38</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -1113,16 +1113,16 @@
         <v>42</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
@@ -1139,16 +1139,16 @@
         <v>44</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -1165,16 +1165,16 @@
         <v>46</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
@@ -1191,7 +1191,7 @@
         <v>48</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1217,16 +1217,16 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -1243,16 +1243,16 @@
         <v>52</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G19">
         <v>0</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
@@ -1269,16 +1269,16 @@
         <v>54</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -1321,16 +1321,16 @@
         <v>58</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -1347,16 +1347,16 @@
         <v>60</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
@@ -1373,16 +1373,16 @@
         <v>62</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G24">
         <v>0</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
@@ -1399,16 +1399,16 @@
         <v>64</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
@@ -1425,16 +1425,16 @@
         <v>66</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
@@ -1451,16 +1451,16 @@
         <v>68</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
@@ -1477,16 +1477,16 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
@@ -1503,16 +1503,16 @@
         <v>72</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (16:19:32)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{908F79E1-9056-4231-A405-68714E605DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D1FC4E1-467C-44EB-87E5-0481D5D14583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{5020C1BC-B932-4CAB-A188-0DC4C59BA1F2}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{099F9BC6-7985-4EF7-A87E-9E58195D876A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="73">
   <si>
     <t>17th ELO</t>
   </si>
@@ -71,12 +71,18 @@
     <t>바이에른 뮌헨</t>
   </si>
   <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
     <t>Voor</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>첼시</t>
   </si>
   <si>
@@ -95,7 +101,7 @@
     <t>AS 로마</t>
   </si>
   <si>
-    <t/>
+    <t>3부리그</t>
   </si>
   <si>
     <t>검정소</t>
@@ -113,7 +119,7 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>Error</t>
+    <t>UEFA_D조</t>
   </si>
   <si>
     <t>은안</t>
@@ -146,10 +152,10 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
   </si>
   <si>
     <t>앙쿠</t>
@@ -158,42 +164,36 @@
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>방덕</t>
   </si>
   <si>
     <t>인테르</t>
   </si>
   <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>여수가스</t>
+  </si>
+  <si>
+    <t>AS 모나코</t>
+  </si>
+  <si>
     <t>suma수마</t>
   </si>
   <si>
     <t>ACF 피오렌티나</t>
   </si>
   <si>
-    <t>여수가스</t>
-  </si>
-  <si>
-    <t>AS 모나코</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
@@ -218,18 +218,18 @@
     <t>레알 마드리드</t>
   </si>
   <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
     <t>경남FC가즈아</t>
   </si>
   <si>
     <t>경남 FC</t>
   </si>
   <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
     <t>A지냐크</t>
   </si>
   <si>
@@ -248,16 +248,16 @@
     <t>상하이 선화</t>
   </si>
   <si>
+    <t>겐지간지</t>
+  </si>
+  <si>
+    <t>파리 생제르맹</t>
+  </si>
+  <si>
     <t>Legend독수리</t>
   </si>
   <si>
     <t>맨체스터 유나이티드</t>
-  </si>
-  <si>
-    <t>겐지간지</t>
-  </si>
-  <si>
-    <t>파리 생제르맹</t>
   </si>
 </sst>
 </file>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4378D927-4E13-4370-A034-8495D1ACE3F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4ACA09E-077A-40FF-AAEF-2B9BBB72ED24}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -672,10 +672,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1149.50125</v>
+        <v>1153.174</v>
       </c>
       <c r="B2">
-        <v>39.339999999999918</v>
+        <v>38.309999999999945</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -701,22 +701,22 @@
       <c r="L2" t="s">
         <v>11</v>
       </c>
-      <c r="M2" t="e">
-        <v>#N/A</v>
+      <c r="M2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1129.0725</v>
+        <v>1128.3224999999998</v>
       </c>
       <c r="B3">
-        <v>4.4300000000000637</v>
+        <v>4.0999999999999091</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>11</v>
@@ -731,13 +731,13 @@
         <v>3</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -751,60 +751,60 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1119.54</v>
+        <v>1120.9575000000002</v>
       </c>
       <c r="B4">
-        <v>88</v>
+        <v>90.1400000000001</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>17.3</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1092.395</v>
+        <v>1091.6175000000001</v>
       </c>
       <c r="B5">
-        <v>42.319999999999936</v>
+        <v>42.660000000000082</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5">
         <v>7</v>
@@ -819,16 +819,16 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>19.489999999999998</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -839,16 +839,16 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1090.82</v>
+        <v>1090.7725000000003</v>
       </c>
       <c r="B6">
-        <v>51.779999999999973</v>
+        <v>51.160000000000082</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>8</v>
@@ -863,36 +863,36 @@
         <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>0</v>
+        <v>26.12</v>
       </c>
       <c r="L6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N6">
         <v>0</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1084.4150000000002</v>
+        <v>1083.2649999999999</v>
       </c>
       <c r="B7">
-        <v>39.200000000000045</v>
+        <v>39.099999999999909</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -907,7 +907,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -927,16 +927,16 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1056.81125</v>
+        <v>1054.1590000000003</v>
       </c>
       <c r="B8">
-        <v>17.930000000000064</v>
+        <v>13.6400000000001</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E8">
         <v>18</v>
@@ -951,36 +951,36 @@
         <v>3</v>
       </c>
       <c r="J8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K8">
-        <v>0</v>
+        <v>62.91</v>
       </c>
       <c r="L8">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="N8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1028.7775000000001</v>
+        <v>1027.4275</v>
       </c>
       <c r="B9">
-        <v>-26.769999999999982</v>
+        <v>-26.789999999999964</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -997,16 +997,16 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1019.7900000000001</v>
+        <v>1018.7049999999998</v>
       </c>
       <c r="B10">
-        <v>-18.42999999999995</v>
+        <v>-18.600000000000023</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10">
         <v>9</v>
@@ -1023,42 +1023,42 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1006.7609090909091</v>
+        <v>1001.8340000000001</v>
       </c>
       <c r="B11">
-        <v>70.960000000000036</v>
+        <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E11">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="F11">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1006.55</v>
+        <v>1000.0350000000001</v>
       </c>
       <c r="B12">
-        <v>13.289999999999964</v>
+        <v>7.4500000000000455</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E12">
         <v>10</v>
@@ -1075,62 +1075,62 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1001.55125</v>
+        <v>995.99900000000014</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>-30.870000000000005</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>998.44125000000008</v>
+        <v>993.79086363636361</v>
       </c>
       <c r="B14">
-        <v>-31.559999999999945</v>
+        <v>62.909999999999968</v>
       </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E14">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F14">
+        <v>12</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
         <v>4</v>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-      <c r="H14">
-        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>976.28090909090906</v>
+        <v>974.96086363636368</v>
       </c>
       <c r="B15">
-        <v>40.480000000000018</v>
+        <v>44.080000000000041</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -1139,24 +1139,24 @@
         <v>44</v>
       </c>
       <c r="E15">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F15">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>973.00090909090909</v>
+        <v>966.74</v>
       </c>
       <c r="B16">
-        <v>37.200000000000045</v>
+        <v>-40.360000000000014</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
@@ -1165,24 +1165,24 @@
         <v>46</v>
       </c>
       <c r="E16">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>967.49750000000006</v>
+        <v>965.67086363636361</v>
       </c>
       <c r="B17">
-        <v>-40.330000000000041</v>
+        <v>34.789999999999964</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1191,24 +1191,24 @@
         <v>48</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>955.31090909090904</v>
+        <v>963.45086363636369</v>
       </c>
       <c r="B18">
-        <v>19.509999999999991</v>
+        <v>32.57000000000005</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -1217,13 +1217,13 @@
         <v>50</v>
       </c>
       <c r="E18">
+        <v>19</v>
+      </c>
+      <c r="F18">
         <v>12</v>
       </c>
-      <c r="F18">
-        <v>4</v>
-      </c>
       <c r="G18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H18">
         <v>6</v>
@@ -1231,10 +1231,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>951.13250000000005</v>
+        <v>948.86</v>
       </c>
       <c r="B19">
-        <v>-19.809999999999945</v>
+        <v>-21.159999999999968</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1257,10 +1257,10 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>948.55090909090904</v>
+        <v>948.06086363636359</v>
       </c>
       <c r="B20">
-        <v>12.75</v>
+        <v>17.17999999999995</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -1283,10 +1283,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>935.80090909090904</v>
+        <v>929.84086363636368</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>-1.0399999999999636</v>
       </c>
       <c r="C21" t="s">
         <v>55</v>
@@ -1295,24 +1295,24 @@
         <v>56</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21">
         <v>0</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>933.23090909090899</v>
+        <v>929.4308636363636</v>
       </c>
       <c r="B22">
-        <v>-2.57000000000005</v>
+        <v>-1.4500000000000455</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1335,10 +1335,10 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>928.66125000000011</v>
+        <v>928.27086363636363</v>
       </c>
       <c r="B23">
-        <v>-26.799999999999955</v>
+        <v>-2.6100000000000136</v>
       </c>
       <c r="C23" t="s">
         <v>59</v>
@@ -1347,24 +1347,24 @@
         <v>60</v>
       </c>
       <c r="E23">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F23">
         <v>3</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>926.50090909090909</v>
+        <v>922.31900000000007</v>
       </c>
       <c r="B24">
-        <v>-9.2999999999999545</v>
+        <v>-29.389999999999986</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
@@ -1373,24 +1373,24 @@
         <v>62</v>
       </c>
       <c r="E24">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H24">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>918.03090909090906</v>
+        <v>919.69086363636359</v>
       </c>
       <c r="B25">
-        <v>-17.769999999999982</v>
+        <v>-11.190000000000055</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1413,10 +1413,10 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>913.26249999999993</v>
+        <v>911.94749999999999</v>
       </c>
       <c r="B26">
-        <v>-69.139999999999986</v>
+        <v>-69.710000000000036</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
@@ -1439,10 +1439,10 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>906.470909090909</v>
+        <v>906.11086363636366</v>
       </c>
       <c r="B27">
-        <v>-29.330000000000041</v>
+        <v>-24.769999999999982</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
@@ -1465,10 +1465,10 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>902.18124999999998</v>
+        <v>889.4308636363636</v>
       </c>
       <c r="B28">
-        <v>-42.110000000000014</v>
+        <v>-41.450000000000045</v>
       </c>
       <c r="C28" t="s">
         <v>69</v>
@@ -1477,24 +1477,24 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
         <v>6</v>
-      </c>
-      <c r="G28">
-        <v>3</v>
-      </c>
-      <c r="H28">
-        <v>16</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>892.01090909090908</v>
+        <v>874.76400000000001</v>
       </c>
       <c r="B29">
-        <v>-43.789999999999964</v>
+        <v>-59.460000000000036</v>
       </c>
       <c r="C29" t="s">
         <v>71</v>
@@ -1503,16 +1503,16 @@
         <v>72</v>
       </c>
       <c r="E29">
+        <v>31</v>
+      </c>
+      <c r="F29">
         <v>7</v>
       </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
       <c r="G29">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H29">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (17:50:32)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D1FC4E1-467C-44EB-87E5-0481D5D14583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{436D941D-D376-41E3-85AE-00454B941A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{099F9BC6-7985-4EF7-A87E-9E58195D876A}"/>
+    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{08AC64DD-D408-446A-8D53-1C8C0BB9AD55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,93 +71,99 @@
     <t>바이에른 뮌헨</t>
   </si>
   <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
+    <t>Voor</t>
+  </si>
+  <si>
+    <t>첼시</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>UEFA_A조</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>킹왕두</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
     <t>ZD장인지참치</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>레버쿠젠</t>
   </si>
   <si>
-    <t>Voor</t>
-  </si>
-  <si>
-    <t>첼시</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>UEFA_D조</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>킹왕두</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>앙쿠</t>
   </si>
   <si>
@@ -252,12 +258,6 @@
   </si>
   <si>
     <t>파리 생제르맹</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
   </si>
 </sst>
 </file>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4ACA09E-077A-40FF-AAEF-2B9BBB72ED24}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E17814C-5B13-45B5-867D-9782C7304042}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -707,10 +707,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1128.3224999999998</v>
+        <v>1146.2275000000002</v>
       </c>
       <c r="B3">
-        <v>4.0999999999999091</v>
+        <v>115.41000000000008</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -719,16 +719,16 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G3">
+        <v>3</v>
+      </c>
+      <c r="H3">
         <v>2</v>
-      </c>
-      <c r="H3">
-        <v>3</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
@@ -751,10 +751,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1120.9575000000002</v>
+        <v>1128.3224999999998</v>
       </c>
       <c r="B4">
-        <v>90.1400000000001</v>
+        <v>4.0999999999999091</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -763,34 +763,34 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4">
         <v>3</v>
-      </c>
-      <c r="H4">
-        <v>2</v>
       </c>
       <c r="J4" t="s">
         <v>20</v>
       </c>
       <c r="K4">
-        <v>17.3</v>
+        <v>-18.990000000000002</v>
       </c>
       <c r="L4">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="M4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N4">
         <v>1</v>
       </c>
       <c r="O4">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -822,7 +822,7 @@
         <v>23</v>
       </c>
       <c r="K5">
-        <v>19.489999999999998</v>
+        <v>24.36</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -866,19 +866,19 @@
         <v>26</v>
       </c>
       <c r="K6">
-        <v>26.12</v>
+        <v>-65.31</v>
       </c>
       <c r="L6">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="O6">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -927,10 +927,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1054.1590000000003</v>
+        <v>1035.8690000000001</v>
       </c>
       <c r="B8">
-        <v>13.6400000000001</v>
+        <v>-4.6500000000000909</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -939,34 +939,34 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F8">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G8">
         <v>5</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
       </c>
       <c r="K8">
-        <v>62.91</v>
+        <v>-59.940000000000005</v>
       </c>
       <c r="L8">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="N8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O8">
-        <v>4</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1049,10 +1049,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1000.0350000000001</v>
+        <v>1000.7408636363637</v>
       </c>
       <c r="B12">
-        <v>7.4500000000000455</v>
+        <v>69.860000000000014</v>
       </c>
       <c r="C12" t="s">
         <v>39</v>
@@ -1061,24 +1061,24 @@
         <v>40</v>
       </c>
       <c r="E12">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>995.99900000000014</v>
+        <v>1000.0350000000001</v>
       </c>
       <c r="B13">
-        <v>-30.870000000000005</v>
+        <v>7.4500000000000455</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1090,53 +1090,53 @@
         <v>10</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>993.79086363636361</v>
+        <v>995.99900000000014</v>
       </c>
       <c r="B14">
-        <v>62.909999999999968</v>
+        <v>-30.870000000000005</v>
       </c>
       <c r="C14" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14">
         <v>10</v>
       </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14">
-        <v>17</v>
-      </c>
       <c r="F14">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>974.96086363636368</v>
+        <v>974.45086363636369</v>
       </c>
       <c r="B15">
-        <v>44.080000000000041</v>
+        <v>43.57000000000005</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E15">
         <v>16</v>
@@ -1159,10 +1159,10 @@
         <v>-40.360000000000014</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -1179,16 +1179,16 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>965.67086363636361</v>
+        <v>965.73086363636367</v>
       </c>
       <c r="B17">
-        <v>34.789999999999964</v>
+        <v>34.850000000000023</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E17">
         <v>15</v>
@@ -1205,19 +1205,19 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>963.45086363636369</v>
+        <v>957.64086363636363</v>
       </c>
       <c r="B18">
-        <v>32.57000000000005</v>
+        <v>26.759999999999991</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E18">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F18">
         <v>12</v>
@@ -1226,21 +1226,21 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>948.86</v>
+        <v>948.87</v>
       </c>
       <c r="B19">
-        <v>-21.159999999999968</v>
+        <v>-21.149999999999977</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E19">
         <v>5</v>
@@ -1257,19 +1257,19 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>948.06086363636359</v>
+        <v>941.88086363636364</v>
       </c>
       <c r="B20">
-        <v>17.17999999999995</v>
+        <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D20" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E20">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F20">
         <v>5</v>
@@ -1278,7 +1278,7 @@
         <v>3</v>
       </c>
       <c r="H20">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
@@ -1289,10 +1289,10 @@
         <v>-1.0399999999999636</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>-1.4500000000000455</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E22">
         <v>2</v>
@@ -1341,10 +1341,10 @@
         <v>-2.6100000000000136</v>
       </c>
       <c r="C23" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E23">
         <v>11</v>
@@ -1361,16 +1361,16 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>922.31900000000007</v>
+        <v>923.04900000000009</v>
       </c>
       <c r="B24">
-        <v>-29.389999999999986</v>
+        <v>-28.659999999999968</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -1393,10 +1393,10 @@
         <v>-11.190000000000055</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D25" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E25">
         <v>6</v>
@@ -1419,10 +1419,10 @@
         <v>-69.710000000000036</v>
       </c>
       <c r="C26" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D26" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E26">
         <v>15</v>
@@ -1445,10 +1445,10 @@
         <v>-24.769999999999982</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E27">
         <v>7</v>
@@ -1465,16 +1465,16 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>889.4308636363636</v>
+        <v>889.4408636363637</v>
       </c>
       <c r="B28">
-        <v>-41.450000000000045</v>
+        <v>-41.439999999999941</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E28">
         <v>7</v>
@@ -1491,16 +1491,16 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>874.76400000000001</v>
+        <v>874.28399999999999</v>
       </c>
       <c r="B29">
-        <v>-59.460000000000036</v>
+        <v>-59.940000000000055</v>
       </c>
       <c r="C29" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="E29">
         <v>31</v>

</xml_diff>

<commit_message>
Update: Ranking Data (17:53:53)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{436D941D-D376-41E3-85AE-00454B941A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0C1F079-8EC9-4916-93ED-B6334E3F0518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{08AC64DD-D408-446A-8D53-1C8C0BB9AD55}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{7FD324CC-1F2F-4F87-853F-C9D8FCD7DE16}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E17814C-5B13-45B5-867D-9782C7304042}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BFAA15-8B7E-443F-9A3D-B8662BDD0CB7}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (18:50:30)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C0C1F079-8EC9-4916-93ED-B6334E3F0518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82550896-9CD6-47FC-8EAD-A05BAF0D5F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{7FD324CC-1F2F-4F87-853F-C9D8FCD7DE16}"/>
+    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{FA2F530E-1245-4823-BF29-F03146172C21}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,199 +65,199 @@
     <t>패</t>
   </si>
   <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
     <t>개포동덕배</t>
   </si>
   <si>
     <t>바이에른 뮌헨</t>
   </si>
   <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
+    <t>Voor</t>
+  </si>
+  <si>
+    <t>첼시</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>UEFA_A조</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>킹왕두</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>여수가스</t>
+  </si>
+  <si>
+    <t>AS 모나코</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>스페인전도사</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
+  </si>
+  <si>
+    <t>겐지간지</t>
+  </si>
+  <si>
+    <t>파리 생제르맹</t>
+  </si>
+  <si>
     <t>Legend독수리</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>맨체스터 유나이티드</t>
-  </si>
-  <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>Voor</t>
-  </si>
-  <si>
-    <t>첼시</t>
-  </si>
-  <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>UEFA_A조</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>킹왕두</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>여수가스</t>
-  </si>
-  <si>
-    <t>AS 모나코</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
-  </si>
-  <si>
-    <t>스페인전도사</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>겐지간지</t>
-  </si>
-  <si>
-    <t>파리 생제르맹</t>
   </si>
 </sst>
 </file>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59BFAA15-8B7E-443F-9A3D-B8662BDD0CB7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{423D8815-80B3-4E7A-ADF5-A869B9E07DDF}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -672,10 +672,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1153.174</v>
+        <v>1157.8975</v>
       </c>
       <c r="B2">
-        <v>38.309999999999945</v>
+        <v>127.07999999999993</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -684,60 +684,60 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" t="s">
         <v>10</v>
       </c>
-      <c r="L2" t="s">
-        <v>11</v>
-      </c>
       <c r="M2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1146.2275000000002</v>
+        <v>1153.174</v>
       </c>
       <c r="B3">
-        <v>115.41000000000008</v>
+        <v>38.309999999999945</v>
       </c>
       <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="K3" t="s">
         <v>14</v>
       </c>
-      <c r="E3">
+      <c r="L3" t="s">
         <v>15</v>
-      </c>
-      <c r="F3">
-        <v>10</v>
-      </c>
-      <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="H3">
-        <v>2</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L3" t="s">
-        <v>17</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -757,10 +757,10 @@
         <v>4.0999999999999091</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E4">
         <v>11</v>
@@ -775,54 +775,54 @@
         <v>3</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K4">
-        <v>-18.990000000000002</v>
+        <v>67.53</v>
       </c>
       <c r="L4">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O4">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1091.6175000000001</v>
+        <v>1093.6675</v>
       </c>
       <c r="B5">
-        <v>42.660000000000082</v>
+        <v>44.710000000000036</v>
       </c>
       <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5">
+        <v>11</v>
+      </c>
+      <c r="F5">
+        <v>6</v>
+      </c>
+      <c r="G5">
+        <v>2</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+      <c r="J5" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5">
-        <v>7</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>23</v>
-      </c>
       <c r="K5">
-        <v>24.36</v>
+        <v>19.260000000000002</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -845,10 +845,10 @@
         <v>51.160000000000082</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E6">
         <v>8</v>
@@ -863,22 +863,22 @@
         <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K6">
-        <v>-65.31</v>
+        <v>40.290000000000006</v>
       </c>
       <c r="L6">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O6">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -889,10 +889,10 @@
         <v>39.099999999999909</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -907,7 +907,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -927,60 +927,60 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1035.8690000000001</v>
+        <v>1035.0690000000002</v>
       </c>
       <c r="B8">
-        <v>-4.6500000000000909</v>
+        <v>-5.4500000000000455</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E8">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F8">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G8">
         <v>5</v>
       </c>
       <c r="H8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K8">
-        <v>-59.940000000000005</v>
+        <v>127.08000000000001</v>
       </c>
       <c r="L8">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="M8">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O8">
-        <v>20</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1027.4275</v>
+        <v>1027.5374999999999</v>
       </c>
       <c r="B9">
-        <v>-26.789999999999964</v>
+        <v>-26.680000000000064</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -997,106 +997,106 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1018.7049999999998</v>
+        <v>1022.585</v>
       </c>
       <c r="B10">
-        <v>-18.600000000000023</v>
+        <v>30</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E10">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1001.8340000000001</v>
+        <v>1018.7049999999998</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>-18.600000000000023</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1000.7408636363637</v>
+        <v>1001.8340000000001</v>
       </c>
       <c r="B12">
-        <v>69.860000000000014</v>
+        <v>0</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E12">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1000.0350000000001</v>
+        <v>1001.6208636363637</v>
       </c>
       <c r="B13">
-        <v>7.4500000000000455</v>
+        <v>70.740000000000009</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E13">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F13">
+        <v>15</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
         <v>5</v>
-      </c>
-      <c r="G13">
-        <v>2</v>
-      </c>
-      <c r="H13">
-        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
@@ -1107,10 +1107,10 @@
         <v>-30.870000000000005</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -1127,16 +1127,16 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>974.45086363636369</v>
+        <v>974.53086363636362</v>
       </c>
       <c r="B15">
-        <v>43.57000000000005</v>
+        <v>43.649999999999977</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E15">
         <v>16</v>
@@ -1159,10 +1159,10 @@
         <v>-40.360000000000014</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E16">
         <v>3</v>
@@ -1185,10 +1185,10 @@
         <v>34.850000000000023</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E17">
         <v>15</v>
@@ -1211,10 +1211,10 @@
         <v>26.759999999999991</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E18">
         <v>21</v>
@@ -1237,10 +1237,10 @@
         <v>-21.149999999999977</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E19">
         <v>5</v>
@@ -1263,10 +1263,10 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E20">
         <v>17</v>
@@ -1289,10 +1289,10 @@
         <v>-1.0399999999999636</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -1315,10 +1315,10 @@
         <v>-1.4500000000000455</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E22">
         <v>2</v>
@@ -1341,10 +1341,10 @@
         <v>-2.6100000000000136</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D23" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E23">
         <v>11</v>
@@ -1367,10 +1367,10 @@
         <v>-28.659999999999968</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E24">
         <v>10</v>
@@ -1393,10 +1393,10 @@
         <v>-11.190000000000055</v>
       </c>
       <c r="C25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E25">
         <v>6</v>
@@ -1419,10 +1419,10 @@
         <v>-69.710000000000036</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E26">
         <v>15</v>
@@ -1445,10 +1445,10 @@
         <v>-24.769999999999982</v>
       </c>
       <c r="C27" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E27">
         <v>7</v>
@@ -1471,10 +1471,10 @@
         <v>-41.439999999999941</v>
       </c>
       <c r="C28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D28" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E28">
         <v>7</v>
@@ -1497,10 +1497,10 @@
         <v>-59.940000000000055</v>
       </c>
       <c r="C29" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="E29">
         <v>31</v>

</xml_diff>

<commit_message>
Update: Ranking Data (19:37:50)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82550896-9CD6-47FC-8EAD-A05BAF0D5F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5AEA0F0-BF73-460F-A2F3-D61844EC34B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{FA2F530E-1245-4823-BF29-F03146172C21}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{8B38A288-13A2-4443-8FCB-35F7E84A212C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,16 +134,16 @@
     <t>전체 합계</t>
   </si>
   <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
     <t>킹왕두</t>
   </si>
   <si>
     <t>리버풀</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
   </si>
   <si>
     <t>아들러</t>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{423D8815-80B3-4E7A-ADF5-A869B9E07DDF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D52FCAB9-7180-4A6E-AB8F-291A814ACB03}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -971,10 +971,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1027.5374999999999</v>
+        <v>1029.7650000000001</v>
       </c>
       <c r="B9">
-        <v>-26.680000000000064</v>
+        <v>37.180000000000064</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -983,24 +983,24 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1022.585</v>
+        <v>1027.5374999999999</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>-26.680000000000064</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1009,16 +1009,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
@@ -1387,10 +1387,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>919.69086363636359</v>
+        <v>912.82086363636358</v>
       </c>
       <c r="B25">
-        <v>-11.190000000000055</v>
+        <v>-18.060000000000059</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1399,16 +1399,16 @@
         <v>64</v>
       </c>
       <c r="E25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (21:36:52)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5AEA0F0-BF73-460F-A2F3-D61844EC34B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A0E0A14-03F7-4C2F-AEE5-B8F81F510696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{8B38A288-13A2-4443-8FCB-35F7E84A212C}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{16874035-6221-4864-A65D-A1353B0DC5BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -200,6 +200,12 @@
     <t>함부르크SV</t>
   </si>
   <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
     <t>스페인전도사</t>
   </si>
   <si>
@@ -224,28 +230,22 @@
     <t>토트넘</t>
   </si>
   <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
   </si>
   <si>
     <t>A지냐크</t>
   </si>
   <si>
     <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
   </si>
   <si>
     <t>겐지간지</t>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D52FCAB9-7180-4A6E-AB8F-291A814ACB03}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E31039C-8F62-4298-80C3-A0FC88ED44C1}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -672,10 +672,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1157.8975</v>
+        <v>1155.4175</v>
       </c>
       <c r="B2">
-        <v>127.07999999999993</v>
+        <v>124.59999999999991</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -684,13 +684,13 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
         <v>3</v>
@@ -866,16 +866,16 @@
         <v>24</v>
       </c>
       <c r="K6">
-        <v>40.290000000000006</v>
+        <v>37.81</v>
       </c>
       <c r="L6">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6">
         <v>2</v>
@@ -954,16 +954,16 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>127.08000000000001</v>
+        <v>124.60000000000001</v>
       </c>
       <c r="L8">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M8">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -1075,10 +1075,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1001.6208636363637</v>
+        <v>998.58086363636369</v>
       </c>
       <c r="B13">
-        <v>70.740000000000009</v>
+        <v>67.700000000000045</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
@@ -1087,16 +1087,16 @@
         <v>40</v>
       </c>
       <c r="E13">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F13">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
@@ -1205,10 +1205,10 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>957.64086363636363</v>
+        <v>953.15086363636362</v>
       </c>
       <c r="B18">
-        <v>26.759999999999991</v>
+        <v>22.269999999999982</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -1217,16 +1217,16 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F18">
         <v>12</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -1257,10 +1257,10 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>941.88086363636364</v>
+        <v>941.61900000000003</v>
       </c>
       <c r="B20">
-        <v>11</v>
+        <v>-10.090000000000032</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -1269,24 +1269,24 @@
         <v>54</v>
       </c>
       <c r="E20">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F20">
+        <v>6</v>
+      </c>
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
         <v>5</v>
-      </c>
-      <c r="G20">
-        <v>3</v>
-      </c>
-      <c r="H20">
-        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>929.84086363636368</v>
+        <v>941.3208636363637</v>
       </c>
       <c r="B21">
-        <v>-1.0399999999999636</v>
+        <v>10.440000000000055</v>
       </c>
       <c r="C21" t="s">
         <v>55</v>
@@ -1295,24 +1295,24 @@
         <v>56</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G21">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>929.4308636363636</v>
+        <v>938.33086363636369</v>
       </c>
       <c r="B22">
-        <v>-1.4500000000000455</v>
+        <v>7.4500000000000455</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1321,24 +1321,24 @@
         <v>58</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>928.27086363636363</v>
+        <v>929.4308636363636</v>
       </c>
       <c r="B23">
-        <v>-2.6100000000000136</v>
+        <v>-1.4500000000000455</v>
       </c>
       <c r="C23" t="s">
         <v>59</v>
@@ -1347,24 +1347,24 @@
         <v>60</v>
       </c>
       <c r="E23">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>923.04900000000009</v>
+        <v>928.27086363636363</v>
       </c>
       <c r="B24">
-        <v>-28.659999999999968</v>
+        <v>-2.6100000000000136</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
@@ -1373,24 +1373,24 @@
         <v>62</v>
       </c>
       <c r="E24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>912.82086363636358</v>
+        <v>911.94749999999999</v>
       </c>
       <c r="B25">
-        <v>-18.060000000000059</v>
+        <v>-69.710000000000036</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1399,24 +1399,24 @@
         <v>64</v>
       </c>
       <c r="E25">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>911.94749999999999</v>
+        <v>906.11086363636366</v>
       </c>
       <c r="B26">
-        <v>-69.710000000000036</v>
+        <v>-24.769999999999982</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
@@ -1425,24 +1425,24 @@
         <v>66</v>
       </c>
       <c r="E26">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>906.11086363636366</v>
+        <v>898.62086363636365</v>
       </c>
       <c r="B27">
-        <v>-24.769999999999982</v>
+        <v>-32.259999999999991</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
@@ -1451,16 +1451,16 @@
         <v>68</v>
       </c>
       <c r="E27">
+        <v>11</v>
+      </c>
+      <c r="F27">
+        <v>2</v>
+      </c>
+      <c r="G27">
+        <v>2</v>
+      </c>
+      <c r="H27">
         <v>7</v>
-      </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (21:39:29)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8A0E0A14-03F7-4C2F-AEE5-B8F81F510696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{281A37ED-857D-4923-978E-4BD17FAD50E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{16874035-6221-4864-A65D-A1353B0DC5BA}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{5CAA5E78-16DA-4BC0-9284-6E226C75FF81}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E31039C-8F62-4298-80C3-A0FC88ED44C1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7010920-4F4D-4D1C-B896-09D027111F1B}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (01:19:40)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{281A37ED-857D-4923-978E-4BD17FAD50E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{34CB78B9-4D69-4EA5-9D14-85D19AF0B2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{5CAA5E78-16DA-4BC0-9284-6E226C75FF81}"/>
+    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{0F75D7A4-D9D3-4413-BBAA-EA6619C02FF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,15 +65,21 @@
     <t>패</t>
   </si>
   <si>
+    <t>Voor</t>
+  </si>
+  <si>
+    <t>첼시</t>
+  </si>
+  <si>
     <t>UNIT</t>
   </si>
   <si>
+    <t>17시즌</t>
+  </si>
+  <si>
     <t>AS 로마</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>개포동덕배</t>
   </si>
   <si>
@@ -89,12 +95,6 @@
     <t>경기 수</t>
   </si>
   <si>
-    <t>Voor</t>
-  </si>
-  <si>
-    <t>첼시</t>
-  </si>
-  <si>
     <t>1부리그</t>
   </si>
   <si>
@@ -152,22 +152,28 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
   </si>
   <si>
     <t>비주류중독</t>
@@ -176,12 +182,6 @@
     <t>셀틱 FC</t>
   </si>
   <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
     <t>여수가스</t>
   </si>
   <si>
@@ -206,34 +206,34 @@
     <t>경남 FC</t>
   </si>
   <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
     <t>스페인전도사</t>
   </si>
   <si>
     <t>RC 셀타 비고</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
   </si>
   <si>
     <t>ShangHaiPortFC</t>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7010920-4F4D-4D1C-B896-09D027111F1B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A14B3B7B-48B6-4792-80CD-2D46108ED9EF}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -672,10 +672,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1155.4175</v>
+        <v>1222.1724999999999</v>
       </c>
       <c r="B2">
-        <v>124.59999999999991</v>
+        <v>97.950000000000045</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -684,39 +684,39 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F2">
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" t="s">
         <v>12</v>
-      </c>
-      <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>3</v>
-      </c>
-      <c r="J2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1153.174</v>
+        <v>1157.5340000000001</v>
       </c>
       <c r="B3">
-        <v>38.309999999999945</v>
+        <v>42.670000000000073</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>4</v>
@@ -731,13 +731,13 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -751,37 +751,37 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1128.3224999999998</v>
+        <v>1142.4875000000002</v>
       </c>
       <c r="B4">
-        <v>4.0999999999999091</v>
+        <v>111.67000000000007</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E4">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J4" t="s">
         <v>18</v>
       </c>
       <c r="K4">
-        <v>67.53</v>
+        <v>37.36999999999999</v>
       </c>
       <c r="L4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M4">
         <v>3</v>
@@ -790,15 +790,15 @@
         <v>2</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1093.6675</v>
+        <v>1105.5274999999999</v>
       </c>
       <c r="B5">
-        <v>44.710000000000036</v>
+        <v>56.569999999999936</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -822,7 +822,7 @@
         <v>21</v>
       </c>
       <c r="K5">
-        <v>19.260000000000002</v>
+        <v>18.809999999999999</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -839,10 +839,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1090.7725000000003</v>
+        <v>1098.7825000000003</v>
       </c>
       <c r="B6">
-        <v>51.160000000000082</v>
+        <v>59.170000000000073</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -866,7 +866,7 @@
         <v>24</v>
       </c>
       <c r="K6">
-        <v>37.81</v>
+        <v>55.489999999999995</v>
       </c>
       <c r="L6">
         <v>12</v>
@@ -883,10 +883,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1083.2649999999999</v>
+        <v>1079.865</v>
       </c>
       <c r="B7">
-        <v>39.099999999999909</v>
+        <v>35.700000000000045</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -895,16 +895,16 @@
         <v>26</v>
       </c>
       <c r="E7">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="s">
         <v>27</v>
@@ -927,10 +927,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1035.0690000000002</v>
+        <v>1045.4490000000003</v>
       </c>
       <c r="B8">
-        <v>-5.4500000000000455</v>
+        <v>4.9300000000000637</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -954,10 +954,10 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>124.60000000000001</v>
+        <v>111.66999999999999</v>
       </c>
       <c r="L8">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M8">
         <v>12</v>
@@ -966,15 +966,15 @@
         <v>4</v>
       </c>
       <c r="O8">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1029.7650000000001</v>
+        <v>1040.3150000000001</v>
       </c>
       <c r="B9">
-        <v>37.180000000000064</v>
+        <v>47.730000000000018</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -997,10 +997,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1027.5374999999999</v>
+        <v>1028.1575</v>
       </c>
       <c r="B10">
-        <v>-26.680000000000064</v>
+        <v>-26.059999999999945</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1020,13 +1020,19 @@
       <c r="H10">
         <v>2</v>
       </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>38</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1018.7049999999998</v>
+        <v>1023.0649999999998</v>
       </c>
       <c r="B11">
-        <v>-18.600000000000023</v>
+        <v>-14.240000000000009</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1046,13 +1052,19 @@
       <c r="H11">
         <v>5</v>
       </c>
+      <c r="J11">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="K11">
+        <v>46.750000000000007</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1001.8340000000001</v>
+        <v>1013.4508636363637</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>82.57000000000005</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
@@ -1061,24 +1073,30 @@
         <v>38</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="J12">
+        <v>1.2</v>
+      </c>
+      <c r="K12">
+        <v>55.489999999999995</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>998.58086363636369</v>
+        <v>1007.3890000000001</v>
       </c>
       <c r="B13">
-        <v>67.700000000000045</v>
+        <v>-19.480000000000018</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
@@ -1087,24 +1105,24 @@
         <v>40</v>
       </c>
       <c r="E13">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F13">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>995.99900000000014</v>
+        <v>1001.8340000000001</v>
       </c>
       <c r="B14">
-        <v>-30.870000000000005</v>
+        <v>0</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -1113,24 +1131,24 @@
         <v>42</v>
       </c>
       <c r="E14">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>974.53086363636362</v>
+        <v>1001.47</v>
       </c>
       <c r="B15">
-        <v>43.649999999999977</v>
+        <v>-5.6299999999999955</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -1139,24 +1157,24 @@
         <v>44</v>
       </c>
       <c r="E15">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>966.74</v>
+        <v>992.59086363636368</v>
       </c>
       <c r="B16">
-        <v>-40.360000000000014</v>
+        <v>61.710000000000036</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
@@ -1165,24 +1183,24 @@
         <v>46</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>965.73086363636367</v>
+        <v>976.06086363636359</v>
       </c>
       <c r="B17">
-        <v>34.850000000000023</v>
+        <v>45.17999999999995</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1205,10 +1223,10 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>953.15086363636362</v>
+        <v>962.26086363636364</v>
       </c>
       <c r="B18">
-        <v>22.269999999999982</v>
+        <v>31.379999999999995</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -1231,10 +1249,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>948.87</v>
+        <v>955.8</v>
       </c>
       <c r="B19">
-        <v>-21.149999999999977</v>
+        <v>-14.220000000000027</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1257,10 +1275,10 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>941.61900000000003</v>
+        <v>948.84900000000005</v>
       </c>
       <c r="B20">
-        <v>-10.090000000000032</v>
+        <v>-2.8600000000000136</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -1283,10 +1301,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>941.3208636363637</v>
+        <v>946.0708636363637</v>
       </c>
       <c r="B21">
-        <v>10.440000000000055</v>
+        <v>15.190000000000055</v>
       </c>
       <c r="C21" t="s">
         <v>55</v>
@@ -1295,24 +1313,24 @@
         <v>56</v>
       </c>
       <c r="E21">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="F21">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>938.33086363636369</v>
+        <v>929.3208636363637</v>
       </c>
       <c r="B22">
-        <v>7.4500000000000455</v>
+        <v>-1.5599999999999454</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1321,24 +1339,24 @@
         <v>58</v>
       </c>
       <c r="E22">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>929.4308636363636</v>
+        <v>927.1808636363636</v>
       </c>
       <c r="B23">
-        <v>-1.4500000000000455</v>
+        <v>-3.7000000000000455</v>
       </c>
       <c r="C23" t="s">
         <v>59</v>
@@ -1347,24 +1365,24 @@
         <v>60</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>928.27086363636363</v>
+        <v>922.16750000000002</v>
       </c>
       <c r="B24">
-        <v>-2.6100000000000136</v>
+        <v>-59.490000000000009</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
@@ -1373,24 +1391,24 @@
         <v>62</v>
       </c>
       <c r="E24">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F24">
         <v>3</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H24">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>911.94749999999999</v>
+        <v>921.79086363636361</v>
       </c>
       <c r="B25">
-        <v>-69.710000000000036</v>
+        <v>-9.0900000000000318</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1399,24 +1417,24 @@
         <v>64</v>
       </c>
       <c r="E25">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G25">
         <v>3</v>
       </c>
       <c r="H25">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>906.11086363636366</v>
+        <v>906.37086363636365</v>
       </c>
       <c r="B26">
-        <v>-24.769999999999982</v>
+        <v>-24.509999999999991</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
@@ -1439,10 +1457,10 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>898.62086363636365</v>
+        <v>899.15086363636362</v>
       </c>
       <c r="B27">
-        <v>-32.259999999999991</v>
+        <v>-31.730000000000018</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
@@ -1465,10 +1483,10 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>889.4408636363637</v>
+        <v>894.03086363636362</v>
       </c>
       <c r="B28">
-        <v>-41.439999999999941</v>
+        <v>-36.850000000000023</v>
       </c>
       <c r="C28" t="s">
         <v>69</v>
@@ -1491,10 +1509,10 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>874.28399999999999</v>
+        <v>879.42400000000009</v>
       </c>
       <c r="B29">
-        <v>-59.940000000000055</v>
+        <v>-54.799999999999955</v>
       </c>
       <c r="C29" t="s">
         <v>71</v>

</xml_diff>

<commit_message>
Update: Ranking Data (06:05:05)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34CB78B9-4D69-4EA5-9D14-85D19AF0B2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6171E380-D0D4-4782-8DD4-39BFF54F8F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{0F75D7A4-D9D3-4413-BBAA-EA6619C02FF5}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{EB5D6DF8-0E7D-4EC6-B786-34D4968816A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -224,16 +224,16 @@
     <t>토트넘</t>
   </si>
   <si>
+    <t>스페인전도사</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>스페인전도사</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
   </si>
   <si>
     <t>ShangHaiPortFC</t>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A14B3B7B-48B6-4792-80CD-2D46108ED9EF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{568F1821-E4A4-4868-A77F-3A1DB1C3F062}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1197,10 +1197,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>976.06086363636359</v>
+        <v>974.47086363636367</v>
       </c>
       <c r="B17">
-        <v>45.17999999999995</v>
+        <v>43.590000000000032</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1209,16 +1209,16 @@
         <v>48</v>
       </c>
       <c r="E17">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F17">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G17">
         <v>1</v>
       </c>
       <c r="H17">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
@@ -1379,10 +1379,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>922.16750000000002</v>
+        <v>923.37086363636365</v>
       </c>
       <c r="B24">
-        <v>-59.490000000000009</v>
+        <v>-7.5099999999999909</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
@@ -1391,24 +1391,24 @@
         <v>62</v>
       </c>
       <c r="E24">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F24">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G24">
         <v>3</v>
       </c>
       <c r="H24">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>921.79086363636361</v>
+        <v>922.16750000000002</v>
       </c>
       <c r="B25">
-        <v>-9.0900000000000318</v>
+        <v>-59.490000000000009</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1417,16 +1417,16 @@
         <v>64</v>
       </c>
       <c r="E25">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F25">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G25">
         <v>3</v>
       </c>
       <c r="H25">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (15:33:33)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6171E380-D0D4-4782-8DD4-39BFF54F8F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB5F242A-FCB5-4148-8D8C-3854C1FECB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{EB5D6DF8-0E7D-4EC6-B786-34D4968816A9}"/>
+    <workbookView xWindow="314" yWindow="385" windowWidth="36185" windowHeight="19575" xr2:uid="{B5D5244B-7930-4820-9551-6F42C31889C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -125,21 +125,21 @@
     <t>UEFA Tournament</t>
   </si>
   <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
     <t>마인츠</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
     <t>킹왕두</t>
   </si>
   <si>
@@ -182,18 +182,18 @@
     <t>셀틱 FC</t>
   </si>
   <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
   </si>
   <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
@@ -236,28 +236,28 @@
     <t>전북 현대 모터스</t>
   </si>
   <si>
+    <t>겐지간지</t>
+  </si>
+  <si>
+    <t>파리 생제르맹</t>
+  </si>
+  <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
     <t>ShangHaiPortFC</t>
   </si>
   <si>
     <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>겐지간지</t>
-  </si>
-  <si>
-    <t>파리 생제르맹</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
   </si>
 </sst>
 </file>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{568F1821-E4A4-4868-A77F-3A1DB1C3F062}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A75AD318-DB5E-4010-99E6-4DBD9036AE98}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -927,10 +927,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1045.4490000000003</v>
+        <v>1067.645</v>
       </c>
       <c r="B8">
-        <v>4.9300000000000637</v>
+        <v>75.059999999999945</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -939,16 +939,16 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F8">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J8" t="s">
         <v>30</v>
@@ -971,10 +971,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1040.3150000000001</v>
+        <v>1045.4490000000003</v>
       </c>
       <c r="B9">
-        <v>47.730000000000018</v>
+        <v>4.9300000000000637</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -983,16 +983,16 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F9">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -1197,10 +1197,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>974.47086363636367</v>
+        <v>977.15086363636362</v>
       </c>
       <c r="B17">
-        <v>43.590000000000032</v>
+        <v>46.269999999999982</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1209,24 +1209,24 @@
         <v>48</v>
       </c>
       <c r="E17">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F17">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>962.26086363636364</v>
+        <v>974.47086363636367</v>
       </c>
       <c r="B18">
-        <v>31.379999999999995</v>
+        <v>43.590000000000032</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -1235,16 +1235,16 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F18">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
@@ -1301,10 +1301,10 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>946.0708636363637</v>
+        <v>944.42086363636361</v>
       </c>
       <c r="B21">
-        <v>15.190000000000055</v>
+        <v>13.539999999999964</v>
       </c>
       <c r="C21" t="s">
         <v>55</v>
@@ -1313,16 +1313,16 @@
         <v>56</v>
       </c>
       <c r="E21">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -1431,10 +1431,10 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>906.37086363636365</v>
+        <v>894.03086363636362</v>
       </c>
       <c r="B26">
-        <v>-24.509999999999991</v>
+        <v>-36.850000000000023</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
@@ -1457,10 +1457,10 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>899.15086363636362</v>
+        <v>891.67086363636361</v>
       </c>
       <c r="B27">
-        <v>-31.730000000000018</v>
+        <v>-39.210000000000036</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
@@ -1469,7 +1469,7 @@
         <v>68</v>
       </c>
       <c r="E27">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F27">
         <v>2</v>
@@ -1478,15 +1478,15 @@
         <v>2</v>
       </c>
       <c r="H27">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>894.03086363636362</v>
+        <v>881.654</v>
       </c>
       <c r="B28">
-        <v>-36.850000000000023</v>
+        <v>-52.57000000000005</v>
       </c>
       <c r="C28" t="s">
         <v>69</v>
@@ -1495,24 +1495,24 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H28">
-        <v>6</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>879.42400000000009</v>
+        <v>874.17086363636361</v>
       </c>
       <c r="B29">
-        <v>-54.799999999999955</v>
+        <v>-56.710000000000036</v>
       </c>
       <c r="C29" t="s">
         <v>71</v>
@@ -1521,16 +1521,16 @@
         <v>72</v>
       </c>
       <c r="E29">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="F29">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G29">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (15:47:39)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB5F242A-FCB5-4148-8D8C-3854C1FECB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9708DFE1-BF38-4C83-935F-1D84EE545B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="385" windowWidth="36185" windowHeight="19575" xr2:uid="{B5D5244B-7930-4820-9551-6F42C31889C1}"/>
+    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{5D7B50A9-F110-441C-8191-B5B058D3A024}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A75AD318-DB5E-4010-99E6-4DBD9036AE98}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538FC0CF-9E46-4E65-81E8-6AC8D2407C35}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (23:29:21)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9708DFE1-BF38-4C83-935F-1D84EE545B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15D6A3CF-BBE8-4AD4-98CF-1583CB5C1124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="770" windowWidth="36185" windowHeight="19575" xr2:uid="{5D7B50A9-F110-441C-8191-B5B058D3A024}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{7AA21383-31F0-4A7B-8215-D6D41C99AD3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,31 +71,40 @@
     <t>첼시</t>
   </si>
   <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
     <t>UNIT</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>AS 로마</t>
   </si>
   <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>1부리그</t>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>FA컵</t>
   </si>
   <si>
     <t>검정소</t>
@@ -104,7 +113,7 @@
     <t>AC 밀란</t>
   </si>
   <si>
-    <t>FA컵</t>
+    <t>UEFA_D조</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -113,15 +122,6 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>UEFA_A조</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
     <t>UEFA Tournament</t>
   </si>
   <si>
@@ -146,54 +146,60 @@
     <t>리버풀</t>
   </si>
   <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
     <t>아들러</t>
   </si>
   <si>
     <t>프랑크푸르트</t>
   </si>
   <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
     <t>ZD장인지참치</t>
   </si>
   <si>
     <t>레버쿠젠</t>
   </si>
   <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>여수가스</t>
+  </si>
+  <si>
+    <t>AS 모나코</t>
+  </si>
+  <si>
     <t>방덕</t>
   </si>
   <si>
     <t>인테르</t>
   </si>
   <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
     <t>suma수마</t>
   </si>
   <si>
     <t>ACF 피오렌티나</t>
   </si>
   <si>
-    <t>여수가스</t>
-  </si>
-  <si>
-    <t>AS 모나코</t>
-  </si>
-  <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
@@ -206,12 +212,6 @@
     <t>경남 FC</t>
   </si>
   <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
     <t>0708ManUtd</t>
   </si>
   <si>
@@ -224,40 +224,40 @@
     <t>토트넘</t>
   </si>
   <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
     <t>스페인전도사</t>
   </si>
   <si>
     <t>RC 셀타 비고</t>
   </si>
   <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
   </si>
   <si>
     <t>겐지간지</t>
   </si>
   <si>
     <t>파리 생제르맹</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
   </si>
 </sst>
 </file>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538FC0CF-9E46-4E65-81E8-6AC8D2407C35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669FFC42-4CC7-429E-8C94-AF846B59E9C6}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -707,37 +707,37 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1157.5340000000001</v>
+        <v>1197.374</v>
       </c>
       <c r="B3">
-        <v>42.670000000000073</v>
+        <v>82.509999999999991</v>
       </c>
       <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>9</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="K3" t="s">
         <v>14</v>
       </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-      <c r="F3">
-        <v>4</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L3" t="s">
-        <v>17</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -757,10 +757,10 @@
         <v>111.67000000000007</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E4">
         <v>21</v>
@@ -778,27 +778,27 @@
         <v>18</v>
       </c>
       <c r="K4">
-        <v>37.36999999999999</v>
+        <v>17.86</v>
       </c>
       <c r="L4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M4">
         <v>3</v>
       </c>
       <c r="N4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O4">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1105.5274999999999</v>
+        <v>1120.7149999999999</v>
       </c>
       <c r="B5">
-        <v>56.569999999999936</v>
+        <v>76.549999999999955</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -813,22 +813,22 @@
         <v>6</v>
       </c>
       <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="H5">
         <v>2</v>
-      </c>
-      <c r="H5">
-        <v>3</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
       </c>
       <c r="K5">
-        <v>18.809999999999999</v>
+        <v>0</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -839,10 +839,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1098.7825000000003</v>
+        <v>1105.5274999999999</v>
       </c>
       <c r="B6">
-        <v>59.170000000000073</v>
+        <v>56.569999999999936</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -851,42 +851,42 @@
         <v>23</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F6">
         <v>6</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" t="s">
         <v>24</v>
       </c>
       <c r="K6">
-        <v>55.489999999999995</v>
+        <v>64.649999999999991</v>
       </c>
       <c r="L6">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O6">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1079.865</v>
+        <v>1098.7825000000003</v>
       </c>
       <c r="B7">
-        <v>35.700000000000045</v>
+        <v>59.170000000000073</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -895,13 +895,13 @@
         <v>26</v>
       </c>
       <c r="E7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H7">
         <v>2</v>
@@ -954,19 +954,19 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>111.66999999999999</v>
+        <v>82.509999999999991</v>
       </c>
       <c r="L8">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O8">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1029,10 +1029,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1023.0649999999998</v>
+        <v>1023.144</v>
       </c>
       <c r="B11">
-        <v>-14.240000000000009</v>
+        <v>21.309999999999945</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1041,16 +1041,16 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>1.1000000000000001</v>
@@ -1061,10 +1061,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1013.4508636363637</v>
+        <v>1023.0649999999998</v>
       </c>
       <c r="B12">
-        <v>82.57000000000005</v>
+        <v>-14.240000000000009</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
@@ -1073,16 +1073,16 @@
         <v>38</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="F12">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J12">
         <v>1.2</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1007.3890000000001</v>
+        <v>1001.47</v>
       </c>
       <c r="B13">
-        <v>-19.480000000000018</v>
+        <v>-5.6299999999999955</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
@@ -1105,24 +1105,24 @@
         <v>40</v>
       </c>
       <c r="E13">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1001.8340000000001</v>
+        <v>996.91086363636362</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>66.029999999999973</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -1131,24 +1131,24 @@
         <v>42</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1001.47</v>
+        <v>992.59086363636368</v>
       </c>
       <c r="B15">
-        <v>-5.6299999999999955</v>
+        <v>61.710000000000036</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -1157,24 +1157,24 @@
         <v>44</v>
       </c>
       <c r="E15">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>992.59086363636368</v>
+        <v>987.50086363636365</v>
       </c>
       <c r="B16">
-        <v>61.710000000000036</v>
+        <v>56.620000000000005</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
@@ -1183,24 +1183,24 @@
         <v>46</v>
       </c>
       <c r="E16">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F16">
         <v>6</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>977.15086363636362</v>
+        <v>981.77086363636363</v>
       </c>
       <c r="B17">
-        <v>46.269999999999982</v>
+        <v>50.889999999999986</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1209,24 +1209,24 @@
         <v>48</v>
       </c>
       <c r="E17">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="F17">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>974.47086363636367</v>
+        <v>973.44900000000018</v>
       </c>
       <c r="B18">
-        <v>43.590000000000032</v>
+        <v>-53.419999999999959</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -1235,24 +1235,24 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F18">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
       <c r="H18">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>955.8</v>
+        <v>957.12086363636365</v>
       </c>
       <c r="B19">
-        <v>-14.220000000000027</v>
+        <v>26.240000000000009</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1261,24 +1261,24 @@
         <v>52</v>
       </c>
       <c r="E19">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="F19">
+        <v>16</v>
+      </c>
+      <c r="G19">
         <v>2</v>
       </c>
-      <c r="G19">
-        <v>0</v>
-      </c>
       <c r="H19">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>948.84900000000005</v>
+        <v>955.8</v>
       </c>
       <c r="B20">
-        <v>-2.8600000000000136</v>
+        <v>-14.220000000000027</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -1287,24 +1287,24 @@
         <v>54</v>
       </c>
       <c r="E20">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F20">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>944.42086363636361</v>
+        <v>948.84900000000005</v>
       </c>
       <c r="B21">
-        <v>13.539999999999964</v>
+        <v>-2.8600000000000136</v>
       </c>
       <c r="C21" t="s">
         <v>55</v>
@@ -1313,24 +1313,24 @@
         <v>56</v>
       </c>
       <c r="E21">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>929.3208636363637</v>
+        <v>928.0508636363636</v>
       </c>
       <c r="B22">
-        <v>-1.5599999999999454</v>
+        <v>-2.8300000000000409</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1339,13 +1339,13 @@
         <v>58</v>
       </c>
       <c r="E22">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F22">
         <v>0</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -1379,10 +1379,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>923.37086363636365</v>
+        <v>922.16750000000002</v>
       </c>
       <c r="B24">
-        <v>-7.5099999999999909</v>
+        <v>-59.490000000000009</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
@@ -1391,24 +1391,24 @@
         <v>62</v>
       </c>
       <c r="E24">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="F24">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G24">
         <v>3</v>
       </c>
       <c r="H24">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>922.16750000000002</v>
+        <v>911.04086363636361</v>
       </c>
       <c r="B25">
-        <v>-59.490000000000009</v>
+        <v>-19.840000000000032</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1417,24 +1417,24 @@
         <v>64</v>
       </c>
       <c r="E25">
+        <v>25</v>
+      </c>
+      <c r="F25">
+        <v>7</v>
+      </c>
+      <c r="G25">
+        <v>3</v>
+      </c>
+      <c r="H25">
         <v>15</v>
-      </c>
-      <c r="F25">
-        <v>3</v>
-      </c>
-      <c r="G25">
-        <v>3</v>
-      </c>
-      <c r="H25">
-        <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>894.03086363636362</v>
+        <v>891.85086363636367</v>
       </c>
       <c r="B26">
-        <v>-36.850000000000023</v>
+        <v>-39.029999999999973</v>
       </c>
       <c r="C26" t="s">
         <v>65</v>
@@ -1443,24 +1443,24 @@
         <v>66</v>
       </c>
       <c r="E26">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>891.67086363636361</v>
+        <v>883.32400000000007</v>
       </c>
       <c r="B27">
-        <v>-39.210000000000036</v>
+        <v>-50.899999999999977</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>
@@ -1469,24 +1469,24 @@
         <v>68</v>
       </c>
       <c r="E27">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G27">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H27">
-        <v>9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>881.654</v>
+        <v>874.17086363636361</v>
       </c>
       <c r="B28">
-        <v>-52.57000000000005</v>
+        <v>-56.710000000000036</v>
       </c>
       <c r="C28" t="s">
         <v>69</v>
@@ -1495,24 +1495,24 @@
         <v>70</v>
       </c>
       <c r="E28">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="F28">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>874.17086363636361</v>
+        <v>852.85086363636367</v>
       </c>
       <c r="B29">
-        <v>-56.710000000000036</v>
+        <v>-78.029999999999973</v>
       </c>
       <c r="C29" t="s">
         <v>71</v>
@@ -1521,16 +1521,16 @@
         <v>72</v>
       </c>
       <c r="E29">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (08:14:16)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15D6A3CF-BBE8-4AD4-98CF-1583CB5C1124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AC47324-B063-4CEF-BB5B-A2F949262A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{7AA21383-31F0-4A7B-8215-D6D41C99AD3C}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{4A172D24-2D9B-4568-A3F0-111F83EBA2FF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,12 +71,18 @@
     <t>첼시</t>
   </si>
   <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
     <t>개포동덕배</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>바이에른 뮌헨</t>
   </si>
   <si>
@@ -95,13 +101,7 @@
     <t>AS 로마</t>
   </si>
   <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
+    <t>1부리그</t>
   </si>
   <si>
     <t>FA컵</t>
@@ -113,7 +113,7 @@
     <t>AC 밀란</t>
   </si>
   <si>
-    <t>UEFA_D조</t>
+    <t>UEFA_C조</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -140,6 +140,12 @@
     <t>마인츠</t>
   </si>
   <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
     <t>킹왕두</t>
   </si>
   <si>
@@ -170,12 +176,6 @@
     <t>레버쿠젠</t>
   </si>
   <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
     <t>셀래스틴</t>
   </si>
   <si>
@@ -224,16 +224,16 @@
     <t>토트넘</t>
   </si>
   <si>
+    <t>스페인전도사</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>스페인전도사</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
   </si>
   <si>
     <t>A지냐크</t>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{669FFC42-4CC7-429E-8C94-AF846B59E9C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4596F90-011A-4974-830C-E45C24A40E0E}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -713,10 +713,10 @@
         <v>82.509999999999991</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>10</v>
@@ -731,13 +731,13 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -757,10 +757,10 @@
         <v>111.67000000000007</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>21</v>
@@ -775,57 +775,57 @@
         <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K4">
-        <v>17.86</v>
+        <v>56.839999999999989</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N4">
+        <v>3</v>
+      </c>
+      <c r="O4">
         <v>1</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1120.7149999999999</v>
+        <v>1108.1849999999999</v>
       </c>
       <c r="B5">
-        <v>76.549999999999955</v>
+        <v>64.019999999999982</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E5">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G5">
         <v>3</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>-21.14</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
@@ -866,19 +866,19 @@
         <v>24</v>
       </c>
       <c r="K6">
-        <v>64.649999999999991</v>
+        <v>28.32</v>
       </c>
       <c r="L6">
         <v>6</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N6">
         <v>0</v>
       </c>
       <c r="O6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -954,19 +954,19 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>82.509999999999991</v>
+        <v>64.019999999999982</v>
       </c>
       <c r="L8">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="M8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="N8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O8">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -997,10 +997,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1028.1575</v>
+        <v>1029.8208636363636</v>
       </c>
       <c r="B10">
-        <v>-26.059999999999945</v>
+        <v>98.939999999999941</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1009,16 +1009,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1023.144</v>
+        <v>1028.1575</v>
       </c>
       <c r="B11">
-        <v>21.309999999999945</v>
+        <v>-26.059999999999945</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1041,16 +1041,16 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>2</v>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11">
-        <v>1</v>
       </c>
       <c r="J11">
         <v>1.1000000000000001</v>
@@ -1061,10 +1061,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1023.0649999999998</v>
+        <v>1023.144</v>
       </c>
       <c r="B12">
-        <v>-14.240000000000009</v>
+        <v>21.309999999999945</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
@@ -1073,16 +1073,16 @@
         <v>38</v>
       </c>
       <c r="E12">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J12">
         <v>1.2</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1001.47</v>
+        <v>1023.0649999999998</v>
       </c>
       <c r="B13">
-        <v>-5.6299999999999955</v>
+        <v>-14.240000000000009</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
@@ -1105,24 +1105,24 @@
         <v>40</v>
       </c>
       <c r="E13">
+        <v>9</v>
+      </c>
+      <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
         <v>5</v>
-      </c>
-      <c r="F13">
-        <v>2</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>996.91086363636362</v>
+        <v>1001.47</v>
       </c>
       <c r="B14">
-        <v>66.029999999999973</v>
+        <v>-5.6299999999999955</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -1131,24 +1131,24 @@
         <v>42</v>
       </c>
       <c r="E14">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="F14">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>992.59086363636368</v>
+        <v>996.91086363636362</v>
       </c>
       <c r="B15">
-        <v>61.710000000000036</v>
+        <v>66.029999999999973</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -1157,16 +1157,16 @@
         <v>44</v>
       </c>
       <c r="E15">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -1327,10 +1327,10 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>928.0508636363636</v>
+        <v>936.51086363636364</v>
       </c>
       <c r="B22">
-        <v>-2.8300000000000409</v>
+        <v>5.6299999999999955</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1339,16 +1339,16 @@
         <v>58</v>
       </c>
       <c r="E22">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22">
         <v>3</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -1379,10 +1379,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>922.16750000000002</v>
+        <v>911.04086363636361</v>
       </c>
       <c r="B24">
-        <v>-59.490000000000009</v>
+        <v>-19.840000000000032</v>
       </c>
       <c r="C24" t="s">
         <v>61</v>
@@ -1391,24 +1391,24 @@
         <v>62</v>
       </c>
       <c r="E24">
+        <v>25</v>
+      </c>
+      <c r="F24">
+        <v>7</v>
+      </c>
+      <c r="G24">
+        <v>3</v>
+      </c>
+      <c r="H24">
         <v>15</v>
-      </c>
-      <c r="F24">
-        <v>3</v>
-      </c>
-      <c r="G24">
-        <v>3</v>
-      </c>
-      <c r="H24">
-        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>911.04086363636361</v>
+        <v>898.21749999999997</v>
       </c>
       <c r="B25">
-        <v>-19.840000000000032</v>
+        <v>-83.440000000000055</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1417,16 +1417,16 @@
         <v>64</v>
       </c>
       <c r="E25">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F25">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G25">
         <v>3</v>
       </c>
       <c r="H25">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (14:11:51)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AC47324-B063-4CEF-BB5B-A2F949262A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5313D1B1-0A9A-4DC4-ABFE-0CB8995C6A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{4A172D24-2D9B-4568-A3F0-111F83EBA2FF}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{621BA48E-5518-4FF4-A5AF-8D2855986171}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -140,6 +140,12 @@
     <t>마인츠</t>
   </si>
   <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
     <t>비주류중독</t>
   </si>
   <si>
@@ -164,12 +170,6 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
     <t>ZD장인지참치</t>
   </si>
   <si>
@@ -182,16 +182,16 @@
     <t>바르셀로나</t>
   </si>
   <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
   </si>
   <si>
     <t>suma수마</t>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4596F90-011A-4974-830C-E45C24A40E0E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12A8D11-4204-4A6C-9411-0F4A11EBC98C}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -707,10 +707,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1197.374</v>
+        <v>1185.9940000000001</v>
       </c>
       <c r="B3">
-        <v>82.509999999999991</v>
+        <v>71.130000000000109</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -719,16 +719,16 @@
         <v>14</v>
       </c>
       <c r="E3">
+        <v>12</v>
+      </c>
+      <c r="F3">
         <v>10</v>
-      </c>
-      <c r="F3">
-        <v>9</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
@@ -795,10 +795,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1108.1849999999999</v>
+        <v>1107.7649999999999</v>
       </c>
       <c r="B5">
-        <v>64.019999999999982</v>
+        <v>63.599999999999909</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -866,7 +866,7 @@
         <v>24</v>
       </c>
       <c r="K6">
-        <v>28.32</v>
+        <v>27.9</v>
       </c>
       <c r="L6">
         <v>6</v>
@@ -954,7 +954,7 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>64.019999999999982</v>
+        <v>63.599999999999987</v>
       </c>
       <c r="L8">
         <v>13</v>
@@ -997,10 +997,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1029.8208636363636</v>
+        <v>1033.29</v>
       </c>
       <c r="B10">
-        <v>98.939999999999941</v>
+        <v>26.189999999999941</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1009,16 +1009,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1029,10 +1029,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1028.1575</v>
+        <v>1030.2908636363636</v>
       </c>
       <c r="B11">
-        <v>-26.059999999999945</v>
+        <v>99.409999999999968</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1041,16 +1041,16 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J11">
         <v>1.1000000000000001</v>
@@ -1061,10 +1061,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1023.144</v>
+        <v>1028.1575</v>
       </c>
       <c r="B12">
-        <v>21.309999999999945</v>
+        <v>-26.059999999999945</v>
       </c>
       <c r="C12" t="s">
         <v>37</v>
@@ -1073,16 +1073,16 @@
         <v>38</v>
       </c>
       <c r="E12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
         <v>2</v>
-      </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-      <c r="H12">
-        <v>1</v>
       </c>
       <c r="J12">
         <v>1.2</v>
@@ -1093,10 +1093,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1023.0649999999998</v>
+        <v>1023.144</v>
       </c>
       <c r="B13">
-        <v>-14.240000000000009</v>
+        <v>21.309999999999945</v>
       </c>
       <c r="C13" t="s">
         <v>39</v>
@@ -1105,24 +1105,24 @@
         <v>40</v>
       </c>
       <c r="E13">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1001.47</v>
+        <v>1023.0649999999998</v>
       </c>
       <c r="B14">
-        <v>-5.6299999999999955</v>
+        <v>-14.240000000000009</v>
       </c>
       <c r="C14" t="s">
         <v>41</v>
@@ -1131,24 +1131,24 @@
         <v>42</v>
       </c>
       <c r="E14">
+        <v>9</v>
+      </c>
+      <c r="F14">
+        <v>4</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
         <v>5</v>
-      </c>
-      <c r="F14">
-        <v>2</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>996.91086363636362</v>
+        <v>1014.8608636363637</v>
       </c>
       <c r="B15">
-        <v>66.029999999999973</v>
+        <v>83.980000000000018</v>
       </c>
       <c r="C15" t="s">
         <v>43</v>
@@ -1157,16 +1157,16 @@
         <v>44</v>
       </c>
       <c r="E15">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F15">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -1197,10 +1197,10 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>981.77086363636363</v>
+        <v>973.44900000000018</v>
       </c>
       <c r="B17">
-        <v>50.889999999999986</v>
+        <v>-53.419999999999959</v>
       </c>
       <c r="C17" t="s">
         <v>47</v>
@@ -1209,24 +1209,24 @@
         <v>48</v>
       </c>
       <c r="E17">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F17">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G17">
         <v>1</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>973.44900000000018</v>
+        <v>958.92086363636361</v>
       </c>
       <c r="B18">
-        <v>-53.419999999999959</v>
+        <v>28.039999999999964</v>
       </c>
       <c r="C18" t="s">
         <v>49</v>
@@ -1235,24 +1235,24 @@
         <v>50</v>
       </c>
       <c r="E18">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F18">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>957.12086363636365</v>
+        <v>956.67086363636361</v>
       </c>
       <c r="B19">
-        <v>26.240000000000009</v>
+        <v>25.789999999999964</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -1327,10 +1327,10 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>936.51086363636364</v>
+        <v>936.50086363636365</v>
       </c>
       <c r="B22">
-        <v>5.6299999999999955</v>
+        <v>5.6200000000000045</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
@@ -1405,10 +1405,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>898.21749999999997</v>
+        <v>898.70749999999998</v>
       </c>
       <c r="B25">
-        <v>-83.440000000000055</v>
+        <v>-82.950000000000045</v>
       </c>
       <c r="C25" t="s">
         <v>63</v>
@@ -1457,10 +1457,10 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>883.32400000000007</v>
+        <v>883.33400000000006</v>
       </c>
       <c r="B27">
-        <v>-50.899999999999977</v>
+        <v>-50.889999999999986</v>
       </c>
       <c r="C27" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Update: Ranking Data (14:14:15)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5313D1B1-0A9A-4DC4-ABFE-0CB8995C6A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D0B7205-2C30-4975-B8B3-A0FC8AC67DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{621BA48E-5518-4FF4-A5AF-8D2855986171}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{71DD982B-41FD-42B4-93A1-A1091781E57B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12A8D11-4204-4A6C-9411-0F4A11EBC98C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4BF72B8-64AF-4FDD-A549-E4E4DB890BEC}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (15:58:54)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D0B7205-2C30-4975-B8B3-A0FC8AC67DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DD8B18B-7726-4894-94D1-313D2FC0CDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{71DD982B-41FD-42B4-93A1-A1091781E57B}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{DF95977B-FB7A-4C15-A8CE-98EF5BB95DE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -640,7 +640,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4BF72B8-64AF-4FDD-A549-E4E4DB890BEC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0200C9EC-6A1F-434C-9F1E-849057A6DB27}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (20:13:05)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DD8B18B-7726-4894-94D1-313D2FC0CDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{96524FC5-A71D-4670-8D60-CE327269554A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{DF95977B-FB7A-4C15-A8CE-98EF5BB95DE3}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{9D77D0E4-5AFB-41CF-A462-4D5AC083CE51}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="90">
   <si>
     <t>17th ELO</t>
   </si>
@@ -71,39 +71,39 @@
     <t>첼시</t>
   </si>
   <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
     <t>은안</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>맨체스터 시티</t>
   </si>
   <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>1부리그</t>
-  </si>
-  <si>
     <t>FA컵</t>
   </si>
   <si>
@@ -113,7 +113,7 @@
     <t>AC 밀란</t>
   </si>
   <si>
-    <t>UEFA_C조</t>
+    <t>UEFA_A조</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -140,34 +140,46 @@
     <t>마인츠</t>
   </si>
   <si>
+    <t>킹왕두</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
     <t>콩콩콩룔</t>
   </si>
   <si>
     <t>라치오</t>
   </si>
   <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
     <t>비주류중독</t>
   </si>
   <si>
     <t>셀틱 FC</t>
   </si>
   <si>
-    <t>킹왕두</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>ZD장인지참치</t>
@@ -176,34 +188,52 @@
     <t>레버쿠젠</t>
   </si>
   <si>
+    <t>FA컵_8강</t>
+  </si>
+  <si>
     <t>셀래스틴</t>
   </si>
   <si>
     <t>바르셀로나</t>
   </si>
   <si>
+    <t>FA컵_16강</t>
+  </si>
+  <si>
     <t>방덕</t>
   </si>
   <si>
     <t>인테르</t>
   </si>
   <si>
+    <t>FA컵_32강</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
   </si>
   <si>
+    <t>UEFA</t>
+  </si>
+  <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>UCL_결승전</t>
+  </si>
+  <si>
     <t>suma수마</t>
   </si>
   <si>
     <t>ACF 피오렌티나</t>
   </si>
   <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
+    <t>UCL_4강</t>
   </si>
   <si>
     <t>경남FC가즈아</t>
@@ -212,16 +242,25 @@
     <t>경남 FC</t>
   </si>
   <si>
+    <t>UCL_8강</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>UEL_FINAL</t>
+  </si>
+  <si>
     <t>0708ManUtd</t>
   </si>
   <si>
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
+    <t>UEL_4강</t>
   </si>
   <si>
     <t>스페인전도사</t>
@@ -230,22 +269,34 @@
     <t>RC 셀타 비고</t>
   </si>
   <si>
+    <t>UEL_8강</t>
+  </si>
+  <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
   </si>
   <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
+    <t>UECL_4강</t>
   </si>
   <si>
     <t>Legend독수리</t>
   </si>
   <si>
     <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>UECL_8강</t>
   </si>
   <si>
     <t>ShangHaiPortFC</t>
@@ -640,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0200C9EC-6A1F-434C-9F1E-849057A6DB27}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C060934B-E56B-4845-B081-5FE82B00DA6B}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -672,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1222.1724999999999</v>
+        <v>1214.9424999999999</v>
       </c>
       <c r="B2">
-        <v>97.950000000000045</v>
+        <v>90.720000000000027</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -707,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1185.9940000000001</v>
+        <v>1173.3240000000001</v>
       </c>
       <c r="B3">
-        <v>71.130000000000109</v>
+        <v>58.460000000000036</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -751,16 +802,16 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1142.4875000000002</v>
+        <v>1130.2275000000002</v>
       </c>
       <c r="B4">
-        <v>111.67000000000007</v>
+        <v>99.410000000000082</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E4">
         <v>21</v>
@@ -775,36 +826,36 @@
         <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K4">
-        <v>56.839999999999989</v>
+        <v>39.370000000000005</v>
       </c>
       <c r="L4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O4">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1107.7649999999999</v>
+        <v>1097.5650000000001</v>
       </c>
       <c r="B5">
-        <v>63.599999999999909</v>
+        <v>53.400000000000091</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E5">
         <v>13</v>
@@ -822,27 +873,27 @@
         <v>21</v>
       </c>
       <c r="K5">
-        <v>-21.14</v>
+        <v>22.51</v>
       </c>
       <c r="L5">
         <v>1</v>
       </c>
       <c r="M5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5">
         <v>0</v>
       </c>
       <c r="O5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1105.5274999999999</v>
+        <v>1094.4775</v>
       </c>
       <c r="B6">
-        <v>56.569999999999936</v>
+        <v>45.519999999999982</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -866,27 +917,27 @@
         <v>24</v>
       </c>
       <c r="K6">
-        <v>27.9</v>
+        <v>37.53</v>
       </c>
       <c r="L6">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1098.7825000000003</v>
+        <v>1090.7825000000003</v>
       </c>
       <c r="B7">
-        <v>59.170000000000073</v>
+        <v>51.170000000000073</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -927,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1067.645</v>
+        <v>1058.075</v>
       </c>
       <c r="B8">
-        <v>75.059999999999945</v>
+        <v>65.490000000000009</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -954,27 +1005,27 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>63.599999999999987</v>
+        <v>99.410000000000011</v>
       </c>
       <c r="L8">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="M8">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="N8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O8">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1045.4490000000003</v>
+        <v>1037.0890000000002</v>
       </c>
       <c r="B9">
-        <v>4.9300000000000637</v>
+        <v>-3.4300000000000637</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -997,10 +1048,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1033.29</v>
+        <v>1027.7774999999999</v>
       </c>
       <c r="B10">
-        <v>26.189999999999941</v>
+        <v>-26.440000000000055</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1009,30 +1060,30 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>5</v>
-      </c>
-      <c r="J10">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J10" t="s">
+        <v>18</v>
       </c>
       <c r="K10">
-        <v>38</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1030.2908636363636</v>
+        <v>1018.8149999999998</v>
       </c>
       <c r="B11">
-        <v>99.409999999999968</v>
+        <v>-18.490000000000009</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1041,120 +1092,132 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F11">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>7</v>
-      </c>
-      <c r="J11">
-        <v>1.1000000000000001</v>
+        <v>5</v>
+      </c>
+      <c r="J11" t="s">
+        <v>37</v>
       </c>
       <c r="K11">
-        <v>46.750000000000007</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1028.1575</v>
+        <v>1018.484</v>
       </c>
       <c r="B12">
-        <v>-26.059999999999945</v>
+        <v>16.649999999999977</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>2</v>
-      </c>
-      <c r="J12">
-        <v>1.2</v>
+        <v>1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>40</v>
       </c>
       <c r="K12">
-        <v>55.489999999999995</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1023.144</v>
+        <v>1017.33</v>
       </c>
       <c r="B13">
-        <v>21.309999999999945</v>
+        <v>10.230000000000018</v>
       </c>
       <c r="C13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="J13" t="s">
+        <v>43</v>
+      </c>
+      <c r="K13">
+        <v>2.1</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1023.0649999999998</v>
+        <v>1016.5408636363636</v>
       </c>
       <c r="B14">
-        <v>-14.240000000000009</v>
+        <v>85.659999999999968</v>
       </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D14" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E14">
+        <v>19</v>
+      </c>
+      <c r="F14">
         <v>9</v>
       </c>
-      <c r="F14">
-        <v>4</v>
-      </c>
       <c r="G14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="J14" t="s">
+        <v>46</v>
+      </c>
+      <c r="K14">
+        <v>1.9</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1014.8608636363637</v>
+        <v>1002.3108636363636</v>
       </c>
       <c r="B15">
-        <v>83.980000000000018</v>
+        <v>71.42999999999995</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E15">
         <v>31</v>
@@ -1168,19 +1231,25 @@
       <c r="H15">
         <v>10</v>
       </c>
+      <c r="J15" t="s">
+        <v>49</v>
+      </c>
+      <c r="K15">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>987.50086363636365</v>
+        <v>973.90086363636362</v>
       </c>
       <c r="B16">
-        <v>56.620000000000005</v>
+        <v>43.019999999999982</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="E16">
         <v>12</v>
@@ -1194,19 +1263,25 @@
       <c r="H16">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J16" t="s">
+        <v>52</v>
+      </c>
+      <c r="K16">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>973.44900000000018</v>
+        <v>962.12900000000013</v>
       </c>
       <c r="B17">
-        <v>-53.419999999999959</v>
+        <v>-64.740000000000009</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D17" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E17">
         <v>12</v>
@@ -1220,19 +1295,25 @@
       <c r="H17">
         <v>7</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J17" t="s">
+        <v>55</v>
+      </c>
+      <c r="K17">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>958.92086363636361</v>
+        <v>952.13086363636364</v>
       </c>
       <c r="B18">
-        <v>28.039999999999964</v>
+        <v>21.25</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="E18">
         <v>23</v>
@@ -1246,71 +1327,89 @@
       <c r="H18">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J18" t="s">
+        <v>58</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>956.67086363636361</v>
+        <v>949.25</v>
       </c>
       <c r="B19">
-        <v>25.789999999999964</v>
+        <v>-20.769999999999982</v>
       </c>
       <c r="C19" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D19" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>3</v>
+      </c>
+      <c r="J19" t="s">
+        <v>61</v>
+      </c>
+      <c r="K19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>949.20086363636369</v>
+      </c>
+      <c r="B20">
+        <v>18.32000000000005</v>
+      </c>
+      <c r="C20" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20">
         <v>29</v>
       </c>
-      <c r="F19">
+      <c r="F20">
         <v>16</v>
       </c>
-      <c r="G19">
-        <v>2</v>
-      </c>
-      <c r="H19">
+      <c r="G20">
+        <v>2</v>
+      </c>
+      <c r="H20">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>955.8</v>
-      </c>
-      <c r="B20">
-        <v>-14.220000000000027</v>
-      </c>
-      <c r="C20" t="s">
-        <v>53</v>
-      </c>
-      <c r="D20" t="s">
-        <v>54</v>
-      </c>
-      <c r="E20">
-        <v>5</v>
-      </c>
-      <c r="F20">
-        <v>2</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J20" t="s">
+        <v>64</v>
+      </c>
+      <c r="K20">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>948.84900000000005</v>
+        <v>947.70900000000006</v>
       </c>
       <c r="B21">
-        <v>-2.8600000000000136</v>
+        <v>-4</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D21" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="E21">
         <v>13</v>
@@ -1324,71 +1423,89 @@
       <c r="H21">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J21" t="s">
+        <v>67</v>
+      </c>
+      <c r="K21">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>936.50086363636365</v>
+        <v>930.88086363636364</v>
       </c>
       <c r="B22">
-        <v>5.6200000000000045</v>
+        <v>0</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="E22">
+        <v>11</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>8</v>
+      </c>
+      <c r="J22" t="s">
+        <v>70</v>
+      </c>
+      <c r="K22">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>930.37086363636365</v>
+      </c>
+      <c r="B23">
+        <v>-0.50999999999999091</v>
+      </c>
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23">
         <v>7</v>
       </c>
-      <c r="F22">
+      <c r="F23">
         <v>1</v>
       </c>
-      <c r="G22">
-        <v>3</v>
-      </c>
-      <c r="H22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>927.1808636363636</v>
-      </c>
-      <c r="B23">
-        <v>-3.7000000000000455</v>
-      </c>
-      <c r="C23" t="s">
-        <v>59</v>
-      </c>
-      <c r="D23" t="s">
-        <v>60</v>
-      </c>
-      <c r="E23">
-        <v>11</v>
-      </c>
-      <c r="F23">
-        <v>3</v>
-      </c>
       <c r="G23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H23">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+      <c r="J23" t="s">
+        <v>73</v>
+      </c>
+      <c r="K23">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>911.04086363636361</v>
+        <v>903.50086363636365</v>
       </c>
       <c r="B24">
-        <v>-19.840000000000032</v>
+        <v>-27.379999999999995</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E24">
         <v>25</v>
@@ -1402,71 +1519,89 @@
       <c r="H24">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J24" t="s">
+        <v>76</v>
+      </c>
+      <c r="K24">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>898.70749999999998</v>
+        <v>889.98086363636367</v>
       </c>
       <c r="B25">
-        <v>-82.950000000000045</v>
+        <v>-40.899999999999977</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>77</v>
       </c>
       <c r="D25" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="E25">
+        <v>15</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25">
+        <v>10</v>
+      </c>
+      <c r="J25" t="s">
+        <v>79</v>
+      </c>
+      <c r="K25">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>888.03750000000002</v>
+      </c>
+      <c r="B26">
+        <v>-93.62</v>
+      </c>
+      <c r="C26" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26">
         <v>17</v>
       </c>
-      <c r="F25">
-        <v>3</v>
-      </c>
-      <c r="G25">
-        <v>3</v>
-      </c>
-      <c r="H25">
+      <c r="F26">
+        <v>3</v>
+      </c>
+      <c r="G26">
+        <v>3</v>
+      </c>
+      <c r="H26">
         <v>11</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A26">
-        <v>891.85086363636367</v>
-      </c>
-      <c r="B26">
-        <v>-39.029999999999973</v>
-      </c>
-      <c r="C26" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" t="s">
-        <v>66</v>
-      </c>
-      <c r="E26">
-        <v>15</v>
-      </c>
-      <c r="F26">
-        <v>3</v>
-      </c>
-      <c r="G26">
-        <v>2</v>
-      </c>
-      <c r="H26">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J26" t="s">
+        <v>82</v>
+      </c>
+      <c r="K26">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>883.33400000000006</v>
+        <v>878.71400000000006</v>
       </c>
       <c r="B27">
-        <v>-50.889999999999986</v>
+        <v>-55.509999999999991</v>
       </c>
       <c r="C27" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E27">
         <v>39</v>
@@ -1480,19 +1615,25 @@
       <c r="H27">
         <v>23</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="J27" t="s">
+        <v>85</v>
+      </c>
+      <c r="K27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>874.17086363636361</v>
+        <v>874.1808636363636</v>
       </c>
       <c r="B28">
-        <v>-56.710000000000036</v>
+        <v>-56.700000000000045</v>
       </c>
       <c r="C28" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="D28" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="E28">
         <v>15</v>
@@ -1507,18 +1648,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>852.85086363636367</v>
+        <v>847.97086363636367</v>
       </c>
       <c r="B29">
-        <v>-78.029999999999973</v>
+        <v>-82.909999999999968</v>
       </c>
       <c r="C29" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="D29" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="E29">
         <v>17</v>

</xml_diff>

<commit_message>
Update: Ranking Data (11:38:50)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96524FC5-A71D-4670-8D60-CE327269554A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDB039B7-E748-4E27-98C8-DF4E32BC3BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{9D77D0E4-5AFB-41CF-A462-4D5AC083CE51}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{EFB269EA-E02A-4550-B245-737823121798}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -116,24 +116,30 @@
     <t>UEFA_A조</t>
   </si>
   <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
     <t>Special블루</t>
   </si>
   <si>
     <t>아스널</t>
   </si>
   <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
     <t>전체 합계</t>
   </si>
   <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
@@ -146,13 +152,16 @@
     <t>리버풀</t>
   </si>
   <si>
+    <t>2부리그</t>
+  </si>
+  <si>
     <t>아들러</t>
   </si>
   <si>
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>2부리그</t>
+    <t>3부리그</t>
   </si>
   <si>
     <t>호야국2인</t>
@@ -161,15 +170,6 @@
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
     <t>FA컵_결승전</t>
   </si>
   <si>
@@ -209,55 +209,55 @@
     <t>FA컵_32강</t>
   </si>
   <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>UEFA</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
   </si>
   <si>
-    <t>UEFA</t>
+    <t>UCL_결승전</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>UCL_4강</t>
+  </si>
+  <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
+    <t>UCL_8강</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>UEL_FINAL</t>
   </si>
   <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
     <t>함부르크SV</t>
-  </si>
-  <si>
-    <t>UCL_결승전</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>UCL_4강</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
-  </si>
-  <si>
-    <t>UCL_8강</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
-    <t>UEL_FINAL</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
   </si>
   <si>
     <t>UEL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C060934B-E56B-4845-B081-5FE82B00DA6B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22A6A7B1-F850-4709-8D88-0E2F49D858D1}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1214.9424999999999</v>
+        <v>1211.5424999999998</v>
       </c>
       <c r="B2">
-        <v>90.720000000000027</v>
+        <v>87.319999999999936</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -735,16 +735,16 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1173.3240000000001</v>
+        <v>1186.7239999999999</v>
       </c>
       <c r="B3">
-        <v>58.460000000000036</v>
+        <v>71.8599999999999</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,10 +770,10 @@
         <v>14</v>
       </c>
       <c r="E3">
+        <v>14</v>
+      </c>
+      <c r="F3">
         <v>12</v>
-      </c>
-      <c r="F3">
-        <v>10</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1090.7825000000003</v>
+        <v>1075.5050000000001</v>
       </c>
       <c r="B7">
-        <v>51.170000000000073</v>
+        <v>82.920000000000073</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -946,16 +946,16 @@
         <v>26</v>
       </c>
       <c r="E7">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" t="s">
         <v>27</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1058.075</v>
+        <v>1074.1525000000001</v>
       </c>
       <c r="B8">
-        <v>65.490000000000009</v>
+        <v>34.539999999999964</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -990,13 +990,13 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F8">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H8">
         <v>3</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1037.0890000000002</v>
+        <v>1054.5</v>
       </c>
       <c r="B9">
-        <v>-3.4300000000000637</v>
+        <v>47.399999999999977</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1034,13 +1034,13 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F9">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H9">
         <v>6</v>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1027.7774999999999</v>
+        <v>1037.0890000000002</v>
       </c>
       <c r="B10">
-        <v>-26.440000000000055</v>
+        <v>-3.4300000000000637</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1060,16 +1060,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H10">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J10" t="s">
         <v>18</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1018.8149999999998</v>
+        <v>1027.7774999999999</v>
       </c>
       <c r="B11">
-        <v>-18.490000000000009</v>
+        <v>-26.440000000000055</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1092,16 +1092,16 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J11" t="s">
         <v>37</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1018.484</v>
+        <v>1018.8149999999998</v>
       </c>
       <c r="B12">
-        <v>16.649999999999977</v>
+        <v>-18.490000000000009</v>
       </c>
       <c r="C12" t="s">
         <v>38</v>
@@ -1124,16 +1124,16 @@
         <v>39</v>
       </c>
       <c r="E12">
+        <v>9</v>
+      </c>
+      <c r="F12">
         <v>4</v>
       </c>
-      <c r="F12">
-        <v>2</v>
-      </c>
       <c r="G12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J12" t="s">
         <v>40</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1017.33</v>
+        <v>1018.484</v>
       </c>
       <c r="B13">
-        <v>10.230000000000018</v>
+        <v>16.649999999999977</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,16 +1156,16 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J13" t="s">
         <v>43</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1002.3108636363636</v>
+        <v>1009.8008636363636</v>
       </c>
       <c r="B15">
-        <v>71.42999999999995</v>
+        <v>78.919999999999959</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1220,10 +1220,10 @@
         <v>48</v>
       </c>
       <c r="E15">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F15">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G15">
         <v>3</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>973.90086363636362</v>
+        <v>967.85086363636367</v>
       </c>
       <c r="B16">
-        <v>43.019999999999982</v>
+        <v>36.970000000000027</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F16">
         <v>6</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>952.13086363636364</v>
+        <v>959.38086363636364</v>
       </c>
       <c r="B18">
-        <v>21.25</v>
+        <v>28.5</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="F18">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>949.25</v>
+        <v>952.13086363636364</v>
       </c>
       <c r="B19">
-        <v>-20.769999999999982</v>
+        <v>21.25</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="F19">
+        <v>13</v>
+      </c>
+      <c r="G19">
         <v>2</v>
       </c>
-      <c r="G19">
-        <v>0</v>
-      </c>
       <c r="H19">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>930.37086363636365</v>
+        <v>905.8</v>
       </c>
       <c r="B23">
-        <v>-0.50999999999999091</v>
+        <v>-64.220000000000027</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
+        <v>9</v>
+      </c>
+      <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
         <v>7</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>3</v>
-      </c>
-      <c r="H23">
-        <v>3</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
Update: Ranking Data (11:42:58)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDB039B7-E748-4E27-98C8-DF4E32BC3BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD1B3DE5-9BB4-4507-9FC7-14427107C867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{EFB269EA-E02A-4550-B245-737823121798}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{6972D477-0A5C-4AB7-AD16-595B22EA5347}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22A6A7B1-F850-4709-8D88-0E2F49D858D1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15A07E14-E3C2-456A-A426-6083007ACACD}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (23:22:16)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD1B3DE5-9BB4-4507-9FC7-14427107C867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D56E787-DBA7-4522-AA70-8744DA9E18E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{6972D477-0A5C-4AB7-AD16-595B22EA5347}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{F6F3A7B2-5887-42FE-96CF-97FC4FCD5D25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,81 +71,90 @@
     <t>첼시</t>
   </si>
   <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
     <t>UNIT</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>AS 로마</t>
   </si>
   <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
+    <t>3부리그</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>UEFA_D조</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
   </si>
   <si>
     <t>1부리그</t>
   </si>
   <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>UEFA_A조</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
     <t>킹왕두</t>
   </si>
   <si>
@@ -161,9 +170,6 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>3부리그</t>
-  </si>
-  <si>
     <t>호야국2인</t>
   </si>
   <si>
@@ -182,22 +188,25 @@
     <t>FA컵_4강</t>
   </si>
   <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
     <t>FA컵_8강</t>
   </si>
   <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>FA컵_16강</t>
+  </si>
+  <si>
     <t>셀래스틴</t>
   </si>
   <si>
     <t>바르셀로나</t>
   </si>
   <si>
-    <t>FA컵_16강</t>
+    <t>FA컵_32강</t>
   </si>
   <si>
     <t>방덕</t>
@@ -206,25 +215,34 @@
     <t>인테르</t>
   </si>
   <si>
-    <t>FA컵_32강</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
     <t>UEFA</t>
   </si>
   <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>UCL_결승전</t>
+  </si>
+  <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
+    <t>UCL_4강</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
   </si>
   <si>
-    <t>UCL_결승전</t>
+    <t>UCL_8강</t>
   </si>
   <si>
     <t>suma수마</t>
@@ -233,24 +251,6 @@
     <t>ACF 피오렌티나</t>
   </si>
   <si>
-    <t>UCL_4강</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
-  </si>
-  <si>
-    <t>UCL_8강</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
     <t>UEL_FINAL</t>
   </si>
   <si>
@@ -272,37 +272,37 @@
     <t>UEL_8강</t>
   </si>
   <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>UECL_4강</t>
+  </si>
+  <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
+  </si>
+  <si>
+    <t>UECL_8강</t>
+  </si>
+  <si>
     <t>A지냐크</t>
   </si>
   <si>
     <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>UECL_4강</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
-  </si>
-  <si>
-    <t>UECL_8강</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
   </si>
   <si>
     <t>겐지간지</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15A07E14-E3C2-456A-A426-6083007ACACD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11B339A5-07E3-41B4-BB91-4D96F3A6DFBC}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1211.5424999999998</v>
+        <v>1220.0024999999998</v>
       </c>
       <c r="B2">
-        <v>87.319999999999936</v>
+        <v>95.779999999999973</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -735,10 +735,10 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -808,10 +808,10 @@
         <v>99.410000000000082</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>21</v>
@@ -826,22 +826,22 @@
         <v>5</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K4">
-        <v>39.370000000000005</v>
+        <v>27.469999999999995</v>
       </c>
       <c r="L4">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="M4">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="N4">
         <v>2</v>
       </c>
       <c r="O4">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -852,10 +852,10 @@
         <v>53.400000000000091</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5">
         <v>13</v>
@@ -870,10 +870,10 @@
         <v>3</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K5">
-        <v>22.51</v>
+        <v>22.98</v>
       </c>
       <c r="L5">
         <v>1</v>
@@ -896,10 +896,10 @@
         <v>45.519999999999982</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>11</v>
@@ -914,51 +914,51 @@
         <v>3</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>37.53</v>
+        <v>28.520000000000003</v>
       </c>
       <c r="L6">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1075.5050000000001</v>
+        <v>1074.1525000000001</v>
       </c>
       <c r="B7">
-        <v>82.920000000000073</v>
+        <v>34.539999999999964</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E7">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="G7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H7">
         <v>3</v>
       </c>
       <c r="J7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -978,46 +978,46 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1074.1525000000001</v>
+        <v>1070.2550000000001</v>
       </c>
       <c r="B8">
-        <v>34.539999999999964</v>
+        <v>77.670000000000073</v>
       </c>
       <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8">
         <v>28</v>
       </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8">
+      <c r="F8">
+        <v>17</v>
+      </c>
+      <c r="G8">
+        <v>7</v>
+      </c>
+      <c r="H8">
+        <v>4</v>
+      </c>
+      <c r="J8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8">
+        <v>78.97</v>
+      </c>
+      <c r="L8">
+        <v>33</v>
+      </c>
+      <c r="M8">
+        <v>20</v>
+      </c>
+      <c r="N8">
+        <v>3</v>
+      </c>
+      <c r="O8">
         <v>10</v>
-      </c>
-      <c r="F8">
-        <v>6</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8">
-        <v>3</v>
-      </c>
-      <c r="J8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K8">
-        <v>99.410000000000011</v>
-      </c>
-      <c r="L8">
-        <v>21</v>
-      </c>
-      <c r="M8">
-        <v>12</v>
-      </c>
-      <c r="N8">
-        <v>4</v>
-      </c>
-      <c r="O8">
-        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1028,10 +1028,10 @@
         <v>47.399999999999977</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E9">
         <v>13</v>
@@ -1048,31 +1048,31 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1037.0890000000002</v>
+        <v>1035.5690000000002</v>
       </c>
       <c r="B10">
-        <v>-3.4300000000000637</v>
+        <v>-4.9500000000000455</v>
       </c>
       <c r="C10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E10">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F10">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J10" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1086,10 +1086,10 @@
         <v>-26.440000000000055</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E11">
         <v>2</v>
@@ -1104,7 +1104,7 @@
         <v>2</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -1118,10 +1118,10 @@
         <v>-18.490000000000009</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E12">
         <v>9</v>
@@ -1136,7 +1136,7 @@
         <v>5</v>
       </c>
       <c r="J12" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K12">
         <v>0.3</v>
@@ -1150,10 +1150,10 @@
         <v>16.649999999999977</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -1168,7 +1168,7 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K13">
         <v>2.1</v>
@@ -1182,10 +1182,10 @@
         <v>85.659999999999968</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E14">
         <v>19</v>
@@ -1200,7 +1200,7 @@
         <v>7</v>
       </c>
       <c r="J14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K14">
         <v>1.9</v>
@@ -1208,16 +1208,16 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1009.8008636363636</v>
+        <v>1009.8508636363637</v>
       </c>
       <c r="B15">
-        <v>78.919999999999959</v>
+        <v>78.970000000000027</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="E15">
         <v>33</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>967.85086363636367</v>
+        <v>982.97086363636367</v>
       </c>
       <c r="B16">
-        <v>36.970000000000027</v>
+        <v>52.090000000000032</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>962.12900000000013</v>
+        <v>967.85086363636367</v>
       </c>
       <c r="B17">
-        <v>-64.740000000000009</v>
+        <v>36.970000000000027</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H17">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>959.38086363636364</v>
+        <v>962.12900000000013</v>
       </c>
       <c r="B18">
-        <v>28.5</v>
+        <v>-64.740000000000009</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F18">
         <v>4</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>952.13086363636364</v>
+        <v>959.89086363636363</v>
       </c>
       <c r="B19">
-        <v>21.25</v>
+        <v>29.009999999999991</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F19">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
@@ -1368,10 +1368,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>949.20086363636369</v>
+        <v>958.65900000000011</v>
       </c>
       <c r="B20">
-        <v>18.32000000000005</v>
+        <v>6.9500000000000455</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,16 +1380,16 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F20">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>947.70900000000006</v>
+        <v>952.13086363636364</v>
       </c>
       <c r="B21">
-        <v>-4</v>
+        <v>21.25</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
+        <v>23</v>
+      </c>
+      <c r="F21">
         <v>13</v>
-      </c>
-      <c r="F21">
-        <v>6</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>930.88086363636364</v>
+        <v>920.42086363636361</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>-10.460000000000036</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,16 +1444,16 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="J22" t="s">
         <v>70</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>905.8</v>
+        <v>906.48</v>
       </c>
       <c r="B23">
-        <v>-64.220000000000027</v>
+        <v>-63.539999999999964</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>889.98086363636367</v>
+        <v>888.03750000000002</v>
       </c>
       <c r="B25">
-        <v>-40.899999999999977</v>
+        <v>-93.62</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,16 +1540,16 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F25">
         <v>3</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>888.03750000000002</v>
+        <v>878.71400000000006</v>
       </c>
       <c r="B26">
-        <v>-93.62</v>
+        <v>-55.509999999999991</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H26">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1592,10 +1592,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>878.71400000000006</v>
+        <v>866.87086363636365</v>
       </c>
       <c r="B27">
-        <v>-55.509999999999991</v>
+        <v>-64.009999999999991</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,16 +1604,16 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="F27">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="J27" t="s">
         <v>85</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>874.1808636363636</v>
+        <v>862.17086363636361</v>
       </c>
       <c r="B28">
-        <v>-56.700000000000045</v>
+        <v>-68.710000000000036</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,16 +1636,16 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H28">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (04:38:21)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D56E787-DBA7-4522-AA70-8744DA9E18E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9154495-72D9-4F57-9D62-F5844D6BBD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{F6F3A7B2-5887-42FE-96CF-97FC4FCD5D25}"/>
+    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{AAC5866D-8DEA-439F-96B9-579164AEC16C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11B339A5-07E3-41B4-BB91-4D96F3A6DFBC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{741D0B83-0E36-43DB-86D7-830265EDD5E2}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (03:00:45)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9154495-72D9-4F57-9D62-F5844D6BBD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{92A8EF2D-36E2-4DD6-B3E1-759CF1096D03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="955" windowWidth="36185" windowHeight="19576" xr2:uid="{AAC5866D-8DEA-439F-96B9-579164AEC16C}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{F223174A-6B61-4EBD-928D-0C8B95FBB1D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -122,21 +122,21 @@
     <t>UEFA_D조</t>
   </si>
   <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
     <t>Special블루</t>
   </si>
   <si>
     <t>아스널</t>
   </si>
   <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
     <t>전체 합계</t>
   </si>
   <si>
@@ -155,21 +155,21 @@
     <t>1부리그</t>
   </si>
   <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
     <t>킹왕두</t>
   </si>
   <si>
     <t>리버풀</t>
   </si>
   <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
-  </si>
-  <si>
     <t>호야국2인</t>
   </si>
   <si>
@@ -227,19 +227,19 @@
     <t>UCL_결승전</t>
   </si>
   <si>
+    <t>여수가스</t>
+  </si>
+  <si>
+    <t>AS 모나코</t>
+  </si>
+  <si>
+    <t>UCL_4강</t>
+  </si>
+  <si>
     <t>경남FC가즈아</t>
   </si>
   <si>
     <t>경남 FC</t>
-  </si>
-  <si>
-    <t>UCL_4강</t>
-  </si>
-  <si>
-    <t>여수가스</t>
-  </si>
-  <si>
-    <t>AS 모나코</t>
   </si>
   <si>
     <t>UCL_8강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{741D0B83-0E36-43DB-86D7-830265EDD5E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A38ACE6-52E3-4659-8FDD-06E3BB10B006}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -829,19 +829,19 @@
         <v>20</v>
       </c>
       <c r="K4">
-        <v>27.469999999999995</v>
+        <v>24.209999999999997</v>
       </c>
       <c r="L4">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="M4">
         <v>14</v>
       </c>
       <c r="N4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -917,27 +917,27 @@
         <v>26</v>
       </c>
       <c r="K6">
-        <v>28.520000000000003</v>
+        <v>31.770000000000003</v>
       </c>
       <c r="L6">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N6">
         <v>1</v>
       </c>
       <c r="O6">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1074.1525000000001</v>
+        <v>1075.325</v>
       </c>
       <c r="B7">
-        <v>34.539999999999964</v>
+        <v>82.740000000000009</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -946,16 +946,16 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7" t="s">
         <v>29</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1070.2550000000001</v>
+        <v>1074.1525000000001</v>
       </c>
       <c r="B8">
-        <v>77.670000000000073</v>
+        <v>34.539999999999964</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,42 +990,42 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="F8">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
       </c>
       <c r="K8">
-        <v>78.97</v>
+        <v>78.960000000000008</v>
       </c>
       <c r="L8">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="M8">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O8">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1054.5</v>
+        <v>1057.23</v>
       </c>
       <c r="B9">
-        <v>47.399999999999977</v>
+        <v>50.129999999999995</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1034,24 +1034,24 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F9">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1035.5690000000002</v>
+        <v>1040.3790000000001</v>
       </c>
       <c r="B10">
-        <v>-4.9500000000000455</v>
+        <v>-0.14000000000010004</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1060,10 +1060,10 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F10">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G10">
         <v>6</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1027.7774999999999</v>
+        <v>1029.0049999999999</v>
       </c>
       <c r="B11">
-        <v>-26.440000000000055</v>
+        <v>-8.2999999999999545</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,16 +1092,16 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1018.8149999999998</v>
+        <v>1027.7774999999999</v>
       </c>
       <c r="B12">
-        <v>-18.490000000000009</v>
+        <v>-26.440000000000055</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,16 +1124,16 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1009.8508636363637</v>
+        <v>1009.8408636363637</v>
       </c>
       <c r="B15">
-        <v>78.970000000000027</v>
+        <v>78.960000000000036</v>
       </c>
       <c r="C15" t="s">
         <v>10</v>
@@ -1220,16 +1220,16 @@
         <v>12</v>
       </c>
       <c r="E15">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F15">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J15" t="s">
         <v>49</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>982.97086363636367</v>
+        <v>1002.0008636363636</v>
       </c>
       <c r="B16">
-        <v>52.090000000000032</v>
+        <v>71.12</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,10 +1252,10 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F16">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G16">
         <v>4</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>967.85086363636367</v>
+        <v>965.97086363636367</v>
       </c>
       <c r="B17">
-        <v>36.970000000000027</v>
+        <v>35.090000000000032</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F17">
         <v>6</v>
       </c>
       <c r="G17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1368,10 +1368,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>958.65900000000011</v>
+        <v>952.13086363636364</v>
       </c>
       <c r="B20">
-        <v>6.9500000000000455</v>
+        <v>21.25</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,16 +1380,16 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>952.13086363636364</v>
+        <v>943.30900000000008</v>
       </c>
       <c r="B21">
-        <v>21.25</v>
+        <v>-8.3999999999999773</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1415,13 +1415,13 @@
         <v>23</v>
       </c>
       <c r="F21">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1650,10 +1650,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>847.97086363636367</v>
+        <v>824.90086363636362</v>
       </c>
       <c r="B29">
-        <v>-82.909999999999968</v>
+        <v>-105.98000000000002</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1662,7 +1662,7 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F29">
         <v>3</v>
@@ -1671,7 +1671,7 @@
         <v>0</v>
       </c>
       <c r="H29">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (03:17:38)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{92A8EF2D-36E2-4DD6-B3E1-759CF1096D03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2EEE746-B0F7-49EC-96E5-9D3CD23ED870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{F223174A-6B61-4EBD-928D-0C8B95FBB1D6}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{A403DBE8-227E-49E0-AB44-ED3DE30F7C19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A38ACE6-52E3-4659-8FDD-06E3BB10B006}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3032FA4E-8225-4894-9860-F5D40B738964}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1002.0008636363636</v>
+        <v>1000.5408636363636</v>
       </c>
       <c r="B16">
-        <v>71.12</v>
+        <v>69.659999999999968</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G16">
         <v>4</v>
       </c>
       <c r="H16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1368,10 +1368,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>952.13086363636364</v>
+        <v>953.60086363636367</v>
       </c>
       <c r="B20">
-        <v>21.25</v>
+        <v>22.720000000000027</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,16 +1380,16 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F20">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Update: Ranking Data (19:22:13)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2EEE746-B0F7-49EC-96E5-9D3CD23ED870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AECAE31B-3FE2-4BBD-BB82-C48CE2DE4CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{A403DBE8-227E-49E0-AB44-ED3DE30F7C19}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{18D55A86-2F14-4804-8017-CA3BF2B1FA30}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -104,55 +104,64 @@
     <t>3부리그</t>
   </si>
   <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>UEFA_D조</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>은안</t>
   </si>
   <si>
     <t>맨체스터 시티</t>
   </si>
   <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>UEFA_D조</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
     <t>콩콩콩룔</t>
   </si>
   <si>
     <t>라치오</t>
   </si>
   <si>
+    <t>1부리그</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
     <t>마인츠</t>
   </si>
   <si>
-    <t>1부리그</t>
+    <t>2부리그</t>
   </si>
   <si>
     <t>아들러</t>
@@ -161,7 +170,7 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>2부리그</t>
+    <t>FA컵_결승전</t>
   </si>
   <si>
     <t>킹왕두</t>
@@ -170,13 +179,16 @@
     <t>리버풀</t>
   </si>
   <si>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_8강</t>
   </si>
   <si>
     <t>비주류중독</t>
@@ -185,10 +197,7 @@
     <t>셀틱 FC</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
+    <t>FA컵_16강</t>
   </si>
   <si>
     <t>0708ManUtd</t>
@@ -197,7 +206,7 @@
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>FA컵_16강</t>
+    <t>FA컵_32강</t>
   </si>
   <si>
     <t>셀래스틴</t>
@@ -206,15 +215,6 @@
     <t>바르셀로나</t>
   </si>
   <si>
-    <t>FA컵_32강</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
     <t>UEFA</t>
   </si>
   <si>
@@ -290,19 +290,19 @@
     <t>UECL_4강</t>
   </si>
   <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>UECL_8강</t>
+  </si>
+  <si>
     <t>ShangHaiPortFC</t>
   </si>
   <si>
     <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>UECL_8강</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
   </si>
   <si>
     <t>겐지간지</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3032FA4E-8225-4894-9860-F5D40B738964}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A75418F9-C858-4E31-A4D2-0C4C3B36E58D}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -829,27 +829,27 @@
         <v>20</v>
       </c>
       <c r="K4">
-        <v>24.209999999999997</v>
+        <v>22.979999999999997</v>
       </c>
       <c r="L4">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N4">
         <v>3</v>
       </c>
       <c r="O4">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1097.5650000000001</v>
+        <v>1094.4775</v>
       </c>
       <c r="B5">
-        <v>53.400000000000091</v>
+        <v>45.519999999999982</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -858,13 +858,13 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5">
         <v>3</v>
@@ -873,16 +873,16 @@
         <v>23</v>
       </c>
       <c r="K5">
-        <v>22.98</v>
+        <v>23.44</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5">
         <v>1</v>
       </c>
       <c r="N5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1094.4775</v>
+        <v>1075.325</v>
       </c>
       <c r="B6">
-        <v>45.519999999999982</v>
+        <v>82.740000000000009</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -902,16 +902,16 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" t="s">
         <v>26</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1075.325</v>
+        <v>1074.1525000000001</v>
       </c>
       <c r="B7">
-        <v>82.740000000000009</v>
+        <v>34.539999999999964</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -946,16 +946,16 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" t="s">
         <v>29</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1074.1525000000001</v>
+        <v>1064.1590000000001</v>
       </c>
       <c r="B8">
-        <v>34.539999999999964</v>
+        <v>37.289999999999964</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,42 +990,42 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
       </c>
       <c r="K8">
-        <v>78.960000000000008</v>
+        <v>78.19</v>
       </c>
       <c r="L8">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="M8">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1057.23</v>
+        <v>1061.7349999999999</v>
       </c>
       <c r="B9">
-        <v>50.129999999999995</v>
+        <v>17.569999999999936</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1034,24 +1034,24 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1040.3790000000001</v>
+        <v>1057.23</v>
       </c>
       <c r="B10">
-        <v>-0.14000000000010004</v>
+        <v>50.129999999999995</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1060,13 +1060,13 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F10">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="G10">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H10">
         <v>7</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1029.0049999999999</v>
+        <v>1040.3790000000001</v>
       </c>
       <c r="B11">
-        <v>-8.2999999999999545</v>
+        <v>-0.14000000000010004</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,13 +1092,13 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H11">
         <v>7</v>
@@ -1112,28 +1112,28 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1027.7774999999999</v>
+        <v>1033.0708636363636</v>
       </c>
       <c r="B12">
-        <v>-26.440000000000055</v>
+        <v>102.18999999999994</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,31 +1144,31 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1018.484</v>
+        <v>1029.0049999999999</v>
       </c>
       <c r="B13">
-        <v>16.649999999999977</v>
+        <v>-8.2999999999999545</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="K13">
         <v>2.1</v>
@@ -1176,31 +1176,31 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1016.5408636363636</v>
+        <v>1027.7774999999999</v>
       </c>
       <c r="B14">
-        <v>85.659999999999968</v>
+        <v>-26.440000000000055</v>
       </c>
       <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14">
+        <v>2</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>2</v>
+      </c>
+      <c r="J14" t="s">
         <v>46</v>
-      </c>
-      <c r="D14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14">
-        <v>19</v>
-      </c>
-      <c r="F14">
-        <v>9</v>
-      </c>
-      <c r="G14">
-        <v>3</v>
-      </c>
-      <c r="H14">
-        <v>7</v>
-      </c>
-      <c r="J14" t="s">
-        <v>48</v>
       </c>
       <c r="K14">
         <v>1.9</v>
@@ -1208,28 +1208,28 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1009.8408636363637</v>
+        <v>1018.484</v>
       </c>
       <c r="B15">
-        <v>78.960000000000036</v>
+        <v>16.649999999999977</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="E15">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="F15">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H15">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="J15" t="s">
         <v>49</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1000.5408636363636</v>
+        <v>1001.3508636363637</v>
       </c>
       <c r="B16">
-        <v>69.659999999999968</v>
+        <v>70.470000000000027</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F16">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G16">
         <v>4</v>
       </c>
       <c r="H16">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>965.97086363636367</v>
+        <v>1000.5408636363636</v>
       </c>
       <c r="B17">
-        <v>35.090000000000032</v>
+        <v>69.659999999999968</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F17">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G17">
         <v>4</v>
       </c>
       <c r="H17">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>962.12900000000013</v>
+        <v>965.97086363636367</v>
       </c>
       <c r="B18">
-        <v>-64.740000000000009</v>
+        <v>35.090000000000032</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F18">
+        <v>6</v>
+      </c>
+      <c r="G18">
         <v>4</v>
       </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
       <c r="H18">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>959.89086363636363</v>
+        <v>961.11086363636366</v>
       </c>
       <c r="B19">
-        <v>29.009999999999991</v>
+        <v>30.230000000000018</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,30 +1348,30 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G19">
         <v>4</v>
       </c>
       <c r="H19">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
       </c>
       <c r="K19">
-        <v>2</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>953.60086363636367</v>
+        <v>946.61086363636366</v>
       </c>
       <c r="B20">
-        <v>22.720000000000027</v>
+        <v>15.730000000000018</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,22 +1380,22 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F20">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
       </c>
       <c r="K20">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
@@ -1427,7 +1427,7 @@
         <v>67</v>
       </c>
       <c r="K21">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
@@ -1459,7 +1459,7 @@
         <v>70</v>
       </c>
       <c r="K22">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
@@ -1555,7 +1555,7 @@
         <v>79</v>
       </c>
       <c r="K25">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
@@ -1592,10 +1592,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>866.87086363636365</v>
+        <v>862.17086363636361</v>
       </c>
       <c r="B27">
-        <v>-64.009999999999991</v>
+        <v>-68.710000000000036</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,30 +1604,30 @@
         <v>84</v>
       </c>
       <c r="E27">
+        <v>25</v>
+      </c>
+      <c r="F27">
+        <v>3</v>
+      </c>
+      <c r="G27">
+        <v>5</v>
+      </c>
+      <c r="H27">
         <v>17</v>
-      </c>
-      <c r="F27">
-        <v>2</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>15</v>
       </c>
       <c r="J27" t="s">
         <v>85</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>862.17086363636361</v>
+        <v>859.4308636363636</v>
       </c>
       <c r="B28">
-        <v>-68.710000000000036</v>
+        <v>-71.450000000000045</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,13 +1636,13 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H28">
         <v>17</v>

</xml_diff>

<commit_message>
Update: Ranking Data (13:47:14)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AECAE31B-3FE2-4BBD-BB82-C48CE2DE4CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C940AF0-0452-485F-A5E4-33F373268A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{18D55A86-2F14-4804-8017-CA3BF2B1FA30}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{F480BE97-D90C-4B1A-9DFB-10E26CFA4FE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A75418F9-C858-4E31-A4D2-0C4C3B36E58D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFCBDFDF-7C45-4F6A-A7D2-9355A3A5B665}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (23:30:20)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C940AF0-0452-485F-A5E4-33F373268A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{483FCE7C-6E43-49AA-9DBD-41F7C5F1425E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{F480BE97-D90C-4B1A-9DFB-10E26CFA4FE8}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{7FE835FB-5F1E-4664-93A9-CF1A5C74688F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
   <si>
     <t>17th ELO</t>
   </si>
@@ -104,13 +104,22 @@
     <t>3부리그</t>
   </si>
   <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
     <t>검정소</t>
   </si>
   <si>
     <t>AC 밀란</t>
   </si>
   <si>
-    <t>FA컵</t>
+    <t>UEFA_D조</t>
   </si>
   <si>
     <t>앙쿠</t>
@@ -119,7 +128,7 @@
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
-    <t>UEFA_D조</t>
+    <t>UEFA Tournament</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -128,15 +137,6 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
     <t>전체 합계</t>
   </si>
   <si>
@@ -155,48 +155,48 @@
     <t>1부리그</t>
   </si>
   <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
     <t>마인츠</t>
   </si>
   <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
+    <t>킹왕두</t>
+  </si>
+  <si>
+    <t>리버풀</t>
   </si>
   <si>
     <t>FA컵_결승전</t>
   </si>
   <si>
-    <t>킹왕두</t>
-  </si>
-  <si>
-    <t>리버풀</t>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
   </si>
   <si>
     <t>FA컵_4강</t>
   </si>
   <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
   </si>
   <si>
     <t>FA컵_8강</t>
   </si>
   <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
     <t>FA컵_16강</t>
   </si>
   <si>
@@ -245,28 +245,25 @@
     <t>UCL_8강</t>
   </si>
   <si>
+    <t>스페인전도사</t>
+  </si>
+  <si>
+    <t>UEL_FINAL</t>
+  </si>
+  <si>
     <t>suma수마</t>
   </si>
   <si>
     <t>ACF 피오렌티나</t>
   </si>
   <si>
-    <t>UEL_FINAL</t>
+    <t>UEL_4강</t>
   </si>
   <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
     <t>함부르크SV</t>
-  </si>
-  <si>
-    <t>UEL_4강</t>
-  </si>
-  <si>
-    <t>스페인전도사</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
   </si>
   <si>
     <t>UEL_8강</t>
@@ -691,7 +688,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFCBDFDF-7C45-4F6A-A7D2-9355A3A5B665}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3C3E3E7-0497-4DD3-84F5-FA45F52E25A7}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +720,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1220.0024999999998</v>
+        <v>1220.6224999999999</v>
       </c>
       <c r="B2">
-        <v>95.779999999999973</v>
+        <v>96.400000000000091</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -758,10 +755,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1186.7239999999999</v>
+        <v>1210.444</v>
       </c>
       <c r="B3">
-        <v>71.8599999999999</v>
+        <v>95.579999999999927</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,10 +767,10 @@
         <v>14</v>
       </c>
       <c r="E3">
+        <v>16</v>
+      </c>
+      <c r="F3">
         <v>14</v>
-      </c>
-      <c r="F3">
-        <v>12</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -802,10 +799,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1130.2275000000002</v>
+        <v>1112.6575</v>
       </c>
       <c r="B4">
-        <v>99.410000000000082</v>
+        <v>81.839999999999918</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -814,22 +811,22 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F4">
         <v>12</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" t="s">
         <v>20</v>
       </c>
       <c r="K4">
-        <v>22.979999999999997</v>
+        <v>23.26</v>
       </c>
       <c r="L4">
         <v>26</v>
@@ -846,10 +843,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1094.4775</v>
+        <v>1103.5290000000002</v>
       </c>
       <c r="B5">
-        <v>45.519999999999982</v>
+        <v>76.660000000000082</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -858,22 +855,22 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J5" t="s">
         <v>23</v>
       </c>
       <c r="K5">
-        <v>23.44</v>
+        <v>22.91</v>
       </c>
       <c r="L5">
         <v>2</v>
@@ -890,10 +887,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1075.325</v>
+        <v>1094.5074999999999</v>
       </c>
       <c r="B6">
-        <v>82.740000000000009</v>
+        <v>45.549999999999955</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -902,22 +899,22 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="F6">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J6" t="s">
         <v>26</v>
       </c>
       <c r="K6">
-        <v>31.770000000000003</v>
+        <v>35.979999999999997</v>
       </c>
       <c r="L6">
         <v>12</v>
@@ -934,10 +931,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1074.1525000000001</v>
+        <v>1075.575</v>
       </c>
       <c r="B7">
-        <v>34.539999999999964</v>
+        <v>82.990000000000009</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -946,16 +943,16 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J7" t="s">
         <v>29</v>
@@ -978,10 +975,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1064.1590000000001</v>
+        <v>1070.6625000000001</v>
       </c>
       <c r="B8">
-        <v>37.289999999999964</v>
+        <v>31.049999999999955</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,7 +987,7 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F8">
         <v>7</v>
@@ -999,13 +996,13 @@
         <v>1</v>
       </c>
       <c r="H8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
       </c>
       <c r="K8">
-        <v>78.19</v>
+        <v>82.15</v>
       </c>
       <c r="L8">
         <v>40</v>
@@ -1022,10 +1019,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1061.7349999999999</v>
+        <v>1061.9849999999999</v>
       </c>
       <c r="B9">
-        <v>17.569999999999936</v>
+        <v>17.819999999999936</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1048,10 +1045,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1057.23</v>
+        <v>1060.67</v>
       </c>
       <c r="B10">
-        <v>50.129999999999995</v>
+        <v>53.57000000000005</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1080,10 +1077,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1040.3790000000001</v>
+        <v>1033.3949999999998</v>
       </c>
       <c r="B11">
-        <v>-0.14000000000010004</v>
+        <v>-3.9100000000000819</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,13 +1089,13 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F11">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="G11">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H11">
         <v>7</v>
@@ -1112,28 +1109,28 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1033.0708636363636</v>
+        <v>1028.1290000000001</v>
       </c>
       <c r="B12">
-        <v>102.18999999999994</v>
+        <v>-12.3900000000001</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="E12">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="F12">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,31 +1141,31 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1029.0049999999999</v>
+        <v>1027.7774999999999</v>
       </c>
       <c r="B13">
-        <v>-8.2999999999999545</v>
+        <v>-26.440000000000055</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E13">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F13">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J13" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K13">
         <v>2.1</v>
@@ -1176,31 +1173,31 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1027.7774999999999</v>
+        <v>1018.8240000000001</v>
       </c>
       <c r="B14">
-        <v>-26.440000000000055</v>
+        <v>16.990000000000009</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14">
         <v>2</v>
       </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
       <c r="G14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K14">
         <v>1.9</v>
@@ -1208,31 +1205,31 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1018.484</v>
+        <v>1016.8308636363637</v>
       </c>
       <c r="B15">
-        <v>16.649999999999977</v>
+        <v>85.950000000000045</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E15">
+        <v>20</v>
+      </c>
+      <c r="F15">
+        <v>9</v>
+      </c>
+      <c r="G15">
         <v>4</v>
       </c>
-      <c r="F15">
-        <v>2</v>
-      </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
       <c r="H15">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K15">
         <v>1.7</v>
@@ -1240,28 +1237,28 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1001.3508636363637</v>
+        <v>1013.0308636363636</v>
       </c>
       <c r="B16">
-        <v>70.470000000000027</v>
+        <v>82.149999999999977</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E16">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F16">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H16">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1269,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1000.5408636363636</v>
+        <v>1001.2208636363637</v>
       </c>
       <c r="B17">
-        <v>69.659999999999968</v>
+        <v>70.340000000000032</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1304,10 +1301,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>965.97086363636367</v>
+        <v>966.26086363636364</v>
       </c>
       <c r="B18">
-        <v>35.090000000000032</v>
+        <v>35.379999999999995</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1336,10 +1333,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>961.11086363636366</v>
+        <v>961.36086363636366</v>
       </c>
       <c r="B19">
-        <v>30.230000000000018</v>
+        <v>30.480000000000018</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1368,10 +1365,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>946.61086363636366</v>
+        <v>951.05086363636372</v>
       </c>
       <c r="B20">
-        <v>15.730000000000018</v>
+        <v>20.170000000000073</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1400,10 +1397,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>943.30900000000008</v>
+        <v>947.40900000000011</v>
       </c>
       <c r="B21">
-        <v>-8.3999999999999773</v>
+        <v>-4.2999999999999545</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1432,31 +1429,31 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>920.42086363636361</v>
+        <v>930.88086363636364</v>
       </c>
       <c r="B22">
-        <v>-10.460000000000036</v>
+        <v>0</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="J22" t="s">
         <v>69</v>
-      </c>
-      <c r="E22">
-        <v>31</v>
-      </c>
-      <c r="F22">
-        <v>16</v>
-      </c>
-      <c r="G22">
-        <v>2</v>
-      </c>
-      <c r="H22">
-        <v>13</v>
-      </c>
-      <c r="J22" t="s">
-        <v>70</v>
       </c>
       <c r="K22">
         <v>1.6</v>
@@ -1464,31 +1461,31 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>906.48</v>
+        <v>921.70086363636369</v>
       </c>
       <c r="B23">
-        <v>-63.539999999999964</v>
+        <v>-9.17999999999995</v>
       </c>
       <c r="C23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" t="s">
         <v>71</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23">
+        <v>31</v>
+      </c>
+      <c r="F23">
+        <v>16</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23">
+        <v>13</v>
+      </c>
+      <c r="J23" t="s">
         <v>72</v>
-      </c>
-      <c r="E23">
-        <v>9</v>
-      </c>
-      <c r="F23">
-        <v>2</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23">
-        <v>7</v>
-      </c>
-      <c r="J23" t="s">
-        <v>73</v>
       </c>
       <c r="K23">
         <v>1.4</v>
@@ -1496,31 +1493,31 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>903.50086363636365</v>
+        <v>907.05</v>
       </c>
       <c r="B24">
-        <v>-27.379999999999995</v>
+        <v>-62.970000000000027</v>
       </c>
       <c r="C24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" t="s">
         <v>74</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24">
+        <v>9</v>
+      </c>
+      <c r="F24">
+        <v>2</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>7</v>
+      </c>
+      <c r="J24" t="s">
         <v>75</v>
-      </c>
-      <c r="E24">
-        <v>25</v>
-      </c>
-      <c r="F24">
-        <v>7</v>
-      </c>
-      <c r="G24">
-        <v>3</v>
-      </c>
-      <c r="H24">
-        <v>15</v>
-      </c>
-      <c r="J24" t="s">
-        <v>76</v>
       </c>
       <c r="K24">
         <v>1.2</v>
@@ -1528,16 +1525,16 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>888.03750000000002</v>
+        <v>888.44749999999999</v>
       </c>
       <c r="B25">
-        <v>-93.62</v>
+        <v>-93.210000000000036</v>
       </c>
       <c r="C25" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" t="s">
         <v>77</v>
-      </c>
-      <c r="D25" t="s">
-        <v>78</v>
       </c>
       <c r="E25">
         <v>17</v>
@@ -1552,7 +1549,7 @@
         <v>11</v>
       </c>
       <c r="J25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K25">
         <v>1.3</v>
@@ -1560,16 +1557,16 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>878.71400000000006</v>
+        <v>880.0440000000001</v>
       </c>
       <c r="B26">
-        <v>-55.509999999999991</v>
+        <v>-54.17999999999995</v>
       </c>
       <c r="C26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" t="s">
         <v>80</v>
-      </c>
-      <c r="D26" t="s">
-        <v>81</v>
       </c>
       <c r="E26">
         <v>39</v>
@@ -1584,7 +1581,7 @@
         <v>23</v>
       </c>
       <c r="J26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K26">
         <v>1.2</v>
@@ -1592,16 +1589,16 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>862.17086363636361</v>
+        <v>863.32086363636358</v>
       </c>
       <c r="B27">
-        <v>-68.710000000000036</v>
+        <v>-67.560000000000059</v>
       </c>
       <c r="C27" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" t="s">
         <v>83</v>
-      </c>
-      <c r="D27" t="s">
-        <v>84</v>
       </c>
       <c r="E27">
         <v>25</v>
@@ -1616,7 +1613,7 @@
         <v>17</v>
       </c>
       <c r="J27" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K27">
         <v>1.1000000000000001</v>
@@ -1624,16 +1621,16 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>859.4308636363636</v>
+        <v>859.84086363636368</v>
       </c>
       <c r="B28">
-        <v>-71.450000000000045</v>
+        <v>-71.039999999999964</v>
       </c>
       <c r="C28" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" t="s">
         <v>86</v>
-      </c>
-      <c r="D28" t="s">
-        <v>87</v>
       </c>
       <c r="E28">
         <v>19</v>
@@ -1650,16 +1647,16 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>824.90086363636362</v>
+        <v>826.9308636363636</v>
       </c>
       <c r="B29">
-        <v>-105.98000000000002</v>
+        <v>-103.95000000000005</v>
       </c>
       <c r="C29" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" t="s">
         <v>88</v>
-      </c>
-      <c r="D29" t="s">
-        <v>89</v>
       </c>
       <c r="E29">
         <v>21</v>

</xml_diff>

<commit_message>
Update: Ranking Data (03:09:35)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{483FCE7C-6E43-49AA-9DBD-41F7C5F1425E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14BB8696-8BBB-473D-B33C-0B09204EDFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{7FE835FB-5F1E-4664-93A9-CF1A5C74688F}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{0C6CA90E-E0A1-4201-8759-25C46AFC2CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="90">
   <si>
     <t>17th ELO</t>
   </si>
@@ -131,28 +131,43 @@
     <t>UEFA Tournament</t>
   </si>
   <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>킹왕두</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
     <t>Special블루</t>
   </si>
   <si>
     <t>아스널</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>1부리그</t>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
   </si>
   <si>
     <t>아들러</t>
@@ -161,7 +176,7 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>2부리그</t>
+    <t>FA컵_결승전</t>
   </si>
   <si>
     <t>오스트리아</t>
@@ -170,13 +185,19 @@
     <t>마인츠</t>
   </si>
   <si>
-    <t>킹왕두</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>FA컵_8강</t>
+  </si>
+  <si>
+    <t>FA컵_16강</t>
   </si>
   <si>
     <t>호야국2인</t>
@@ -185,37 +206,25 @@
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
-  </si>
-  <si>
-    <t>FA컵_16강</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
     <t>FA컵_32강</t>
   </si>
   <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
+    <t>UEFA</t>
+  </si>
+  <si>
     <t>셀래스틴</t>
   </si>
   <si>
     <t>바르셀로나</t>
   </si>
   <si>
-    <t>UEFA</t>
+    <t>UCL_결승전</t>
   </si>
   <si>
     <t>용신</t>
@@ -224,7 +233,7 @@
     <t>토트넘</t>
   </si>
   <si>
-    <t>UCL_결승전</t>
+    <t>UCL_4강</t>
   </si>
   <si>
     <t>여수가스</t>
@@ -233,55 +242,49 @@
     <t>AS 모나코</t>
   </si>
   <si>
-    <t>UCL_4강</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
-  </si>
-  <si>
     <t>UCL_8강</t>
   </si>
   <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>UEL_FINAL</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>UEL_4강</t>
+  </si>
+  <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>UEL_8강</t>
+  </si>
+  <si>
     <t>스페인전도사</t>
   </si>
   <si>
-    <t>UEL_FINAL</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>UEL_4강</t>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
   </si>
   <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
     <t>함부르크SV</t>
-  </si>
-  <si>
-    <t>UEL_8강</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
   </si>
   <si>
     <t>UECL_4강</t>
@@ -688,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3C3E3E7-0497-4DD3-84F5-FA45F52E25A7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C6F3A95-16A1-478C-939E-0BF0F0911E62}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -720,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1220.6224999999999</v>
+        <v>1218.0524999999998</v>
       </c>
       <c r="B2">
-        <v>96.400000000000091</v>
+        <v>93.829999999999927</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -732,16 +735,16 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F2">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G2">
         <v>3</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -755,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1210.444</v>
+        <v>1205.454</v>
       </c>
       <c r="B3">
-        <v>95.579999999999927</v>
+        <v>90.589999999999918</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -767,16 +770,16 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F3">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
@@ -799,10 +802,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1112.6575</v>
+        <v>1112.4875000000002</v>
       </c>
       <c r="B4">
-        <v>81.839999999999918</v>
+        <v>81.670000000000073</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -826,7 +829,7 @@
         <v>20</v>
       </c>
       <c r="K4">
-        <v>23.26</v>
+        <v>22.979999999999997</v>
       </c>
       <c r="L4">
         <v>26</v>
@@ -843,10 +846,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1103.5290000000002</v>
+        <v>1103.1590000000001</v>
       </c>
       <c r="B5">
-        <v>76.660000000000082</v>
+        <v>76.289999999999964</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -870,7 +873,7 @@
         <v>23</v>
       </c>
       <c r="K5">
-        <v>22.91</v>
+        <v>23.44</v>
       </c>
       <c r="L5">
         <v>2</v>
@@ -887,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1094.5074999999999</v>
+        <v>1094.4775</v>
       </c>
       <c r="B6">
-        <v>45.549999999999955</v>
+        <v>45.519999999999982</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -914,7 +917,7 @@
         <v>26</v>
       </c>
       <c r="K6">
-        <v>35.979999999999997</v>
+        <v>31.770000000000003</v>
       </c>
       <c r="L6">
         <v>12</v>
@@ -931,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1075.575</v>
+        <v>1084.8050000000001</v>
       </c>
       <c r="B7">
-        <v>82.990000000000009</v>
+        <v>92.220000000000027</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -943,10 +946,10 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F7">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G7">
         <v>9</v>
@@ -975,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1070.6625000000001</v>
+        <v>1061.7349999999999</v>
       </c>
       <c r="B8">
-        <v>31.049999999999955</v>
+        <v>17.569999999999936</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -987,13 +990,13 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F8">
         <v>7</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H8">
         <v>5</v>
@@ -1002,7 +1005,7 @@
         <v>32</v>
       </c>
       <c r="K8">
-        <v>82.15</v>
+        <v>78.19</v>
       </c>
       <c r="L8">
         <v>40</v>
@@ -1019,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1061.9849999999999</v>
+        <v>1057.23</v>
       </c>
       <c r="B9">
-        <v>17.819999999999936</v>
+        <v>50.129999999999995</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1031,24 +1034,24 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F9">
+        <v>8</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
         <v>7</v>
-      </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
-        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1060.67</v>
+        <v>1052.3274999999999</v>
       </c>
       <c r="B10">
-        <v>53.57000000000005</v>
+        <v>-1.8900000000001</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1057,16 +1060,16 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="F10">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J10" t="s">
         <v>37</v>
@@ -1077,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1033.3949999999998</v>
+        <v>1047.6225000000002</v>
       </c>
       <c r="B11">
-        <v>-3.9100000000000819</v>
+        <v>8.0099999999999909</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1089,7 +1092,7 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F11">
         <v>7</v>
@@ -1098,7 +1101,7 @@
         <v>1</v>
       </c>
       <c r="H11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1109,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1028.1290000000001</v>
+        <v>1034.7308636363637</v>
       </c>
       <c r="B12">
-        <v>-12.3900000000001</v>
+        <v>103.85000000000002</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1121,16 +1124,16 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F12">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="G12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1141,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1027.7774999999999</v>
+        <v>1029.8949999999998</v>
       </c>
       <c r="B13">
-        <v>-26.440000000000055</v>
+        <v>-7.4100000000000819</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1153,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1173,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1018.8240000000001</v>
+        <v>1026.7790000000002</v>
       </c>
       <c r="B14">
-        <v>16.990000000000009</v>
+        <v>-13.740000000000009</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1185,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1205,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1016.8308636363637</v>
+        <v>1016.2508636363636</v>
       </c>
       <c r="B15">
-        <v>85.950000000000045</v>
+        <v>85.37</v>
       </c>
       <c r="C15" t="s">
         <v>49</v>
@@ -1237,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1013.0308636363636</v>
+        <v>1009.0708636363636</v>
       </c>
       <c r="B16">
-        <v>82.149999999999977</v>
+        <v>78.189999999999941</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
@@ -1269,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1001.2208636363637</v>
+        <v>978.5440000000001</v>
       </c>
       <c r="B17">
-        <v>70.340000000000032</v>
+        <v>-23.289999999999964</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1281,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="F17">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1301,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>966.26086363636364</v>
+        <v>973.04900000000009</v>
       </c>
       <c r="B18">
-        <v>35.379999999999995</v>
+        <v>21.340000000000032</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1313,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F18">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1333,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>961.36086363636366</v>
+        <v>965.97086363636367</v>
       </c>
       <c r="B19">
-        <v>30.480000000000018</v>
+        <v>35.090000000000032</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1345,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G19">
         <v>4</v>
       </c>
       <c r="H19">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
@@ -1365,10 +1368,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>951.05086363636372</v>
+        <v>961.11086363636366</v>
       </c>
       <c r="B20">
-        <v>20.170000000000073</v>
+        <v>30.230000000000018</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1377,13 +1380,13 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F20">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H20">
         <v>10</v>
@@ -1397,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>947.40900000000011</v>
+        <v>934.84086363636368</v>
       </c>
       <c r="B21">
-        <v>-4.2999999999999545</v>
+        <v>3.9600000000000364</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1409,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F21">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1429,31 +1432,31 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>930.88086363636364</v>
+        <v>929.73750000000007</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>-51.919999999999959</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
       </c>
-      <c r="D22" t="e">
-        <v>#N/A</v>
+      <c r="D22" t="s">
+        <v>69</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J22" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="K22">
         <v>1.6</v>
@@ -1461,16 +1464,16 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>921.70086363636369</v>
+        <v>920.42086363636361</v>
       </c>
       <c r="B23">
-        <v>-9.17999999999995</v>
+        <v>-10.460000000000036</v>
       </c>
       <c r="C23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E23">
         <v>31</v>
@@ -1485,7 +1488,7 @@
         <v>13</v>
       </c>
       <c r="J23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K23">
         <v>1.4</v>
@@ -1493,31 +1496,31 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>907.05</v>
+        <v>914.75400000000002</v>
       </c>
       <c r="B24">
-        <v>-62.970000000000027</v>
+        <v>-19.470000000000027</v>
       </c>
       <c r="C24" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D24" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E24">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H24">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="J24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="K24">
         <v>1.2</v>
@@ -1525,31 +1528,31 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>888.44749999999999</v>
+        <v>903.50086363636365</v>
       </c>
       <c r="B25">
-        <v>-93.210000000000036</v>
+        <v>-27.379999999999995</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D25" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E25">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G25">
         <v>3</v>
       </c>
       <c r="H25">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K25">
         <v>1.3</v>
@@ -1557,31 +1560,31 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>880.0440000000001</v>
+        <v>886.95</v>
       </c>
       <c r="B26">
-        <v>-54.17999999999995</v>
+        <v>-83.069999999999936</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D26" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E26">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="F26">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G26">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="J26" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K26">
         <v>1.2</v>
@@ -1589,16 +1592,16 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>863.32086363636358</v>
+        <v>862.17086363636361</v>
       </c>
       <c r="B27">
-        <v>-67.560000000000059</v>
+        <v>-68.710000000000036</v>
       </c>
       <c r="C27" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D27" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E27">
         <v>25</v>
@@ -1613,7 +1616,7 @@
         <v>17</v>
       </c>
       <c r="J27" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K27">
         <v>1.1000000000000001</v>
@@ -1621,16 +1624,16 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>859.84086363636368</v>
+        <v>859.4308636363636</v>
       </c>
       <c r="B28">
-        <v>-71.039999999999964</v>
+        <v>-71.450000000000045</v>
       </c>
       <c r="C28" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D28" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E28">
         <v>19</v>
@@ -1647,19 +1650,19 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>826.9308636363636</v>
+        <v>802.14086363636363</v>
       </c>
       <c r="B29">
-        <v>-103.95000000000005</v>
+        <v>-128.74</v>
       </c>
       <c r="C29" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D29" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E29">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F29">
         <v>3</v>
@@ -1668,7 +1671,7 @@
         <v>0</v>
       </c>
       <c r="H29">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (06:28:25)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14BB8696-8BBB-473D-B33C-0B09204EDFDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1523ED58-F7AA-4B1F-A687-81C04D31922B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{0C6CA90E-E0A1-4201-8759-25C46AFC2CD8}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{2FCB906A-27CE-4E1D-BE17-4D58B8B0E9D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -131,22 +131,22 @@
     <t>UEFA Tournament</t>
   </si>
   <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>은안</t>
   </si>
   <si>
     <t>맨체스터 시티</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>킹왕두</t>
+    <t>피파왕초보구단주</t>
   </si>
   <si>
     <t>리버풀</t>
@@ -209,13 +209,22 @@
     <t>FA컵_32강</t>
   </si>
   <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>UEFA</t>
+  </si>
+  <si>
     <t>경남FC가즈아</t>
   </si>
   <si>
     <t>경남 FC</t>
   </si>
   <si>
-    <t>UEFA</t>
+    <t>UCL_결승전</t>
   </si>
   <si>
     <t>셀래스틴</t>
@@ -224,15 +233,6 @@
     <t>바르셀로나</t>
   </si>
   <si>
-    <t>UCL_결승전</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
     <t>UCL_4강</t>
   </si>
   <si>
@@ -245,34 +245,34 @@
     <t>UCL_8강</t>
   </si>
   <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>UEL_FINAL</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>UEL_4강</t>
+  </si>
+  <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
   </si>
   <si>
-    <t>UEL_FINAL</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>UEL_4강</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
-  </si>
-  <si>
     <t>UEL_8강</t>
   </si>
   <si>
-    <t>스페인전도사</t>
+    <t>syma</t>
   </si>
   <si>
     <t>RC 셀타 비고</t>
@@ -290,19 +290,19 @@
     <t>UECL_4강</t>
   </si>
   <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
+  </si>
+  <si>
+    <t>UECL_8강</t>
+  </si>
+  <si>
     <t>A지냐크</t>
   </si>
   <si>
     <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>UECL_8강</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
   </si>
   <si>
     <t>겐지간지</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C6F3A95-16A1-478C-939E-0BF0F0911E62}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE85919B-8E68-49AD-BCE8-5E72199E91E4}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -846,10 +846,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1103.1590000000001</v>
+        <v>1111.0490000000002</v>
       </c>
       <c r="B5">
-        <v>76.289999999999964</v>
+        <v>84.180000000000064</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -858,16 +858,16 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J5" t="s">
         <v>23</v>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1094.4775</v>
+        <v>1107.9375</v>
       </c>
       <c r="B6">
-        <v>45.519999999999982</v>
+        <v>58.980000000000018</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -902,10 +902,10 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G6">
         <v>2</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1061.7349999999999</v>
+        <v>1082.6200000000001</v>
       </c>
       <c r="B8">
-        <v>17.569999999999936</v>
+        <v>75.520000000000095</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,16 +990,16 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1057.23</v>
+        <v>1061.7349999999999</v>
       </c>
       <c r="B9">
-        <v>50.129999999999995</v>
+        <v>17.569999999999936</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1034,16 +1034,16 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1047.6225000000002</v>
+        <v>1049.7225000000001</v>
       </c>
       <c r="B11">
-        <v>8.0099999999999909</v>
+        <v>10.1099999999999</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,16 +1092,16 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1034.7308636363637</v>
+        <v>1041.2008636363637</v>
       </c>
       <c r="B12">
-        <v>103.85000000000002</v>
+        <v>110.32000000000005</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,10 +1124,10 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F12">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G12">
         <v>4</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>973.04900000000009</v>
+        <v>970.77086363636363</v>
       </c>
       <c r="B18">
-        <v>21.340000000000032</v>
+        <v>39.889999999999986</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F18">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>965.97086363636367</v>
+        <v>970.05900000000008</v>
       </c>
       <c r="B19">
-        <v>35.090000000000032</v>
+        <v>18.350000000000023</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E19">
+        <v>34</v>
+      </c>
+      <c r="F19">
         <v>16</v>
       </c>
-      <c r="F19">
-        <v>6</v>
-      </c>
       <c r="G19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H19">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
@@ -1368,10 +1368,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>961.11086363636366</v>
+        <v>965.97086363636367</v>
       </c>
       <c r="B20">
-        <v>30.230000000000018</v>
+        <v>35.090000000000032</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,16 +1380,16 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G20">
         <v>4</v>
       </c>
       <c r="H20">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>929.73750000000007</v>
+        <v>914.75400000000002</v>
       </c>
       <c r="B22">
-        <v>-51.919999999999959</v>
+        <v>-19.470000000000027</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,16 +1444,16 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="F22">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H22">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J22" t="s">
         <v>70</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>920.42086363636361</v>
+        <v>914.03086363636362</v>
       </c>
       <c r="B23">
-        <v>-10.460000000000036</v>
+        <v>-16.850000000000023</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,7 +1476,7 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F23">
         <v>16</v>
@@ -1485,7 +1485,7 @@
         <v>2</v>
       </c>
       <c r="H23">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>914.75400000000002</v>
+        <v>910.74750000000006</v>
       </c>
       <c r="B24">
-        <v>-19.470000000000027</v>
+        <v>-70.909999999999968</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1508,16 +1508,16 @@
         <v>75</v>
       </c>
       <c r="E24">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="F24">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G24">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H24">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="J24" t="s">
         <v>76</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>886.95</v>
+        <v>888.81999999999994</v>
       </c>
       <c r="B26">
-        <v>-83.069999999999936</v>
+        <v>-81.200000000000045</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
+        <v>15</v>
+      </c>
+      <c r="F26">
+        <v>3</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
         <v>11</v>
-      </c>
-      <c r="F26">
-        <v>2</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <v>9</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1592,10 +1592,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>862.17086363636361</v>
+        <v>859.4308636363636</v>
       </c>
       <c r="B27">
-        <v>-68.710000000000036</v>
+        <v>-71.450000000000045</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,13 +1604,13 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H27">
         <v>17</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>859.4308636363636</v>
+        <v>858.45086363636358</v>
       </c>
       <c r="B28">
-        <v>-71.450000000000045</v>
+        <v>-72.430000000000064</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,16 +1636,16 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H28">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (03:09:19)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1523ED58-F7AA-4B1F-A687-81C04D31922B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6EAA0B1-4F9E-440A-8804-A8CF9BF2E7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{2FCB906A-27CE-4E1D-BE17-4D58B8B0E9D5}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{DD2A30FF-3FBD-4216-9764-A2DBD66585A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -122,21 +122,21 @@
     <t>UEFA_D조</t>
   </si>
   <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
     <t>앙쿠</t>
   </si>
   <si>
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
     <t>전체 합계</t>
   </si>
   <si>
@@ -200,13 +200,22 @@
     <t>FA컵_16강</t>
   </si>
   <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>FA컵_32강</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>FA컵_32강</t>
+    <t>UEFA</t>
   </si>
   <si>
     <t>용신</t>
@@ -215,7 +224,7 @@
     <t>토트넘</t>
   </si>
   <si>
-    <t>UEFA</t>
+    <t>UCL_결승전</t>
   </si>
   <si>
     <t>경남FC가즈아</t>
@@ -224,15 +233,6 @@
     <t>경남 FC</t>
   </si>
   <si>
-    <t>UCL_결승전</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
     <t>UCL_4강</t>
   </si>
   <si>
@@ -263,21 +263,21 @@
     <t>UEL_4강</t>
   </si>
   <si>
+    <t>syma</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
+    <t>UEL_8강</t>
+  </si>
+  <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
   </si>
   <si>
-    <t>UEL_8강</t>
-  </si>
-  <si>
-    <t>syma</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
-  </si>
-  <si>
     <t>UECL_FINAL</t>
   </si>
   <si>
@@ -290,19 +290,19 @@
     <t>UECL_4강</t>
   </si>
   <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>UECL_8강</t>
+  </si>
+  <si>
     <t>ShangHaiPortFC</t>
   </si>
   <si>
     <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>UECL_8강</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
   </si>
   <si>
     <t>겐지간지</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE85919B-8E68-49AD-BCE8-5E72199E91E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A71B8933-2017-45BE-9DA6-FF0888849FA9}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1205.454</v>
+        <v>1215.144</v>
       </c>
       <c r="B3">
-        <v>90.589999999999918</v>
+        <v>100.27999999999997</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,10 +770,10 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F3">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3">
         <v>2</v>
@@ -802,10 +802,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1112.4875000000002</v>
+        <v>1122.4575</v>
       </c>
       <c r="B4">
-        <v>81.670000000000073</v>
+        <v>91.639999999999873</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -814,16 +814,16 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G4">
         <v>5</v>
       </c>
       <c r="H4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J4" t="s">
         <v>20</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1084.8050000000001</v>
+        <v>1106.18</v>
       </c>
       <c r="B7">
-        <v>92.220000000000027</v>
+        <v>99.080000000000041</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -946,16 +946,16 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
         <v>9</v>
-      </c>
-      <c r="H7">
-        <v>4</v>
       </c>
       <c r="J7" t="s">
         <v>29</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1082.6200000000001</v>
+        <v>1084.8050000000001</v>
       </c>
       <c r="B8">
-        <v>75.520000000000095</v>
+        <v>92.220000000000027</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,16 +990,16 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="F8">
+        <v>23</v>
+      </c>
+      <c r="G8">
         <v>9</v>
       </c>
-      <c r="G8">
-        <v>2</v>
-      </c>
       <c r="H8">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1029.8949999999998</v>
+        <v>1023.0949999999998</v>
       </c>
       <c r="B13">
-        <v>-7.4100000000000819</v>
+        <v>-14.210000000000036</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1026.7790000000002</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B14">
-        <v>-13.740000000000009</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="F14">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H14">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>978.5440000000001</v>
+        <v>989.3008636363636</v>
       </c>
       <c r="B17">
-        <v>-23.289999999999964</v>
+        <v>58.419999999999959</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>970.77086363636363</v>
+        <v>978.5440000000001</v>
       </c>
       <c r="B18">
-        <v>39.889999999999986</v>
+        <v>-23.289999999999964</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="F18">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>970.05900000000008</v>
+        <v>970.77086363636363</v>
       </c>
       <c r="B19">
-        <v>18.350000000000023</v>
+        <v>39.889999999999986</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,30 +1348,30 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="F19">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H19">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
       </c>
       <c r="K19">
-        <v>2.2000000000000002</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>965.97086363636367</v>
+        <v>970.05900000000008</v>
       </c>
       <c r="B20">
-        <v>35.090000000000032</v>
+        <v>18.350000000000023</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,30 +1380,30 @@
         <v>63</v>
       </c>
       <c r="E20">
+        <v>34</v>
+      </c>
+      <c r="F20">
         <v>16</v>
       </c>
-      <c r="F20">
-        <v>6</v>
-      </c>
       <c r="G20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H20">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
       </c>
       <c r="K20">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>934.84086363636368</v>
+        <v>934.26086363636364</v>
       </c>
       <c r="B21">
-        <v>3.9600000000000364</v>
+        <v>3.3799999999999955</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,22 +1412,22 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F21">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G21">
         <v>2</v>
       </c>
       <c r="H21">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
       </c>
       <c r="K21">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
@@ -1459,7 +1459,7 @@
         <v>70</v>
       </c>
       <c r="K22">
-        <v>1.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
@@ -1491,15 +1491,15 @@
         <v>73</v>
       </c>
       <c r="K23">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>910.74750000000006</v>
+        <v>903.50086363636365</v>
       </c>
       <c r="B24">
-        <v>-70.909999999999968</v>
+        <v>-27.379999999999995</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1508,30 +1508,30 @@
         <v>75</v>
       </c>
       <c r="E24">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F24">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H24">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J24" t="s">
         <v>76</v>
       </c>
       <c r="K24">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>903.50086363636365</v>
+        <v>901.28750000000002</v>
       </c>
       <c r="B25">
-        <v>-27.379999999999995</v>
+        <v>-80.37</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,22 +1540,22 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F25">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H25">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
       </c>
       <c r="K25">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
@@ -1587,15 +1587,15 @@
         <v>82</v>
       </c>
       <c r="K26">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>859.4308636363636</v>
+        <v>858.45086363636358</v>
       </c>
       <c r="B27">
-        <v>-71.450000000000045</v>
+        <v>-72.430000000000064</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,16 +1604,16 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H27">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="J27" t="s">
         <v>85</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>858.45086363636358</v>
+        <v>853.88086363636364</v>
       </c>
       <c r="B28">
-        <v>-72.430000000000064</v>
+        <v>-77</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,16 +1636,16 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (20:16:41)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6EAA0B1-4F9E-440A-8804-A8CF9BF2E7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15B3C1D8-F0DD-4557-81C2-42EFF34D09B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{DD2A30FF-3FBD-4216-9764-A2DBD66585A9}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{DE7113BA-29C5-410F-9773-32522CF172AE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -104,28 +104,28 @@
     <t>3부리그</t>
   </si>
   <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>UEFA_D조</t>
+  </si>
+  <si>
     <t>방덕</t>
   </si>
   <si>
     <t>인테르</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>UEFA_D조</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
   </si>
   <si>
     <t>UEFA Tournament</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A71B8933-2017-45BE-9DA6-FF0888849FA9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9636E6C-BDF1-4D68-9E68-9D36536E831E}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1218.0524999999998</v>
+        <v>1260.2724999999998</v>
       </c>
       <c r="B2">
-        <v>93.829999999999927</v>
+        <v>136.04999999999995</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -735,10 +735,10 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -846,10 +846,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1111.0490000000002</v>
+        <v>1107.9375</v>
       </c>
       <c r="B5">
-        <v>84.180000000000064</v>
+        <v>58.980000000000018</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -858,16 +858,16 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F5">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
       <c r="H5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="J5" t="s">
         <v>23</v>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1107.9375</v>
+        <v>1106.18</v>
       </c>
       <c r="B6">
-        <v>58.980000000000018</v>
+        <v>99.080000000000041</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -902,16 +902,16 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="F6">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G6">
         <v>2</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="J6" t="s">
         <v>26</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1106.18</v>
+        <v>1091.6190000000001</v>
       </c>
       <c r="B7">
-        <v>99.080000000000041</v>
+        <v>64.75</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -949,13 +949,13 @@
         <v>21</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J7" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Update: Ranking Data (20:37:29)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15B3C1D8-F0DD-4557-81C2-42EFF34D09B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC58BC97-CE41-4219-BE17-A51F9FC73401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{DE7113BA-29C5-410F-9773-32522CF172AE}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{5BFA49CE-DB28-45B9-87EE-D8B7D696A4D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -170,34 +170,43 @@
     <t>레알 마드리드</t>
   </si>
   <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
+    <t>FA컵_8강</t>
+  </si>
+  <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>FA컵_16강</t>
+  </si>
+  <si>
     <t>아들러</t>
   </si>
   <si>
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
-  </si>
-  <si>
-    <t>FA컵_16강</t>
+    <t>FA컵_32강</t>
   </si>
   <si>
     <t>셀래스틴</t>
@@ -206,15 +215,6 @@
     <t>바르셀로나</t>
   </si>
   <si>
-    <t>FA컵_32강</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>UEFA</t>
   </si>
   <si>
@@ -254,37 +254,37 @@
     <t>UEL_FINAL</t>
   </si>
   <si>
+    <t>syma</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
+    <t>UEL_4강</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>UEL_8강</t>
+  </si>
+  <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
     <t>suma수마</t>
   </si>
   <si>
     <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>UEL_4강</t>
-  </si>
-  <si>
-    <t>syma</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
-  </si>
-  <si>
-    <t>UEL_8강</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
   </si>
   <si>
     <t>UECL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9636E6C-BDF1-4D68-9E68-9D36536E831E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472739D0-4D44-4D86-82C6-24F8FDBAF958}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1023.0949999999998</v>
+        <v>1035.8240000000001</v>
       </c>
       <c r="B13">
-        <v>-14.210000000000036</v>
+        <v>33.990000000000009</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F13">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G13">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1208,31 +1208,31 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1016.2508636363636</v>
+        <v>1009.0708636363636</v>
       </c>
       <c r="B15">
-        <v>85.37</v>
+        <v>78.189999999999941</v>
       </c>
       <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15">
+        <v>40</v>
+      </c>
+      <c r="F15">
+        <v>22</v>
+      </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
+      <c r="H15">
+        <v>13</v>
+      </c>
+      <c r="J15" t="s">
         <v>49</v>
-      </c>
-      <c r="D15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15">
-        <v>20</v>
-      </c>
-      <c r="F15">
-        <v>9</v>
-      </c>
-      <c r="G15">
-        <v>4</v>
-      </c>
-      <c r="H15">
-        <v>7</v>
-      </c>
-      <c r="J15" t="s">
-        <v>51</v>
       </c>
       <c r="K15">
         <v>1.7</v>
@@ -1240,28 +1240,28 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1009.0708636363636</v>
+        <v>1003.3908636363636</v>
       </c>
       <c r="B16">
-        <v>78.189999999999941</v>
+        <v>72.509999999999991</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E16">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="F16">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H16">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>989.3008636363636</v>
+        <v>992.30499999999984</v>
       </c>
       <c r="B17">
-        <v>58.419999999999959</v>
+        <v>-45</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F17">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>978.5440000000001</v>
+        <v>990.23086363636367</v>
       </c>
       <c r="B18">
-        <v>-23.289999999999964</v>
+        <v>59.350000000000023</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H18">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>914.03086363636362</v>
+        <v>903.50086363636365</v>
       </c>
       <c r="B23">
-        <v>-16.850000000000023</v>
+        <v>-27.379999999999995</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,13 +1476,13 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F23">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H23">
         <v>15</v>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>903.50086363636365</v>
+        <v>901.28750000000002</v>
       </c>
       <c r="B24">
-        <v>-27.379999999999995</v>
+        <v>-80.37</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1508,16 +1508,16 @@
         <v>75</v>
       </c>
       <c r="E24">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F24">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H24">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J24" t="s">
         <v>76</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>901.28750000000002</v>
+        <v>900.31999999999994</v>
       </c>
       <c r="B25">
-        <v>-80.37</v>
+        <v>-69.700000000000045</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,16 +1540,16 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G25">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H25">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>888.81999999999994</v>
+        <v>897.24086363636366</v>
       </c>
       <c r="B26">
-        <v>-81.200000000000045</v>
+        <v>-33.639999999999986</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1650,10 +1650,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>802.14086363636363</v>
+        <v>795.11086363636366</v>
       </c>
       <c r="B29">
-        <v>-128.74</v>
+        <v>-135.76999999999998</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1662,7 +1662,7 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F29">
         <v>3</v>
@@ -1671,7 +1671,7 @@
         <v>0</v>
       </c>
       <c r="H29">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (08:09:53)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC58BC97-CE41-4219-BE17-A51F9FC73401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{16C4B723-466C-4357-8264-E9E8E971ADDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{5BFA49CE-DB28-45B9-87EE-D8B7D696A4D4}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{AD428602-56BA-4367-BDB2-1B2B81107E91}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -140,28 +140,43 @@
     <t>전체 합계</t>
   </si>
   <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>피파왕초보구단주</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
     <t>은안</t>
   </si>
   <si>
     <t>맨체스터 시티</t>
   </si>
   <si>
-    <t>피파왕초보구단주</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>2부리그</t>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>FA컵_결승전</t>
   </si>
   <si>
     <t>0708ManUtd</t>
@@ -170,21 +185,6 @@
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
     <t>FA컵_4강</t>
   </si>
   <si>
@@ -254,28 +254,28 @@
     <t>UEL_FINAL</t>
   </si>
   <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>UEL_4강</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>UEL_8강</t>
+  </si>
+  <si>
     <t>syma</t>
   </si>
   <si>
     <t>RC 셀타 비고</t>
-  </si>
-  <si>
-    <t>UEL_4강</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>UEL_8강</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
   </si>
   <si>
     <t>UECL_FINAL</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472739D0-4D44-4D86-82C6-24F8FDBAF958}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E884C4E-0182-4454-94C4-BDB0B590ED5D}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1084.8050000000001</v>
+        <v>1089.7550000000001</v>
       </c>
       <c r="B8">
-        <v>92.220000000000027</v>
+        <v>97.170000000000073</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,10 +990,10 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F8">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G8">
         <v>9</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1061.7349999999999</v>
+        <v>1062.9525000000001</v>
       </c>
       <c r="B9">
-        <v>17.569999999999936</v>
+        <v>23.339999999999918</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1034,24 +1034,24 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F9">
+        <v>11</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
         <v>7</v>
-      </c>
-      <c r="G9">
-        <v>3</v>
-      </c>
-      <c r="H9">
-        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1052.3274999999999</v>
+        <v>1058.3174999999999</v>
       </c>
       <c r="B10">
-        <v>-1.8900000000001</v>
+        <v>4.0999999999999091</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1060,13 +1060,13 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H10">
         <v>5</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1049.7225000000001</v>
+        <v>1054.104</v>
       </c>
       <c r="B11">
-        <v>10.1099999999999</v>
+        <v>52.269999999999982</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,16 +1092,16 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1041.2008636363637</v>
+        <v>1047.2049999999999</v>
       </c>
       <c r="B12">
-        <v>110.32000000000005</v>
+        <v>3.0399999999999636</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,16 +1124,16 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F12">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1035.8240000000001</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B13">
-        <v>33.990000000000009</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
+        <v>39</v>
+      </c>
+      <c r="F13">
+        <v>22</v>
+      </c>
+      <c r="G13">
+        <v>7</v>
+      </c>
+      <c r="H13">
         <v>10</v>
-      </c>
-      <c r="F13">
-        <v>6</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-      <c r="H13">
-        <v>3</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1017.1890000000002</v>
+        <v>1010.4208636363636</v>
       </c>
       <c r="B14">
-        <v>-23.330000000000041</v>
+        <v>79.539999999999964</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F14">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G14">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1003.3908636363636</v>
+        <v>1004.8008636363636</v>
       </c>
       <c r="B16">
-        <v>72.509999999999991</v>
+        <v>73.919999999999959</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F16">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G16">
         <v>4</v>
       </c>
       <c r="H16">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1363,7 +1363,7 @@
         <v>61</v>
       </c>
       <c r="K19">
-        <v>2.4</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
@@ -1395,7 +1395,7 @@
         <v>64</v>
       </c>
       <c r="K20">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
@@ -1427,7 +1427,7 @@
         <v>67</v>
       </c>
       <c r="K21">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
@@ -1459,15 +1459,15 @@
         <v>70</v>
       </c>
       <c r="K22">
-        <v>2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>903.50086363636365</v>
+        <v>910.11</v>
       </c>
       <c r="B23">
-        <v>-27.379999999999995</v>
+        <v>-59.909999999999968</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,22 +1476,22 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F23">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
       </c>
       <c r="K23">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>900.31999999999994</v>
+        <v>898.61086363636366</v>
       </c>
       <c r="B25">
-        <v>-69.700000000000045</v>
+        <v>-32.269999999999982</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,30 +1540,30 @@
         <v>78</v>
       </c>
       <c r="E25">
+        <v>27</v>
+      </c>
+      <c r="F25">
+        <v>7</v>
+      </c>
+      <c r="G25">
+        <v>3</v>
+      </c>
+      <c r="H25">
         <v>17</v>
-      </c>
-      <c r="F25">
-        <v>4</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-      <c r="H25">
-        <v>12</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
       </c>
       <c r="K25">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>897.24086363636366</v>
+        <v>895.70086363636369</v>
       </c>
       <c r="B26">
-        <v>-33.639999999999986</v>
+        <v>-35.17999999999995</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,22 +1572,22 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F26">
         <v>18</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
       </c>
       <c r="K26">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (08:25:30)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{16C4B723-466C-4357-8264-E9E8E971ADDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{18B411BB-E86C-466D-9D3D-EEE5F89D8B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{AD428602-56BA-4367-BDB2-1B2B81107E91}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{DCF5980D-72DA-4D98-9AE4-7C474482B333}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -140,34 +140,43 @@
     <t>전체 합계</t>
   </si>
   <si>
+    <t>피파왕초보구단주</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
     <t>Special블루</t>
   </si>
   <si>
     <t>아스널</t>
   </si>
   <si>
-    <t>피파왕초보구단주</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
+    <t>FA컵_결승전</t>
   </si>
   <si>
     <t>오스트리아</t>
@@ -176,7 +185,7 @@
     <t>마인츠</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>0708ManUtd</t>
@@ -185,25 +194,16 @@
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
     <t>FA컵_8강</t>
   </si>
   <si>
+    <t>FA컵_16강</t>
+  </si>
+  <si>
     <t>비주류중독</t>
   </si>
   <si>
     <t>셀틱 FC</t>
-  </si>
-  <si>
-    <t>FA컵_16강</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
   </si>
   <si>
     <t>FA컵_32강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E884C4E-0182-4454-94C4-BDB0B590ED5D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B35F2FE-A0B0-4023-84A4-B10463F11579}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1062.9525000000001</v>
+        <v>1058.3174999999999</v>
       </c>
       <c r="B9">
-        <v>23.339999999999918</v>
+        <v>4.0999999999999091</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1034,24 +1034,24 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F9">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1058.3174999999999</v>
+        <v>1054.104</v>
       </c>
       <c r="B10">
-        <v>4.0999999999999091</v>
+        <v>52.269999999999982</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1060,10 +1060,10 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G10">
         <v>2</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1054.104</v>
+        <v>1047.2049999999999</v>
       </c>
       <c r="B11">
-        <v>52.269999999999982</v>
+        <v>3.0399999999999636</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,16 +1092,16 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1047.2049999999999</v>
+        <v>1029.0349999999999</v>
       </c>
       <c r="B12">
-        <v>3.0399999999999636</v>
+        <v>-8.2699999999999818</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,16 +1124,16 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F12">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1017.1890000000002</v>
+        <v>1027.8825000000002</v>
       </c>
       <c r="B13">
-        <v>-23.330000000000041</v>
+        <v>-11.730000000000018</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="F13">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G13">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1010.4208636363636</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B14">
-        <v>79.539999999999964</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="F14">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1208,31 +1208,31 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1009.0708636363636</v>
+        <v>1010.4208636363636</v>
       </c>
       <c r="B15">
-        <v>78.189999999999941</v>
+        <v>79.539999999999964</v>
       </c>
       <c r="C15" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="E15">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="F15">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G15">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K15">
         <v>1.7</v>
@@ -1240,28 +1240,28 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1004.8008636363636</v>
+        <v>1009.0708636363636</v>
       </c>
       <c r="B16">
-        <v>73.919999999999959</v>
+        <v>78.189999999999941</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E16">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="F16">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H16">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>992.30499999999984</v>
+        <v>1004.8008636363636</v>
       </c>
       <c r="B17">
-        <v>-45</v>
+        <v>73.919999999999959</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F17">
+        <v>12</v>
+      </c>
+      <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17">
         <v>10</v>
-      </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-      <c r="H17">
-        <v>12</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Update: Ranking Data (08:10:52)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18B411BB-E86C-466D-9D3D-EEE5F89D8B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{15D6E846-8C72-465B-A523-DF4F079D7F19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{DCF5980D-72DA-4D98-9AE4-7C474482B333}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{E38BBD64-4905-4DB1-B46E-1CB669EC98CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -113,37 +113,37 @@
     <t>FA컵</t>
   </si>
   <si>
+    <t>피파왕초보구단주</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>UEFA_D조</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>콩콩콩룔</t>
   </si>
   <si>
     <t>라치오</t>
-  </si>
-  <si>
-    <t>UEFA_D조</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>피파왕초보구단주</t>
-  </si>
-  <si>
-    <t>리버풀</t>
   </si>
   <si>
     <t>호야국2인</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B35F2FE-A0B0-4023-84A4-B10463F11579}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CA7E2E5-76CB-4251-8C7D-A577645C67B0}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1106.18</v>
+        <v>1098.4974999999999</v>
       </c>
       <c r="B6">
-        <v>99.080000000000041</v>
+        <v>44.279999999999973</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -902,16 +902,16 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J6" t="s">
         <v>26</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1058.3174999999999</v>
+        <v>1087.93</v>
       </c>
       <c r="B9">
-        <v>4.0999999999999091</v>
+        <v>80.830000000000041</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1034,16 +1034,16 @@
         <v>34</v>
       </c>
       <c r="E9">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (06:50:58)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15D6E846-8C72-465B-A523-DF4F079D7F19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CFC5F6A-1497-4E5D-B9E2-9E12D3B734F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{E38BBD64-4905-4DB1-B46E-1CB669EC98CB}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{0DCE8A15-DF6D-4DBB-91D2-0DD651D003CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CA7E2E5-76CB-4251-8C7D-A577645C67B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358AC08B-EAED-41C0-B31E-5A30E8E9F63B}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1089.7550000000001</v>
+        <v>1090.4550000000002</v>
       </c>
       <c r="B8">
-        <v>97.170000000000073</v>
+        <v>97.870000000000118</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,13 +990,13 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F8">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H8">
         <v>4</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>934.26086363636364</v>
+        <v>933.56086363636359</v>
       </c>
       <c r="B21">
-        <v>3.3799999999999955</v>
+        <v>2.67999999999995</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F21">
         <v>17</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>

</xml_diff>

<commit_message>
Update: Ranking Data (16:44:01)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CFC5F6A-1497-4E5D-B9E2-9E12D3B734F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A463DE5E-F7F6-4F6A-B4DC-7086FCF437BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{0DCE8A15-DF6D-4DBB-91D2-0DD651D003CE}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{A1AF1243-FBC4-4D8B-80B1-B93BE74C7E43}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -146,57 +146,57 @@
     <t>라치오</t>
   </si>
   <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
+    <t>FA컵_8강</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
-  </si>
-  <si>
     <t>FA컵_16강</t>
   </si>
   <si>
@@ -236,13 +236,22 @@
     <t>UCL_4강</t>
   </si>
   <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>UCL_8강</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
   </si>
   <si>
-    <t>UCL_8강</t>
+    <t>UEL_FINAL</t>
   </si>
   <si>
     <t>Legend독수리</t>
@@ -251,15 +260,6 @@
     <t>맨체스터 유나이티드</t>
   </si>
   <si>
-    <t>UEL_FINAL</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
-  </si>
-  <si>
     <t>UEL_4강</t>
   </si>
   <si>
@@ -272,19 +272,19 @@
     <t>UEL_8강</t>
   </si>
   <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
     <t>syma</t>
   </si>
   <si>
     <t>RC 셀타 비고</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
   </si>
   <si>
     <t>UECL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358AC08B-EAED-41C0-B31E-5A30E8E9F63B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5299AA93-348D-4CF8-871D-26176D5FFCD4}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1054.104</v>
+        <v>1078.375</v>
       </c>
       <c r="B10">
-        <v>52.269999999999982</v>
+        <v>34.210000000000036</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1060,16 +1060,16 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J10" t="s">
         <v>37</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1047.2049999999999</v>
+        <v>1029.0349999999999</v>
       </c>
       <c r="B11">
-        <v>3.0399999999999636</v>
+        <v>-8.2699999999999818</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,16 +1092,16 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1029.0349999999999</v>
+        <v>1027.8825000000002</v>
       </c>
       <c r="B12">
-        <v>-8.2699999999999818</v>
+        <v>-11.730000000000018</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,16 +1124,16 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F12">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1027.8825000000002</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B13">
-        <v>-11.730000000000018</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
+        <v>39</v>
+      </c>
+      <c r="F13">
         <v>22</v>
       </c>
-      <c r="F13">
-        <v>11</v>
-      </c>
       <c r="G13">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1017.1890000000002</v>
+        <v>1010.4208636363636</v>
       </c>
       <c r="B14">
-        <v>-23.330000000000041</v>
+        <v>79.539999999999964</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F14">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G14">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1208,31 +1208,31 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1010.4208636363636</v>
+        <v>1009.0708636363636</v>
       </c>
       <c r="B15">
-        <v>79.539999999999964</v>
+        <v>78.189999999999941</v>
       </c>
       <c r="C15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15">
+        <v>40</v>
+      </c>
+      <c r="F15">
+        <v>22</v>
+      </c>
+      <c r="G15">
+        <v>5</v>
+      </c>
+      <c r="H15">
+        <v>13</v>
+      </c>
+      <c r="J15" t="s">
         <v>49</v>
-      </c>
-      <c r="D15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15">
-        <v>29</v>
-      </c>
-      <c r="F15">
-        <v>14</v>
-      </c>
-      <c r="G15">
-        <v>4</v>
-      </c>
-      <c r="H15">
-        <v>11</v>
-      </c>
-      <c r="J15" t="s">
-        <v>51</v>
       </c>
       <c r="K15">
         <v>1.7</v>
@@ -1240,28 +1240,28 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1009.0708636363636</v>
+        <v>1007.904</v>
       </c>
       <c r="B16">
-        <v>78.189999999999941</v>
+        <v>6.0699999999999363</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E16">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="F16">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H16">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>990.23086363636367</v>
+        <v>993.9308636363636</v>
       </c>
       <c r="B18">
-        <v>59.350000000000023</v>
+        <v>63.049999999999955</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F18">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G18">
         <v>5</v>
       </c>
       <c r="H18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>933.56086363636359</v>
+        <v>942.79</v>
       </c>
       <c r="B21">
-        <v>2.67999999999995</v>
+        <v>-27.230000000000018</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="F21">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="G21">
         <v>3</v>
       </c>
       <c r="H21">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>914.75400000000002</v>
+        <v>933.56086363636359</v>
       </c>
       <c r="B22">
-        <v>-19.470000000000027</v>
+        <v>2.67999999999995</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,16 +1444,16 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F22">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="G22">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J22" t="s">
         <v>70</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>910.11</v>
+        <v>914.75400000000002</v>
       </c>
       <c r="B23">
-        <v>-59.909999999999968</v>
+        <v>-19.470000000000027</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G23">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H23">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>898.61086363636366</v>
+        <v>895.70086363636369</v>
       </c>
       <c r="B25">
-        <v>-32.269999999999982</v>
+        <v>-35.17999999999995</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,16 +1540,16 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="F25">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="G25">
         <v>3</v>
       </c>
       <c r="H25">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>895.70086363636369</v>
+        <v>895.39086363636363</v>
       </c>
       <c r="B26">
-        <v>-35.17999999999995</v>
+        <v>-35.490000000000009</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="F26">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H26">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>853.88086363636364</v>
+        <v>842.88086363636364</v>
       </c>
       <c r="B28">
-        <v>-77</v>
+        <v>-88</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,24 +1636,24 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>795.11086363636366</v>
+        <v>796.29086363636361</v>
       </c>
       <c r="B29">
-        <v>-135.76999999999998</v>
+        <v>-134.59000000000003</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1662,16 +1662,16 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (16:53:52)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A463DE5E-F7F6-4F6A-B4DC-7086FCF437BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B959A7CA-3F4C-476D-8D9B-ED98A4225228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{A1AF1243-FBC4-4D8B-80B1-B93BE74C7E43}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{77D11D44-0FCC-406F-A50A-69EA4B11D0A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5299AA93-348D-4CF8-871D-26176D5FFCD4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1CE71F-4539-4E45-9F4B-8330E79A9FA2}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (01:52:52)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B959A7CA-3F4C-476D-8D9B-ED98A4225228}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70653504-632F-4BF4-8188-35D04D22EDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{77D11D44-0FCC-406F-A50A-69EA4B11D0A1}"/>
+    <workbookView xWindow="314" yWindow="1155" windowWidth="36185" windowHeight="12632" xr2:uid="{ADC5A2CE-8F98-40E3-AAFB-DE18127C895F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,57 +95,57 @@
     <t>경기 수</t>
   </si>
   <si>
+    <t>피파왕초보구단주</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
     <t>UNIT</t>
   </si>
   <si>
     <t>AS 로마</t>
   </si>
   <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>피파왕초보구단주</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
     <t>UEFA_D조</t>
   </si>
   <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>UEFA Tournament</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>방덕</t>
   </si>
   <si>
     <t>인테르</t>
   </si>
   <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
     <t>은안</t>
   </si>
   <si>
@@ -164,27 +164,27 @@
     <t>2부리그</t>
   </si>
   <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
     <t>Special블루</t>
   </si>
   <si>
     <t>아스널</t>
   </si>
   <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
     <t>FA컵_4강</t>
   </si>
   <si>
@@ -254,21 +254,21 @@
     <t>UEL_FINAL</t>
   </si>
   <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>UEL_4강</t>
+  </si>
+  <si>
     <t>Legend독수리</t>
   </si>
   <si>
     <t>맨체스터 유나이티드</t>
   </si>
   <si>
-    <t>UEL_4강</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
-  </si>
-  <si>
     <t>UEL_8강</t>
   </si>
   <si>
@@ -299,16 +299,16 @@
     <t>UECL_8강</t>
   </si>
   <si>
+    <t>겐지간지</t>
+  </si>
+  <si>
+    <t>파리 생제르맹</t>
+  </si>
+  <si>
     <t>ShangHaiPortFC</t>
   </si>
   <si>
     <t>상하이 선화</t>
-  </si>
-  <si>
-    <t>겐지간지</t>
-  </si>
-  <si>
-    <t>파리 생제르맹</t>
   </si>
 </sst>
 </file>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1CE71F-4539-4E45-9F4B-8330E79A9FA2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4738530F-90CD-4F3C-B1F4-5BEC5EF72588}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1215.144</v>
+        <v>1225.4840000000002</v>
       </c>
       <c r="B3">
-        <v>100.27999999999997</v>
+        <v>110.62000000000012</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,10 +770,10 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3">
         <v>2</v>
@@ -802,10 +802,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1122.4575</v>
+        <v>1170.3875</v>
       </c>
       <c r="B4">
-        <v>91.639999999999873</v>
+        <v>116.17000000000007</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -814,16 +814,16 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F4">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
         <v>5</v>
-      </c>
-      <c r="H4">
-        <v>7</v>
       </c>
       <c r="J4" t="s">
         <v>20</v>
@@ -846,10 +846,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1107.9375</v>
+        <v>1129.5374999999999</v>
       </c>
       <c r="B5">
-        <v>58.980000000000018</v>
+        <v>80.579999999999927</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -858,10 +858,10 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G5">
         <v>2</v>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1098.4974999999999</v>
+        <v>1122.4575</v>
       </c>
       <c r="B6">
-        <v>44.279999999999973</v>
+        <v>91.639999999999873</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
@@ -902,16 +902,16 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J6" t="s">
         <v>26</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1091.6190000000001</v>
+        <v>1090.4550000000002</v>
       </c>
       <c r="B7">
-        <v>64.75</v>
+        <v>97.870000000000118</v>
       </c>
       <c r="C7" t="s">
         <v>27</v>
@@ -946,16 +946,16 @@
         <v>28</v>
       </c>
       <c r="E7">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="F7">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J7" t="s">
         <v>29</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1090.4550000000002</v>
+        <v>1087.93</v>
       </c>
       <c r="B8">
-        <v>97.870000000000118</v>
+        <v>80.830000000000041</v>
       </c>
       <c r="C8" t="s">
         <v>30</v>
@@ -990,16 +990,16 @@
         <v>31</v>
       </c>
       <c r="E8">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="F8">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
         <v>10</v>
-      </c>
-      <c r="H8">
-        <v>4</v>
       </c>
       <c r="J8" t="s">
         <v>32</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1087.93</v>
+        <v>1064.7690000000002</v>
       </c>
       <c r="B9">
-        <v>80.830000000000041</v>
+        <v>37.900000000000091</v>
       </c>
       <c r="C9" t="s">
         <v>33</v>
@@ -1037,21 +1037,21 @@
         <v>23</v>
       </c>
       <c r="F9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1078.375</v>
+        <v>1050.875</v>
       </c>
       <c r="B10">
-        <v>34.210000000000036</v>
+        <v>6.7100000000000364</v>
       </c>
       <c r="C10" t="s">
         <v>35</v>
@@ -1060,7 +1060,7 @@
         <v>36</v>
       </c>
       <c r="E10">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F10">
         <v>10</v>
@@ -1069,7 +1069,7 @@
         <v>3</v>
       </c>
       <c r="H10">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J10" t="s">
         <v>37</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1027.8825000000002</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B12">
-        <v>-11.730000000000018</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,16 +1124,16 @@
         <v>42</v>
       </c>
       <c r="E12">
+        <v>39</v>
+      </c>
+      <c r="F12">
         <v>22</v>
       </c>
-      <c r="F12">
-        <v>11</v>
-      </c>
       <c r="G12">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H12">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1017.1890000000002</v>
+        <v>1016.3608636363637</v>
       </c>
       <c r="B13">
-        <v>-23.330000000000041</v>
+        <v>85.480000000000018</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F13">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G13">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1010.4208636363636</v>
+        <v>1010.3125000000002</v>
       </c>
       <c r="B14">
-        <v>79.539999999999964</v>
+        <v>-29.299999999999955</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F14">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G14">
         <v>4</v>
       </c>
       <c r="H14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>993.9308636363636</v>
+        <v>981.12086363636365</v>
       </c>
       <c r="B18">
-        <v>63.049999999999955</v>
+        <v>50.240000000000009</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F18">
         <v>12</v>
       </c>
       <c r="G18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>970.77086363636363</v>
+        <v>980.97086363636367</v>
       </c>
       <c r="B19">
-        <v>39.889999999999986</v>
+        <v>50.090000000000032</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,22 +1348,22 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F19">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H19">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
       </c>
       <c r="K19">
-        <v>2.2999999999999998</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
@@ -1395,7 +1395,7 @@
         <v>64</v>
       </c>
       <c r="K20">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
@@ -1427,7 +1427,7 @@
         <v>67</v>
       </c>
       <c r="K21">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
@@ -1459,15 +1459,15 @@
         <v>70</v>
       </c>
       <c r="K22">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>914.75400000000002</v>
+        <v>924.21749999999997</v>
       </c>
       <c r="B23">
-        <v>-19.470000000000027</v>
+        <v>-57.440000000000055</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F23">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H23">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>901.28750000000002</v>
+        <v>914.75400000000002</v>
       </c>
       <c r="B24">
-        <v>-80.37</v>
+        <v>-19.470000000000027</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1508,16 +1508,16 @@
         <v>75</v>
       </c>
       <c r="E24">
+        <v>40</v>
+      </c>
+      <c r="F24">
+        <v>11</v>
+      </c>
+      <c r="G24">
+        <v>6</v>
+      </c>
+      <c r="H24">
         <v>23</v>
-      </c>
-      <c r="F24">
-        <v>5</v>
-      </c>
-      <c r="G24">
-        <v>4</v>
-      </c>
-      <c r="H24">
-        <v>14</v>
       </c>
       <c r="J24" t="s">
         <v>76</v>
@@ -1555,15 +1555,15 @@
         <v>79</v>
       </c>
       <c r="K25">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>895.39086363636363</v>
+        <v>893.73086363636367</v>
       </c>
       <c r="B26">
-        <v>-35.490000000000009</v>
+        <v>-37.149999999999977</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F26">
         <v>8</v>
       </c>
       <c r="G26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H26">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1592,10 +1592,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>858.45086363636358</v>
+        <v>885.92086363636361</v>
       </c>
       <c r="B27">
-        <v>-72.430000000000064</v>
+        <v>-44.960000000000036</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,10 +1604,10 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F27">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G27">
         <v>5</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>842.88086363636364</v>
+        <v>796.29086363636361</v>
       </c>
       <c r="B28">
-        <v>-88</v>
+        <v>-134.59000000000003</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,24 +1636,24 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F28">
         <v>4</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H28">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>796.29086363636361</v>
+        <v>792.37086363636365</v>
       </c>
       <c r="B29">
-        <v>-134.59000000000003</v>
+        <v>-138.51</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1662,16 +1662,16 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F29">
         <v>4</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H29">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (01:59:16)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70653504-632F-4BF4-8188-35D04D22EDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{283B688D-4A40-410D-B15C-2439A75D1127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="314" yWindow="1155" windowWidth="36185" windowHeight="12632" xr2:uid="{ADC5A2CE-8F98-40E3-AAFB-DE18127C895F}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{0F401D83-4CF9-4BEA-833D-FCBB8E94DD21}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4738530F-90CD-4F3C-B1F4-5BEC5EF72588}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6D410C8-5870-4DAA-98A4-60E50A50AC7A}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (21:11:02)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{283B688D-4A40-410D-B15C-2439A75D1127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FCCF983-65B2-4D42-AAC6-ECE2DDBA40A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{0F401D83-4CF9-4BEA-833D-FCBB8E94DD21}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{FA0D57FE-592B-4CEE-AE05-B94615F27580}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -164,19 +164,28 @@
     <t>2부리그</t>
   </si>
   <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
     <t>마인츠</t>
   </si>
   <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
     <t>0708ManUtd</t>
   </si>
   <si>
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -185,18 +194,9 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
     <t>FA컵_8강</t>
   </si>
   <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>FA컵_16강</t>
   </si>
   <si>
@@ -281,34 +281,34 @@
     <t>UECL_FINAL</t>
   </si>
   <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>UECL_4강</t>
+  </si>
+  <si>
     <t>syma</t>
   </si>
   <si>
     <t>RC 셀타 비고</t>
   </si>
   <si>
-    <t>UECL_4강</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
-  </si>
-  <si>
     <t>UECL_8강</t>
   </si>
   <si>
+    <t>ShangHaiPortFC</t>
+  </si>
+  <si>
+    <t>상하이 선화</t>
+  </si>
+  <si>
     <t>겐지간지</t>
   </si>
   <si>
     <t>파리 생제르맹</t>
-  </si>
-  <si>
-    <t>ShangHaiPortFC</t>
-  </si>
-  <si>
-    <t>상하이 선화</t>
   </si>
 </sst>
 </file>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6D410C8-5870-4DAA-98A4-60E50A50AC7A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B859DB71-0302-4996-9CBC-E1EBD93BB6B0}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -802,10 +802,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1170.3875</v>
+        <v>1158.1975</v>
       </c>
       <c r="B4">
-        <v>116.17000000000007</v>
+        <v>103.98000000000002</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -814,16 +814,16 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G4">
         <v>4</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J4" t="s">
         <v>20</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1017.1890000000002</v>
+        <v>1019.654</v>
       </c>
       <c r="B12">
-        <v>-23.330000000000041</v>
+        <v>17.819999999999936</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1124,13 +1124,13 @@
         <v>42</v>
       </c>
       <c r="E12">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="F12">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G12">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H12">
         <v>10</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1016.3608636363637</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B13">
-        <v>85.480000000000018</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,16 +1156,16 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F13">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H13">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J13" t="s">
         <v>45</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1010.3125000000002</v>
+        <v>1016.3608636363637</v>
       </c>
       <c r="B14">
-        <v>-29.299999999999955</v>
+        <v>85.480000000000018</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F14">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1208,31 +1208,31 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1009.0708636363636</v>
+        <v>1010.3125000000002</v>
       </c>
       <c r="B15">
-        <v>78.189999999999941</v>
+        <v>-29.299999999999955</v>
       </c>
       <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15">
+        <v>26</v>
+      </c>
+      <c r="F15">
+        <v>12</v>
+      </c>
+      <c r="G15">
+        <v>4</v>
+      </c>
+      <c r="H15">
         <v>10</v>
       </c>
-      <c r="D15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15">
-        <v>40</v>
-      </c>
-      <c r="F15">
-        <v>22</v>
-      </c>
-      <c r="G15">
-        <v>5</v>
-      </c>
-      <c r="H15">
-        <v>13</v>
-      </c>
       <c r="J15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K15">
         <v>1.7</v>
@@ -1240,28 +1240,28 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1007.904</v>
+        <v>1009.0708636363636</v>
       </c>
       <c r="B16">
-        <v>6.0699999999999363</v>
+        <v>78.189999999999941</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E16">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="F16">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H16">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>981.12086363636365</v>
+        <v>1003.7208636363637</v>
       </c>
       <c r="B18">
-        <v>50.240000000000009</v>
+        <v>72.840000000000032</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,10 +1316,10 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F18">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G18">
         <v>7</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>893.73086363636367</v>
+        <v>885.92086363636361</v>
       </c>
       <c r="B26">
-        <v>-37.149999999999977</v>
+        <v>-44.960000000000036</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1575,13 +1575,13 @@
         <v>33</v>
       </c>
       <c r="F26">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G26">
         <v>5</v>
       </c>
       <c r="H26">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1592,10 +1592,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>885.92086363636361</v>
+        <v>882.4408636363637</v>
       </c>
       <c r="B27">
-        <v>-44.960000000000036</v>
+        <v>-48.439999999999941</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,16 +1604,16 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F27">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G27">
         <v>5</v>
       </c>
       <c r="H27">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J27" t="s">
         <v>85</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>796.29086363636361</v>
+        <v>792.37086363636365</v>
       </c>
       <c r="B28">
-        <v>-134.59000000000003</v>
+        <v>-138.51</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,24 +1636,24 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F28">
         <v>4</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H28">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>792.37086363636365</v>
+        <v>791.83086363636357</v>
       </c>
       <c r="B29">
-        <v>-138.51</v>
+        <v>-139.05000000000007</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1662,16 +1662,16 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F29">
         <v>4</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (21:13:10)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FCCF983-65B2-4D42-AAC6-ECE2DDBA40A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C1B34DC-0CA3-49A3-942B-12B8466E6052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{FA0D57FE-592B-4CEE-AE05-B94615F27580}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{E07F4BE3-A0F3-4333-889C-AC3A7DD5F563}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B859DB71-0302-4996-9CBC-E1EBD93BB6B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B425FF5-5CBA-48E4-B51A-B53B50B91855}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (09:12:54)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C1B34DC-0CA3-49A3-942B-12B8466E6052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CE8AAEA-79F3-4274-9689-3CC6905CAE5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{E07F4BE3-A0F3-4333-889C-AC3A7DD5F563}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{1137C469-F723-4DCE-8B20-DE634D85521A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -155,43 +155,43 @@
     <t>1부리그</t>
   </si>
   <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
     <t>아들러</t>
   </si>
   <si>
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>2부리그</t>
-  </si>
-  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
     <t>마인츠</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>0708ManUtd</t>
   </si>
   <si>
     <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
   </si>
   <si>
     <t>FA컵_8강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B425FF5-5CBA-48E4-B51A-B53B50B91855}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48647981-16F9-4C09-9FD9-3A5DAE88F7D5}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1225.4840000000002</v>
+        <v>1233.2740000000001</v>
       </c>
       <c r="B3">
-        <v>110.62000000000012</v>
+        <v>118.41000000000008</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,10 +770,10 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F3">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3">
         <v>2</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1029.0349999999999</v>
+        <v>1036.0625000000002</v>
       </c>
       <c r="B11">
-        <v>-8.2699999999999818</v>
+        <v>-3.5499999999999545</v>
       </c>
       <c r="C11" t="s">
         <v>38</v>
@@ -1092,16 +1092,16 @@
         <v>39</v>
       </c>
       <c r="E11">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H11">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J11" t="s">
         <v>40</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1019.654</v>
+        <v>1029.0349999999999</v>
       </c>
       <c r="B12">
-        <v>17.819999999999936</v>
+        <v>-8.2699999999999818</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -1130,10 +1130,10 @@
         <v>12</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1017.1890000000002</v>
+        <v>1019.654</v>
       </c>
       <c r="B13">
-        <v>-23.330000000000041</v>
+        <v>17.819999999999936</v>
       </c>
       <c r="C13" t="s">
         <v>43</v>
@@ -1156,13 +1156,13 @@
         <v>44</v>
       </c>
       <c r="E13">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="F13">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="G13">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H13">
         <v>10</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1016.3608636363637</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B14">
-        <v>85.480000000000018</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C14" t="s">
         <v>46</v>
@@ -1188,16 +1188,16 @@
         <v>47</v>
       </c>
       <c r="E14">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F14">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
         <v>48</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1010.3125000000002</v>
+        <v>1016.3608636363637</v>
       </c>
       <c r="B15">
-        <v>-29.299999999999955</v>
+        <v>85.480000000000018</v>
       </c>
       <c r="C15" t="s">
         <v>49</v>
@@ -1220,16 +1220,16 @@
         <v>50</v>
       </c>
       <c r="E15">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F15">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H15">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J15" t="s">
         <v>51</v>
@@ -1270,7 +1270,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1004.8008636363636</v>
       </c>
@@ -1302,7 +1302,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1003.7208636363637</v>
       </c>
@@ -1334,7 +1334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>980.97086363636367</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>970.05900000000008</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>942.79</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>933.56086363636359</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>924.21749999999997</v>
       </c>
@@ -1494,12 +1494,12 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>914.75400000000002</v>
+        <v>910.34400000000005</v>
       </c>
       <c r="B24">
-        <v>-19.470000000000027</v>
+        <v>-23.879999999999995</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1508,7 +1508,7 @@
         <v>75</v>
       </c>
       <c r="E24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F24">
         <v>11</v>
@@ -1517,7 +1517,7 @@
         <v>6</v>
       </c>
       <c r="H24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J24" t="s">
         <v>76</v>
@@ -1526,7 +1526,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>895.70086363636369</v>
       </c>
@@ -1555,10 +1555,16 @@
         <v>79</v>
       </c>
       <c r="K25">
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+        <v>1.5</v>
+      </c>
+      <c r="N25">
+        <v>13.47</v>
+      </c>
+      <c r="O25">
+        <v>19.690000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>885.92086363636361</v>
       </c>
@@ -1587,15 +1593,21 @@
         <v>82</v>
       </c>
       <c r="K26">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+        <v>1.4</v>
+      </c>
+      <c r="N26">
+        <v>12.28</v>
+      </c>
+      <c r="O26">
+        <v>17.52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>882.4408636363637</v>
+        <v>863.63086363636364</v>
       </c>
       <c r="B27">
-        <v>-48.439999999999941</v>
+        <v>-67.25</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1604,7 +1616,7 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F27">
         <v>8</v>
@@ -1613,16 +1625,16 @@
         <v>5</v>
       </c>
       <c r="H27">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J27" t="s">
         <v>85</v>
       </c>
       <c r="K27">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>792.37086363636365</v>
       </c>
@@ -1648,7 +1660,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>791.83086363636357</v>
       </c>

</xml_diff>

<commit_message>
Update: Ranking Data (00:48:57)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CE8AAEA-79F3-4274-9689-3CC6905CAE5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{82E7C6B3-5AFC-486B-83D4-46D06D36D6AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{1137C469-F723-4DCE-8B20-DE634D85521A}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{B8B2CC5A-8DA6-4B99-AB08-AC6C6EDC4849}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,97 +71,115 @@
     <t>첼시</t>
   </si>
   <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
+    <t>1부리그</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>UEFA_A조</t>
+  </si>
+  <si>
+    <t>피파왕초보구단주</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>UCL</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
     <t>ZD장인지참치</t>
   </si>
   <si>
-    <t>17시즌</t>
-  </si>
-  <si>
     <t>레버쿠젠</t>
   </si>
   <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
-    <t>피파왕초보구단주</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>UEFA_D조</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>UEFA Tournament</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>2부리그</t>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>아들러</t>
@@ -170,13 +188,16 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
+    <t>FA컵_8강</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_16강</t>
   </si>
   <si>
     <t>오스트리아</t>
@@ -185,19 +206,25 @@
     <t>마인츠</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
-  </si>
-  <si>
-    <t>FA컵_16강</t>
+    <t>FA컵_32강</t>
+  </si>
+  <si>
+    <t>Gucci차붐</t>
+  </si>
+  <si>
+    <t>전북 현대 모터스</t>
+  </si>
+  <si>
+    <t>UEFA</t>
+  </si>
+  <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>UCL_결승전</t>
   </si>
   <si>
     <t>비주류중독</t>
@@ -206,25 +233,7 @@
     <t>셀틱 FC</t>
   </si>
   <si>
-    <t>FA컵_32강</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>UEFA</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
-  </si>
-  <si>
-    <t>UCL_결승전</t>
+    <t>UCL_4강</t>
   </si>
   <si>
     <t>경남FC가즈아</t>
@@ -233,7 +242,7 @@
     <t>경남 FC</t>
   </si>
   <si>
-    <t>UCL_4강</t>
+    <t>UCL_8강</t>
   </si>
   <si>
     <t>Gucci와퍼</t>
@@ -242,22 +251,13 @@
     <t>함부르크SV</t>
   </si>
   <si>
-    <t>UCL_8강</t>
+    <t>UEL_FINAL</t>
   </si>
   <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
-  </si>
-  <si>
-    <t>UEL_FINAL</t>
-  </si>
-  <si>
-    <t>Gucci차붐</t>
-  </si>
-  <si>
-    <t>전북 현대 모터스</t>
   </si>
   <si>
     <t>UEL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48647981-16F9-4C09-9FD9-3A5DAE88F7D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{076A0AC3-D86F-4018-9C99-973B28F077E0}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1260.2724999999998</v>
+        <v>1245.7924999999998</v>
       </c>
       <c r="B2">
-        <v>136.04999999999995</v>
+        <v>121.56999999999994</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -735,16 +735,16 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F2">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1233.2740000000001</v>
+        <v>1233.3040000000001</v>
       </c>
       <c r="B3">
-        <v>118.41000000000008</v>
+        <v>118.44000000000005</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -802,87 +802,87 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1158.1975</v>
+        <v>1205.8575000000001</v>
       </c>
       <c r="B4">
-        <v>103.98000000000002</v>
+        <v>175.03999999999996</v>
       </c>
       <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4">
+        <v>29</v>
+      </c>
+      <c r="F4">
+        <v>15</v>
+      </c>
+      <c r="G4">
+        <v>6</v>
+      </c>
+      <c r="H4">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4">
-        <v>21</v>
-      </c>
-      <c r="F4">
-        <v>11</v>
-      </c>
-      <c r="G4">
+      <c r="K4">
+        <v>31.600000000000009</v>
+      </c>
+      <c r="L4">
+        <v>12</v>
+      </c>
+      <c r="M4">
         <v>4</v>
-      </c>
-      <c r="H4">
-        <v>6</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4">
-        <v>22.979999999999997</v>
-      </c>
-      <c r="L4">
-        <v>26</v>
-      </c>
-      <c r="M4">
-        <v>15</v>
       </c>
       <c r="N4">
         <v>3</v>
       </c>
       <c r="O4">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1129.5374999999999</v>
+        <v>1172.9675</v>
       </c>
       <c r="B5">
-        <v>80.579999999999927</v>
+        <v>124.00999999999999</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F5">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G5">
         <v>2</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K5">
-        <v>23.44</v>
+        <v>22.51</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <v>1</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5">
         <v>0</v>
@@ -890,90 +890,90 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1122.4575</v>
+        <v>1113.075</v>
       </c>
       <c r="B6">
-        <v>91.639999999999873</v>
+        <v>120.49000000000001</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6">
+        <v>43</v>
+      </c>
+      <c r="F6">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="J6" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6">
-        <v>25</v>
-      </c>
-      <c r="F6">
-        <v>13</v>
-      </c>
-      <c r="G6">
-        <v>5</v>
-      </c>
-      <c r="H6">
-        <v>7</v>
-      </c>
-      <c r="J6" t="s">
-        <v>26</v>
-      </c>
       <c r="K6">
-        <v>31.770000000000003</v>
+        <v>37.53</v>
       </c>
       <c r="L6">
         <v>12</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1090.4550000000002</v>
+        <v>1104.9675</v>
       </c>
       <c r="B7">
-        <v>97.870000000000118</v>
+        <v>50.75</v>
       </c>
       <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7">
+        <v>25</v>
+      </c>
+      <c r="F7">
+        <v>12</v>
+      </c>
+      <c r="G7">
+        <v>4</v>
+      </c>
+      <c r="H7">
+        <v>9</v>
+      </c>
+      <c r="J7" t="s">
         <v>27</v>
       </c>
-      <c r="D7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7">
-        <v>40</v>
-      </c>
-      <c r="F7">
-        <v>26</v>
-      </c>
-      <c r="G7">
-        <v>10</v>
-      </c>
-      <c r="H7">
+      <c r="K7">
+        <v>83.4</v>
+      </c>
+      <c r="L7">
         <v>4</v>
       </c>
-      <c r="J7" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
       <c r="M7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
@@ -984,10 +984,10 @@
         <v>80.830000000000041</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E8">
         <v>23</v>
@@ -1002,77 +1002,77 @@
         <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K8">
-        <v>78.19</v>
+        <v>175.04000000000002</v>
       </c>
       <c r="L8">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="M8">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="N8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O8">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1064.7690000000002</v>
+        <v>1085.2090000000001</v>
       </c>
       <c r="B9">
-        <v>37.900000000000091</v>
+        <v>58.339999999999918</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E9">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G9">
         <v>2</v>
       </c>
       <c r="H9">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1050.875</v>
+        <v>1064.1608636363637</v>
       </c>
       <c r="B10">
-        <v>6.7100000000000364</v>
+        <v>133.28000000000009</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10">
         <v>36</v>
       </c>
-      <c r="E10">
-        <v>21</v>
-      </c>
       <c r="F10">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H10">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J10" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1080,31 +1080,31 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1036.0625000000002</v>
+        <v>1050.7349999999999</v>
       </c>
       <c r="B11">
-        <v>-3.5499999999999545</v>
+        <v>6.5699999999999363</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E11">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -1112,31 +1112,31 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1029.0349999999999</v>
+        <v>1036.1525000000001</v>
       </c>
       <c r="B12">
-        <v>-8.2699999999999818</v>
+        <v>-3.4600000000000364</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D12" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F12">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H12">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J12" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K12">
         <v>0.3</v>
@@ -1144,31 +1144,31 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1019.654</v>
+        <v>1032.8308636363636</v>
       </c>
       <c r="B13">
-        <v>17.819999999999936</v>
+        <v>101.94999999999993</v>
       </c>
       <c r="C13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13">
+        <v>41</v>
+      </c>
+      <c r="F13">
+        <v>23</v>
+      </c>
+      <c r="G13">
+        <v>5</v>
+      </c>
+      <c r="H13">
+        <v>13</v>
+      </c>
+      <c r="J13" t="s">
         <v>43</v>
-      </c>
-      <c r="D13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E13">
-        <v>25</v>
-      </c>
-      <c r="F13">
-        <v>12</v>
-      </c>
-      <c r="G13">
-        <v>3</v>
-      </c>
-      <c r="H13">
-        <v>10</v>
-      </c>
-      <c r="J13" t="s">
-        <v>45</v>
       </c>
       <c r="K13">
         <v>2.1</v>
@@ -1176,31 +1176,31 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1017.1890000000002</v>
+        <v>1020.3208636363636</v>
       </c>
       <c r="B14">
-        <v>-23.330000000000041</v>
+        <v>89.439999999999941</v>
       </c>
       <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14">
+        <v>35</v>
+      </c>
+      <c r="F14">
+        <v>19</v>
+      </c>
+      <c r="G14">
+        <v>5</v>
+      </c>
+      <c r="H14">
+        <v>11</v>
+      </c>
+      <c r="J14" t="s">
         <v>46</v>
-      </c>
-      <c r="D14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E14">
-        <v>39</v>
-      </c>
-      <c r="F14">
-        <v>22</v>
-      </c>
-      <c r="G14">
-        <v>7</v>
-      </c>
-      <c r="H14">
-        <v>10</v>
-      </c>
-      <c r="J14" t="s">
-        <v>48</v>
       </c>
       <c r="K14">
         <v>1.9</v>
@@ -1208,31 +1208,31 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1016.3608636363637</v>
+        <v>1019.7849999999999</v>
       </c>
       <c r="B15">
-        <v>85.480000000000018</v>
+        <v>-17.519999999999982</v>
       </c>
       <c r="C15" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15">
+        <v>28</v>
+      </c>
+      <c r="F15">
+        <v>13</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>14</v>
+      </c>
+      <c r="J15" t="s">
         <v>49</v>
-      </c>
-      <c r="D15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15">
-        <v>33</v>
-      </c>
-      <c r="F15">
-        <v>17</v>
-      </c>
-      <c r="G15">
-        <v>5</v>
-      </c>
-      <c r="H15">
-        <v>11</v>
-      </c>
-      <c r="J15" t="s">
-        <v>51</v>
       </c>
       <c r="K15">
         <v>1.7</v>
@@ -1240,28 +1240,28 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1009.0708636363636</v>
+        <v>1018.8440000000001</v>
       </c>
       <c r="B16">
-        <v>78.189999999999941</v>
+        <v>17.009999999999991</v>
       </c>
       <c r="C16" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16">
+        <v>28</v>
+      </c>
+      <c r="F16">
+        <v>13</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16">
         <v>12</v>
-      </c>
-      <c r="E16">
-        <v>40</v>
-      </c>
-      <c r="F16">
-        <v>22</v>
-      </c>
-      <c r="G16">
-        <v>5</v>
-      </c>
-      <c r="H16">
-        <v>13</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1004.8008636363636</v>
+        <v>1017.1890000000002</v>
       </c>
       <c r="B17">
-        <v>73.919999999999959</v>
+        <v>-23.330000000000041</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,13 +1284,13 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F17">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H17">
         <v>10</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>1003.7208636363637</v>
+        <v>986.98749999999995</v>
       </c>
       <c r="B18">
-        <v>72.840000000000032</v>
+        <v>5.3299999999999272</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F18">
+        <v>8</v>
+      </c>
+      <c r="G18">
+        <v>5</v>
+      </c>
+      <c r="H18">
         <v>15</v>
-      </c>
-      <c r="G18">
-        <v>7</v>
-      </c>
-      <c r="H18">
-        <v>10</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>980.97086363636367</v>
+        <v>981.4308636363636</v>
       </c>
       <c r="B19">
-        <v>50.090000000000032</v>
+        <v>50.549999999999955</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1368,10 +1368,10 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>970.05900000000008</v>
+        <v>975.51086363636364</v>
       </c>
       <c r="B20">
-        <v>18.350000000000023</v>
+        <v>44.629999999999995</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,16 +1380,16 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F20">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H20">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>942.79</v>
+        <v>970.05900000000008</v>
       </c>
       <c r="B21">
-        <v>-27.230000000000018</v>
+        <v>18.350000000000023</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,10 +1412,10 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F21">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="G21">
         <v>3</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>933.56086363636359</v>
+        <v>941.91</v>
       </c>
       <c r="B22">
-        <v>2.67999999999995</v>
+        <v>-28.110000000000014</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,16 +1444,16 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="F22">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="G22">
         <v>3</v>
       </c>
       <c r="H22">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J22" t="s">
         <v>70</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>924.21749999999997</v>
+        <v>933.56086363636359</v>
       </c>
       <c r="B23">
-        <v>-57.440000000000055</v>
+        <v>2.67999999999995</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="F23">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G23">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H23">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>895.70086363636369</v>
+        <v>895.69086363636359</v>
       </c>
       <c r="B25">
-        <v>-35.17999999999995</v>
+        <v>-35.190000000000055</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1604,10 +1604,10 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>863.63086363636364</v>
+        <v>867.36086363636366</v>
       </c>
       <c r="B27">
-        <v>-67.25</v>
+        <v>-63.519999999999982</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1616,13 +1616,13 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F27">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H27">
         <v>23</v>
@@ -1636,10 +1636,10 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>792.37086363636365</v>
+        <v>792.36086363636355</v>
       </c>
       <c r="B28">
-        <v>-138.51</v>
+        <v>-138.5200000000001</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1662,10 +1662,10 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>791.83086363636357</v>
+        <v>785.5708636363637</v>
       </c>
       <c r="B29">
-        <v>-139.05000000000007</v>
+        <v>-145.30999999999995</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1674,16 +1674,16 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F29">
         <v>4</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (00:27:43)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{58343AB5-0166-4C23-A697-F5E847A14A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B66CCA1-0C39-470B-A8B1-A0AEAA8DDEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2224" yWindow="556" windowWidth="32906" windowHeight="12632" xr2:uid="{40937D09-0AA8-42C5-96ED-6608F16CE97E}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{44BBE9A8-27F5-4C92-B22D-67FBE6433A83}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -173,30 +173,30 @@
     <t>FA컵_결승전</t>
   </si>
   <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>FA컵_8강</t>
+  </si>
+  <si>
     <t>0708ManUtd</t>
   </si>
   <si>
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>FA컵_16강</t>
   </si>
   <si>
@@ -209,19 +209,19 @@
     <t>FA컵_32강</t>
   </si>
   <si>
+    <t>용신</t>
+  </si>
+  <si>
+    <t>토트넘</t>
+  </si>
+  <si>
+    <t>UEFA</t>
+  </si>
+  <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>UEFA</t>
-  </si>
-  <si>
-    <t>용신</t>
-  </si>
-  <si>
-    <t>토트넘</t>
   </si>
   <si>
     <t>UCL_결승전</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56764EB4-3023-4071-9A1E-257B57B573F1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94C59142-3C0E-4C00-8B28-A146F60040FC}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1245.7924999999998</v>
+        <v>1257.28</v>
       </c>
       <c r="B2">
-        <v>121.56999999999994</v>
+        <v>122.5</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1233.3040000000001</v>
+        <v>1250.0862500000001</v>
       </c>
       <c r="B3">
-        <v>118.44000000000005</v>
+        <v>113.96000000000004</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -802,10 +802,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1205.8575000000001</v>
+        <v>1231.9599999999998</v>
       </c>
       <c r="B4">
-        <v>175.03999999999996</v>
+        <v>193.15999999999985</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -814,10 +814,10 @@
         <v>12</v>
       </c>
       <c r="E4">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G4">
         <v>6</v>
@@ -829,7 +829,7 @@
         <v>18</v>
       </c>
       <c r="K4">
-        <v>31.600000000000009</v>
+        <v>31.680000000000007</v>
       </c>
       <c r="L4">
         <v>12</v>
@@ -846,10 +846,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1172.9675</v>
+        <v>1182.94</v>
       </c>
       <c r="B5">
-        <v>124.00999999999999</v>
+        <v>125.47000000000003</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -873,13 +873,13 @@
         <v>21</v>
       </c>
       <c r="K5">
-        <v>22.51</v>
+        <v>39.82</v>
       </c>
       <c r="L5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1113.075</v>
+        <v>1124.5225</v>
       </c>
       <c r="B6">
-        <v>120.49000000000001</v>
+        <v>123.90000000000009</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -917,7 +917,7 @@
         <v>24</v>
       </c>
       <c r="K6">
-        <v>37.53</v>
+        <v>37.880000000000003</v>
       </c>
       <c r="L6">
         <v>12</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1104.9675</v>
+        <v>1115.9450000000002</v>
       </c>
       <c r="B7">
-        <v>50.75</v>
+        <v>50.940000000000055</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -961,7 +961,7 @@
         <v>27</v>
       </c>
       <c r="K7">
-        <v>83.4</v>
+        <v>83.78</v>
       </c>
       <c r="L7">
         <v>4</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1087.93</v>
+        <v>1098.1475</v>
       </c>
       <c r="B8">
-        <v>80.830000000000041</v>
+        <v>81.300000000000068</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -1005,13 +1005,13 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>175.04000000000002</v>
+        <v>193.16</v>
       </c>
       <c r="L8">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M8">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N8">
         <v>6</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1085.2090000000001</v>
+        <v>1095.0862499999998</v>
       </c>
       <c r="B9">
-        <v>58.339999999999918</v>
+        <v>61.769999999999982</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1064.1608636363637</v>
+        <v>1077.739</v>
       </c>
       <c r="B10">
-        <v>133.28000000000009</v>
+        <v>138.06999999999994</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1050.7349999999999</v>
+        <v>1060.29</v>
       </c>
       <c r="B11">
-        <v>6.5699999999999363</v>
+        <v>9.9100000000000819</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1036.1525000000001</v>
+        <v>1049.76</v>
       </c>
       <c r="B12">
-        <v>-3.4600000000000364</v>
+        <v>-4.5699999999999363</v>
       </c>
       <c r="C12" t="s">
         <v>38</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1032.8308636363636</v>
+        <v>1037.1590000000001</v>
       </c>
       <c r="B13">
-        <v>101.94999999999993</v>
+        <v>97.490000000000009</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,7 +1156,7 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F13">
         <v>23</v>
@@ -1165,21 +1165,21 @@
         <v>5</v>
       </c>
       <c r="H13">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J13" t="s">
         <v>43</v>
       </c>
       <c r="K13">
-        <v>2.1</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1020.3208636363636</v>
+        <v>1035.58125</v>
       </c>
       <c r="B14">
-        <v>89.439999999999941</v>
+        <v>5.3099999999999454</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1188,30 +1188,30 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F14">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J14" t="s">
         <v>46</v>
       </c>
       <c r="K14">
-        <v>1.9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1019.7849999999999</v>
+        <v>1031.8049999999998</v>
       </c>
       <c r="B15">
-        <v>-17.519999999999982</v>
+        <v>-14.120000000000118</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1235,15 +1235,15 @@
         <v>49</v>
       </c>
       <c r="K15">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1018.8440000000001</v>
+        <v>1030.809</v>
       </c>
       <c r="B16">
-        <v>17.009999999999991</v>
+        <v>91.139999999999873</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,30 +1252,30 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="F16">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H16">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
       </c>
       <c r="K16">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1017.1890000000002</v>
+        <v>1030.3562499999998</v>
       </c>
       <c r="B17">
-        <v>-23.330000000000041</v>
+        <v>-28.230000000000018</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1299,15 +1299,15 @@
         <v>55</v>
       </c>
       <c r="K17">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>986.98749999999995</v>
+        <v>997.39900000000011</v>
       </c>
       <c r="B18">
-        <v>5.3299999999999272</v>
+        <v>57.730000000000018</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F18">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G18">
         <v>5</v>
       </c>
       <c r="H18">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>981.4308636363636</v>
+        <v>997.17500000000007</v>
       </c>
       <c r="B19">
-        <v>50.549999999999955</v>
+        <v>10.200000000000045</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,30 +1348,30 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F19">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G19">
         <v>5</v>
       </c>
       <c r="H19">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
       </c>
       <c r="K19">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>975.51086363636364</v>
+        <v>987.35900000000015</v>
       </c>
       <c r="B20">
-        <v>44.629999999999995</v>
+        <v>47.690000000000055</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1395,15 +1395,15 @@
         <v>64</v>
       </c>
       <c r="K20">
-        <v>2.1</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>970.05900000000008</v>
+        <v>980.19124999999985</v>
       </c>
       <c r="B21">
-        <v>18.350000000000023</v>
+        <v>21.559999999999945</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>941.91</v>
+        <v>954.3599999999999</v>
       </c>
       <c r="B22">
-        <v>-28.110000000000014</v>
+        <v>-27.970000000000027</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>933.56086363636359</v>
+        <v>944.05900000000008</v>
       </c>
       <c r="B23">
-        <v>2.67999999999995</v>
+        <v>4.3899999999999864</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>910.34400000000005</v>
+        <v>924.23124999999993</v>
       </c>
       <c r="B24">
-        <v>-23.879999999999995</v>
+        <v>-21.210000000000036</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>895.69086363636359</v>
+        <v>906.21900000000005</v>
       </c>
       <c r="B25">
-        <v>-35.190000000000055</v>
+        <v>-33.450000000000045</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1566,10 +1566,10 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>885.92086363636361</v>
+        <v>895.80900000000008</v>
       </c>
       <c r="B26">
-        <v>-44.960000000000036</v>
+        <v>-43.860000000000014</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1604,10 +1604,10 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>867.36086363636366</v>
+        <v>878.24900000000014</v>
       </c>
       <c r="B27">
-        <v>-63.519999999999982</v>
+        <v>-61.419999999999959</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1636,10 +1636,10 @@
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>792.36086363636355</v>
+        <v>803.15900000000011</v>
       </c>
       <c r="B28">
-        <v>-138.5200000000001</v>
+        <v>-136.51</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1662,10 +1662,10 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>785.5708636363637</v>
+        <v>791.43900000000008</v>
       </c>
       <c r="B29">
-        <v>-145.30999999999995</v>
+        <v>-148.23000000000002</v>
       </c>
       <c r="C29" t="s">
         <v>88</v>
@@ -1674,7 +1674,7 @@
         <v>89</v>
       </c>
       <c r="E29">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F29">
         <v>4</v>
@@ -1683,7 +1683,7 @@
         <v>1</v>
       </c>
       <c r="H29">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (02:29:43)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B66CCA1-0C39-470B-A8B1-A0AEAA8DDEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB8A1AF4-5FEC-4C8C-A7F8-3228025286F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{44BBE9A8-27F5-4C92-B22D-67FBE6433A83}"/>
+    <workbookView xWindow="399" yWindow="713" windowWidth="32621" windowHeight="17608" xr2:uid="{59C7872C-8E87-4F31-9648-C1DC7885AE44}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,85 +65,112 @@
     <t>패</t>
   </si>
   <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>대회종류</t>
+  </si>
+  <si>
+    <t>ELO 변동값</t>
+  </si>
+  <si>
+    <t>경기 수</t>
+  </si>
+  <si>
     <t>Voor</t>
   </si>
   <si>
     <t>첼시</t>
   </si>
   <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>17시즌</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
-    <t>대회종류</t>
-  </si>
-  <si>
-    <t>ELO 변동값</t>
-  </si>
-  <si>
-    <t>경기 수</t>
-  </si>
-  <si>
     <t>1부리그</t>
   </si>
   <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
     <t>FA컵</t>
   </si>
   <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>UEFA_A조</t>
+  </si>
+  <si>
+    <t>피파왕초보구단주</t>
+  </si>
+  <si>
+    <t>리버풀</t>
+  </si>
+  <si>
+    <t>UCL</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
     <t>앙쿠</t>
   </si>
   <si>
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
-    <t>UEFA_A조</t>
-  </si>
-  <si>
-    <t>피파왕초보구단주</t>
-  </si>
-  <si>
-    <t>리버풀</t>
-  </si>
-  <si>
-    <t>UCL</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>FA컵_결승전</t>
   </si>
   <si>
     <t>은안</t>
@@ -152,33 +179,6 @@
     <t>맨체스터 시티</t>
   </si>
   <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
     <t>FA컵_4강</t>
   </si>
   <si>
@@ -209,28 +209,28 @@
     <t>FA컵_32강</t>
   </si>
   <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>UEFA</t>
+  </si>
+  <si>
     <t>용신</t>
   </si>
   <si>
     <t>토트넘</t>
   </si>
   <si>
-    <t>UEFA</t>
+    <t>UCL_결승전</t>
   </si>
   <si>
     <t>Gucci차붐</t>
   </si>
   <si>
     <t>전북 현대 모터스</t>
-  </si>
-  <si>
-    <t>UCL_결승전</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
   </si>
   <si>
     <t>UCL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94C59142-3C0E-4C00-8B28-A146F60040FC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5381D9CC-2F6D-4E97-B7EA-A98420FCEAFA}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1257.28</v>
+        <v>1307.7962500000001</v>
       </c>
       <c r="B2">
-        <v>122.5</v>
+        <v>171.67000000000007</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -738,13 +738,13 @@
         <v>29</v>
       </c>
       <c r="F2">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1250.0862500000001</v>
+        <v>1273.4100000000001</v>
       </c>
       <c r="B3">
-        <v>113.96000000000004</v>
+        <v>215.94000000000005</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,16 +770,16 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F3">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
@@ -802,31 +802,31 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>1231.9599999999998</v>
+        <v>1257.8</v>
       </c>
       <c r="B4">
-        <v>193.15999999999985</v>
+        <v>123.01999999999998</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E4">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F4">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G4">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K4">
         <v>31.680000000000007</v>
@@ -846,40 +846,40 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1182.94</v>
+        <v>1247.6299999999999</v>
       </c>
       <c r="B5">
-        <v>125.47000000000003</v>
+        <v>208.82999999999993</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E5">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="F5">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="J5" t="s">
         <v>21</v>
       </c>
       <c r="K5">
-        <v>39.82</v>
+        <v>57.83</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -890,10 +890,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1124.5225</v>
+        <v>1135.4090000000001</v>
       </c>
       <c r="B6">
-        <v>123.90000000000009</v>
+        <v>195.74</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -902,16 +902,16 @@
         <v>23</v>
       </c>
       <c r="E6">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="F6">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H6">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="J6" t="s">
         <v>24</v>
@@ -961,19 +961,19 @@
         <v>27</v>
       </c>
       <c r="K7">
-        <v>83.78</v>
+        <v>81.44</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M7">
+        <v>3</v>
+      </c>
+      <c r="N7">
         <v>2</v>
       </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
       <c r="O7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
@@ -1005,19 +1005,19 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>193.16</v>
+        <v>208.83</v>
       </c>
       <c r="L8">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="M8">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O8">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1048,10 +1048,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1077.739</v>
+        <v>1093.259</v>
       </c>
       <c r="B10">
-        <v>138.06999999999994</v>
+        <v>153.58999999999992</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1060,19 +1060,19 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="F10">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G10">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H10">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1060.29</v>
+        <v>1093.0425</v>
       </c>
       <c r="B11">
-        <v>9.9100000000000819</v>
+        <v>92.420000000000073</v>
       </c>
       <c r="C11" t="s">
         <v>35</v>
@@ -1092,16 +1092,16 @@
         <v>36</v>
       </c>
       <c r="E11">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="F11">
+        <v>28</v>
+      </c>
+      <c r="G11">
         <v>10</v>
       </c>
-      <c r="G11">
-        <v>3</v>
-      </c>
       <c r="H11">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J11" t="s">
         <v>37</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1049.76</v>
+        <v>1060.77125</v>
       </c>
       <c r="B12">
-        <v>-4.5699999999999363</v>
+        <v>30.5</v>
       </c>
       <c r="C12" t="s">
         <v>38</v>
@@ -1124,16 +1124,16 @@
         <v>39</v>
       </c>
       <c r="E12">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F12">
         <v>14</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J12" t="s">
         <v>40</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1037.1590000000001</v>
+        <v>1049.76</v>
       </c>
       <c r="B13">
-        <v>97.490000000000009</v>
+        <v>-4.5699999999999363</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,16 +1156,16 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="F13">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H13">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J13" t="s">
         <v>43</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1035.58125</v>
+        <v>1045.9299999999998</v>
       </c>
       <c r="B14">
-        <v>5.3099999999999454</v>
+        <v>-4.4500000000000455</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1188,16 +1188,16 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F14">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G14">
         <v>3</v>
       </c>
       <c r="H14">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
         <v>46</v>
@@ -1270,7 +1270,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1030.3562499999998</v>
       </c>
@@ -1302,12 +1302,12 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>997.39900000000011</v>
+        <v>987.35900000000015</v>
       </c>
       <c r="B18">
-        <v>57.730000000000018</v>
+        <v>47.690000000000055</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,13 +1316,13 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F18">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H18">
         <v>13</v>
@@ -1334,12 +1334,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>997.17500000000007</v>
+        <v>980.00900000000013</v>
       </c>
       <c r="B19">
-        <v>10.200000000000045</v>
+        <v>40.340000000000032</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,13 +1348,13 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="F19">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="G19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H19">
         <v>15</v>
@@ -1366,12 +1366,12 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>987.35900000000015</v>
+        <v>975.125</v>
       </c>
       <c r="B20">
-        <v>47.690000000000055</v>
+        <v>-11.850000000000023</v>
       </c>
       <c r="C20" t="s">
         <v>62</v>
@@ -1380,16 +1380,16 @@
         <v>63</v>
       </c>
       <c r="E20">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F20">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H20">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J20" t="s">
         <v>64</v>
@@ -1398,12 +1398,12 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>980.19124999999985</v>
+        <v>970.53124999999989</v>
       </c>
       <c r="B21">
-        <v>21.559999999999945</v>
+        <v>11.899999999999977</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F21">
         <v>16</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H21">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1430,7 +1430,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>954.3599999999999</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>1.9</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>944.05900000000008</v>
       </c>
@@ -1494,7 +1494,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>924.23124999999993</v>
       </c>
@@ -1526,7 +1526,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>906.21900000000005</v>
       </c>
@@ -1557,14 +1557,8 @@
       <c r="K25">
         <v>1.5</v>
       </c>
-      <c r="N25">
-        <v>13.47</v>
-      </c>
-      <c r="O25">
-        <v>19.690000000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>895.80900000000008</v>
       </c>
@@ -1595,19 +1589,13 @@
       <c r="K26">
         <v>1.4</v>
       </c>
-      <c r="N26">
-        <v>12.28</v>
-      </c>
-      <c r="O26">
-        <v>17.52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>878.24900000000014</v>
+        <v>885.59900000000016</v>
       </c>
       <c r="B27">
-        <v>-61.419999999999959</v>
+        <v>-54.069999999999936</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1616,13 +1604,13 @@
         <v>84</v>
       </c>
       <c r="E27">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H27">
         <v>23</v>
@@ -1634,7 +1622,7 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>803.15900000000011</v>
       </c>
@@ -1660,7 +1648,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>791.43900000000008</v>
       </c>

</xml_diff>

<commit_message>
Update: Ranking Data (02:31:05)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB8A1AF4-5FEC-4C8C-A7F8-3228025286F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEA34473-D72B-463E-A045-97CF6DF77FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="399" yWindow="713" windowWidth="32621" windowHeight="17608" xr2:uid="{59C7872C-8E87-4F31-9648-C1DC7885AE44}"/>
+    <workbookView xWindow="399" yWindow="713" windowWidth="32621" windowHeight="17608" xr2:uid="{FA52CCD2-948F-48C4-B640-3223512B602E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5381D9CC-2F6D-4E97-B7EA-A98420FCEAFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796F12D2-ACD8-4CC4-B9D2-F1381838E237}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (02:32:55)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEA34473-D72B-463E-A045-97CF6DF77FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABD2CC6C-8572-4E53-8627-B1E4317C37A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="399" yWindow="713" windowWidth="32621" windowHeight="17608" xr2:uid="{FA52CCD2-948F-48C4-B640-3223512B602E}"/>
+    <workbookView xWindow="399" yWindow="713" windowWidth="32621" windowHeight="17608" xr2:uid="{15A1EBFA-6923-488A-9059-3FED25C20F40}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{796F12D2-ACD8-4CC4-B9D2-F1381838E237}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDECBEC3-E0B8-413C-925B-05FB41CF9922}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (06:12:34)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1838F154-D4D6-4109-AB27-388C4E5B4C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2638D856-A3BF-4FBD-A506-FFD79B64ED9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1084" yWindow="1397" windowWidth="32621" windowHeight="17608" xr2:uid="{3070C2AF-2AB3-4AE3-8697-3B720F2B6226}"/>
+    <workbookView xWindow="1084" yWindow="1397" windowWidth="32621" windowHeight="17608" xr2:uid="{2EC0834F-999B-4BB0-B54E-65CD1DDE4531}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E737F7B-E491-4A89-B6B7-38C3530AC328}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{067B37A1-CECD-49DE-A2C3-894950F1B46F}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (07:39:39)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2638D856-A3BF-4FBD-A506-FFD79B64ED9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{543DE379-C0DF-4FE1-BFB2-86821631417E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1084" yWindow="1397" windowWidth="32621" windowHeight="17608" xr2:uid="{2EC0834F-999B-4BB0-B54E-65CD1DDE4531}"/>
+    <workbookView xWindow="1084" yWindow="1397" windowWidth="32621" windowHeight="17608" xr2:uid="{59E2070D-6FDE-429B-ADCD-4F6032C2705F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{067B37A1-CECD-49DE-A2C3-894950F1B46F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{502A9930-7F1F-4F32-8E8B-DDA591DFEA1B}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>970.53124999999989</v>
+        <v>969.67124999999987</v>
       </c>
       <c r="B21">
-        <v>11.899999999999977</v>
+        <v>11.039999999999964</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F21">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G21">
         <v>5</v>
       </c>
       <c r="H21">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>944.05900000000008</v>
+        <v>944.89900000000011</v>
       </c>
       <c r="B23">
-        <v>4.3899999999999864</v>
+        <v>5.2300000000000182</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F23">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G23">
         <v>3</v>
       </c>
       <c r="H23">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>

</xml_diff>

<commit_message>
Update: Ranking Data (01:34:46)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{543DE379-C0DF-4FE1-BFB2-86821631417E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EFEE5E0-2575-4F46-AE03-B6AACA6806B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1084" yWindow="1397" windowWidth="32621" windowHeight="17608" xr2:uid="{59E2070D-6FDE-429B-ADCD-4F6032C2705F}"/>
+    <workbookView xWindow="1768" yWindow="2082" windowWidth="32621" windowHeight="17608" xr2:uid="{9676FA2C-4EB3-4B76-AA59-6F1E23D3AFD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -155,13 +155,31 @@
     <t>2부리그</t>
   </si>
   <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>3부리그</t>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -170,16 +188,7 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>FA컵_4강</t>
+    <t>FA컵_8강</t>
   </si>
   <si>
     <t>아들러</t>
@@ -188,7 +197,7 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>FA컵_8강</t>
+    <t>FA컵_16강</t>
   </si>
   <si>
     <t>0708ManUtd</t>
@@ -197,15 +206,6 @@
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>FA컵_16강</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
     <t>FA컵_32강</t>
   </si>
   <si>
@@ -272,19 +272,19 @@
     <t>UEL_8강</t>
   </si>
   <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
     <t>suma수마</t>
   </si>
   <si>
     <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
   </si>
   <si>
     <t>UECL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{502A9930-7F1F-4F32-8E8B-DDA591DFEA1B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B4FFAB-8F37-46E9-8E6C-762D6515ECE3}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1282.19</v>
+        <v>1274.8400000000001</v>
       </c>
       <c r="B3">
-        <v>224.72000000000003</v>
+        <v>217.37000000000012</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -770,16 +770,16 @@
         <v>12</v>
       </c>
       <c r="E3">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3">
         <v>4</v>
       </c>
       <c r="H3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J3" t="s">
         <v>13</v>
@@ -829,19 +829,19 @@
         <v>18</v>
       </c>
       <c r="K4">
-        <v>58.65</v>
+        <v>51.3</v>
       </c>
       <c r="L4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4">
         <v>1</v>
       </c>
       <c r="O4">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1123.2690000000002</v>
+        <v>1122.6390000000001</v>
       </c>
       <c r="B7">
-        <v>183.60000000000014</v>
+        <v>182.97000000000003</v>
       </c>
       <c r="C7" t="s">
         <v>25</v>
@@ -946,16 +946,16 @@
         <v>26</v>
       </c>
       <c r="E7">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F7">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G7">
         <v>9</v>
       </c>
       <c r="H7">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J7" t="s">
         <v>27</v>
@@ -1005,19 +1005,19 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>224.72</v>
+        <v>217.37</v>
       </c>
       <c r="L8">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="M8">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="N8">
         <v>4</v>
       </c>
       <c r="O8">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1060.77125</v>
+        <v>1086.8699999999999</v>
       </c>
       <c r="B12">
-        <v>30.5</v>
+        <v>36.490000000000009</v>
       </c>
       <c r="C12" t="s">
         <v>38</v>
@@ -1124,16 +1124,16 @@
         <v>39</v>
       </c>
       <c r="E12">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F12">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G12">
         <v>3</v>
       </c>
       <c r="H12">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J12" t="s">
         <v>40</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1049.76</v>
+        <v>1060.77125</v>
       </c>
       <c r="B13">
-        <v>-4.5699999999999363</v>
+        <v>30.5</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,16 +1156,16 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F13">
         <v>14</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H13">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J13" t="s">
         <v>43</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1045.9299999999998</v>
+        <v>1056.4762499999999</v>
       </c>
       <c r="B14">
-        <v>-4.4500000000000455</v>
+        <v>-2.1099999999999</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1188,13 +1188,13 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="F14">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H14">
         <v>10</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1031.8049999999998</v>
+        <v>1049.76</v>
       </c>
       <c r="B15">
-        <v>-14.120000000000118</v>
+        <v>-4.5699999999999363</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1223,13 +1223,13 @@
         <v>28</v>
       </c>
       <c r="F15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J15" t="s">
         <v>49</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1030.809</v>
+        <v>1031.8049999999998</v>
       </c>
       <c r="B16">
-        <v>91.139999999999873</v>
+        <v>-14.120000000000118</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F16">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H16">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1030.3562499999998</v>
+        <v>1030.809</v>
       </c>
       <c r="B17">
-        <v>-28.230000000000018</v>
+        <v>91.139999999999873</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F17">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G17">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H17">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>986.87900000000013</v>
+        <v>982.26900000000012</v>
       </c>
       <c r="B19">
-        <v>47.210000000000036</v>
+        <v>42.600000000000023</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F19">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G19">
         <v>6</v>
       </c>
       <c r="H19">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>944.89900000000011</v>
+        <v>949.52900000000011</v>
       </c>
       <c r="B23">
-        <v>5.2300000000000182</v>
+        <v>9.8600000000000136</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F23">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G23">
         <v>3</v>
       </c>
       <c r="H23">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>906.21900000000005</v>
+        <v>889.33900000000006</v>
       </c>
       <c r="B25">
-        <v>-33.450000000000045</v>
+        <v>-50.330000000000041</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,16 +1540,16 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F25">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="G25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H25">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>895.80900000000008</v>
+        <v>887.14900000000011</v>
       </c>
       <c r="B26">
-        <v>-43.860000000000014</v>
+        <v>-52.519999999999982</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="F26">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="G26">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H26">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>803.15900000000011</v>
+        <v>810.29900000000009</v>
       </c>
       <c r="B28">
-        <v>-136.51</v>
+        <v>-129.37</v>
       </c>
       <c r="C28" t="s">
         <v>86</v>
@@ -1636,16 +1636,16 @@
         <v>87</v>
       </c>
       <c r="E28">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F28">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G28">
         <v>2</v>
       </c>
       <c r="H28">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update: Ranking Data (02:00:01)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3EFEE5E0-2575-4F46-AE03-B6AACA6806B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1B7E0E4-812A-4055-8C62-C3EB9AD6F907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1768" yWindow="2082" windowWidth="32621" windowHeight="17608" xr2:uid="{9676FA2C-4EB3-4B76-AA59-6F1E23D3AFD2}"/>
+    <workbookView xWindow="1768" yWindow="2082" windowWidth="32621" windowHeight="17608" xr2:uid="{20519112-9074-4D2A-9A8C-8BD536F29D64}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B4FFAB-8F37-46E9-8E6C-762D6515ECE3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92374BCD-EE1C-45C5-B91D-C5B32C7E718A}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (02:05:34)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1B7E0E4-812A-4055-8C62-C3EB9AD6F907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{220126F8-60E9-4B73-BE88-1D2EC0F220F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1768" yWindow="2082" windowWidth="32621" windowHeight="17608" xr2:uid="{20519112-9074-4D2A-9A8C-8BD536F29D64}"/>
+    <workbookView xWindow="1768" yWindow="2082" windowWidth="32621" windowHeight="17608" xr2:uid="{FBE25928-4B1C-472D-A332-8AB790EDD3DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92374BCD-EE1C-45C5-B91D-C5B32C7E718A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D63FD46F-5F57-4600-B694-F043849C44AC}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (06:57:59)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{220126F8-60E9-4B73-BE88-1D2EC0F220F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73E9B6F2-C23B-4392-B2E1-A893B58ADF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1768" yWindow="2082" windowWidth="32621" windowHeight="17608" xr2:uid="{FBE25928-4B1C-472D-A332-8AB790EDD3DD}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{09FF4F8B-D57F-446B-9BC0-1E1CE2E346EB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D63FD46F-5F57-4600-B694-F043849C44AC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B26FDF8-99EB-40B3-AE6B-E05AA5B6B389}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (06:58:56)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73E9B6F2-C23B-4392-B2E1-A893B58ADF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{813DA5A0-B6BB-481F-A21A-E69F37B430D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{09FF4F8B-D57F-446B-9BC0-1E1CE2E346EB}"/>
+    <workbookView xWindow="356" yWindow="356" windowWidth="27346" windowHeight="14928" xr2:uid="{BD68F837-4A2D-445D-8E00-A03B39CC34B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B26FDF8-99EB-40B3-AE6B-E05AA5B6B389}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE5715B8-2D1B-47A9-9C2B-7F6756B04028}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (07:30:03)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{813DA5A0-B6BB-481F-A21A-E69F37B430D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8549F57-1C77-4EF7-B3D3-56EB0927AF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="356" yWindow="356" windowWidth="27346" windowHeight="14928" xr2:uid="{BD68F837-4A2D-445D-8E00-A03B39CC34B3}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{4BC53C65-DFDC-44D7-859D-6D6B67016694}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE5715B8-2D1B-47A9-9C2B-7F6756B04028}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200DCEA8-5AE5-46EE-AFAA-32B988C5E55D}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (00:31:17)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8549F57-1C77-4EF7-B3D3-56EB0927AF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41427845-26B3-46A4-B4BE-0F91EED1EDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{4BC53C65-DFDC-44D7-859D-6D6B67016694}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{87415DE7-BE76-4953-974A-988ECEBD5C5D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,34 +134,43 @@
     <t>전체 합계</t>
   </si>
   <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>방덕</t>
+  </si>
+  <si>
+    <t>인테르</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>3부리그</t>
+  </si>
+  <si>
     <t>콩콩콩룔</t>
   </si>
   <si>
     <t>라치오</t>
   </si>
   <si>
-    <t>방덕</t>
-  </si>
-  <si>
-    <t>인테르</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
-    <t>3부리그</t>
+    <t>FA컵_결승전</t>
   </si>
   <si>
     <t>호야국2인</t>
@@ -170,7 +179,7 @@
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>FA컵_결승전</t>
+    <t>FA컵_4강</t>
   </si>
   <si>
     <t>오스트리아</t>
@@ -179,7 +188,7 @@
     <t>마인츠</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
+    <t>FA컵_8강</t>
   </si>
   <si>
     <t>Special블루</t>
@@ -188,7 +197,7 @@
     <t>아스널</t>
   </si>
   <si>
-    <t>FA컵_8강</t>
+    <t>FA컵_16강</t>
   </si>
   <si>
     <t>아들러</t>
@@ -197,15 +206,6 @@
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>FA컵_16강</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
     <t>FA컵_32강</t>
   </si>
   <si>
@@ -236,21 +236,21 @@
     <t>UCL_4강</t>
   </si>
   <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>UCL_8강</t>
+  </si>
+  <si>
     <t>경남FC가즈아</t>
   </si>
   <si>
     <t>경남 FC</t>
   </si>
   <si>
-    <t>UCL_8강</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
-  </si>
-  <si>
     <t>UEL_FINAL</t>
   </si>
   <si>
@@ -272,19 +272,19 @@
     <t>UEL_8강</t>
   </si>
   <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
     <t>A지냐크</t>
   </si>
   <si>
     <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
   </si>
   <si>
     <t>UECL_4강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{200DCEA8-5AE5-46EE-AFAA-32B988C5E55D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8249E765-D6FD-4DCA-9444-6AA958C247F6}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1274.8400000000001</v>
+        <v>1293.1500000000001</v>
       </c>
       <c r="B3">
-        <v>217.37000000000012</v>
+        <v>235.68000000000006</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -770,10 +770,10 @@
         <v>12</v>
       </c>
       <c r="E3">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F3">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3">
         <v>4</v>
@@ -829,13 +829,13 @@
         <v>18</v>
       </c>
       <c r="K4">
-        <v>51.3</v>
+        <v>69.61</v>
       </c>
       <c r="L4">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N4">
         <v>1</v>
@@ -1005,13 +1005,13 @@
         <v>30</v>
       </c>
       <c r="K8">
-        <v>217.37</v>
+        <v>235.68</v>
       </c>
       <c r="L8">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="N8">
         <v>4</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1106.2774999999999</v>
+        <v>1105.739</v>
       </c>
       <c r="B9">
-        <v>89.42999999999995</v>
+        <v>166.06999999999994</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1034,13 +1034,13 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F9">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H9">
         <v>11</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1060.77125</v>
+        <v>1073.0374999999999</v>
       </c>
       <c r="B13">
-        <v>30.5</v>
+        <v>56.189999999999941</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,13 +1156,13 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F13">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13">
         <v>13</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1056.4762499999999</v>
+        <v>1060.77125</v>
       </c>
       <c r="B14">
-        <v>-2.1099999999999</v>
+        <v>30.5</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1188,16 +1188,16 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="F14">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G14">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J14" t="s">
         <v>46</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1049.76</v>
+        <v>1056.4762499999999</v>
       </c>
       <c r="B15">
-        <v>-4.5699999999999363</v>
+        <v>-2.1099999999999</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1220,13 +1220,13 @@
         <v>48</v>
       </c>
       <c r="E15">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="F15">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H15">
         <v>10</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1031.8049999999998</v>
+        <v>1049.76</v>
       </c>
       <c r="B16">
-        <v>-14.120000000000118</v>
+        <v>-4.5699999999999363</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1255,13 +1255,13 @@
         <v>28</v>
       </c>
       <c r="F16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H16">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1030.809</v>
+        <v>1031.8049999999998</v>
       </c>
       <c r="B17">
-        <v>91.139999999999873</v>
+        <v>-14.120000000000118</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F17">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="G17">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1336,10 +1336,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>982.26900000000012</v>
+        <v>980.69900000000007</v>
       </c>
       <c r="B19">
-        <v>42.600000000000023</v>
+        <v>41.029999999999973</v>
       </c>
       <c r="C19" t="s">
         <v>59</v>
@@ -1348,16 +1348,16 @@
         <v>60</v>
       </c>
       <c r="E19">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F19">
         <v>18</v>
       </c>
       <c r="G19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H19">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J19" t="s">
         <v>61</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>969.67124999999987</v>
+        <v>972.31999999999994</v>
       </c>
       <c r="B21">
-        <v>11.039999999999964</v>
+        <v>-10.009999999999991</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="F21">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G21">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>954.3599999999999</v>
+        <v>969.67124999999987</v>
       </c>
       <c r="B22">
-        <v>-27.970000000000027</v>
+        <v>11.039999999999964</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,16 +1444,16 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F22">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J22" t="s">
         <v>70</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>889.33900000000006</v>
+        <v>887.14900000000011</v>
       </c>
       <c r="B25">
-        <v>-50.330000000000041</v>
+        <v>-52.519999999999982</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,16 +1540,16 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F25">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="G25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H25">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>887.14900000000011</v>
+        <v>881.87900000000013</v>
       </c>
       <c r="B26">
-        <v>-52.519999999999982</v>
+        <v>-57.789999999999964</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1572,16 +1572,16 @@
         <v>81</v>
       </c>
       <c r="E26">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F26">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H26">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Update: Ranking Data (00:43:05)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41427845-26B3-46A4-B4BE-0F91EED1EDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4135F8BA-D1B8-4119-BE38-2EACA767D189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{87415DE7-BE76-4953-974A-988ECEBD5C5D}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{5A463113-C7F5-4DCB-BE93-2EEC3B57523A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8249E765-D6FD-4DCA-9444-6AA958C247F6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69331036-931E-4024-BA9F-F5E89B8652D3}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (00:45:43)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4135F8BA-D1B8-4119-BE38-2EACA767D189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF13DED5-9476-4A4D-91DB-FDC1D629C09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{5A463113-C7F5-4DCB-BE93-2EEC3B57523A}"/>
+    <workbookView xWindow="1682" yWindow="1654" windowWidth="27731" windowHeight="17394" xr2:uid="{4BB37996-E190-46DF-BF1C-FCCF79CC5FCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69331036-931E-4024-BA9F-F5E89B8652D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1CF9C09-4342-4DCB-86DC-8483EE765F37}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (01:05:33)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF13DED5-9476-4A4D-91DB-FDC1D629C09F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFE19ABA-1B83-4735-BFF3-7BC89C54A325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1682" yWindow="1654" windowWidth="27731" windowHeight="17394" xr2:uid="{4BB37996-E190-46DF-BF1C-FCCF79CC5FCF}"/>
+    <workbookView xWindow="1682" yWindow="1654" windowWidth="27731" windowHeight="17394" xr2:uid="{81ADA542-DD6E-448B-A562-CA57ACBE94F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1CF9C09-4342-4DCB-86DC-8483EE765F37}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A4DD104-89F7-466C-807F-25871C27FB15}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (03:50:15)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFE19ABA-1B83-4735-BFF3-7BC89C54A325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D60644C-7284-4C41-9E33-3F47EC8467C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1682" yWindow="1654" windowWidth="27731" windowHeight="17394" xr2:uid="{81ADA542-DD6E-448B-A562-CA57ACBE94F6}"/>
+    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{A674F3CD-1D97-45A0-91EA-38392124A88B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,21 +65,27 @@
     <t>패</t>
   </si>
   <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
     <t>개포동덕배</t>
   </si>
   <si>
     <t>바이에른 뮌헨</t>
   </si>
   <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>17시즌</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
-  </si>
-  <si>
     <t>대회종류</t>
   </si>
   <si>
@@ -95,34 +101,94 @@
     <t>첼시</t>
   </si>
   <si>
+    <t>3부리그</t>
+  </si>
+  <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>AS 로마</t>
+  </si>
+  <si>
+    <t>FA컵</t>
+  </si>
+  <si>
+    <t>ZD장인지참치</t>
+  </si>
+  <si>
+    <t>레버쿠젠</t>
+  </si>
+  <si>
+    <t>UEFA_A조</t>
+  </si>
+  <si>
+    <t>UEL</t>
+  </si>
+  <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>호야국2인</t>
+  </si>
+  <si>
+    <t>SSC 나폴리</t>
+  </si>
+  <si>
     <t>1부리그</t>
   </si>
   <si>
-    <t>UNIT</t>
-  </si>
-  <si>
-    <t>AS 로마</t>
-  </si>
-  <si>
-    <t>FA컵</t>
-  </si>
-  <si>
-    <t>ZD장인지참치</t>
-  </si>
-  <si>
-    <t>레버쿠젠</t>
-  </si>
-  <si>
-    <t>UEFA_B조</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>UCL</t>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
+    <t>FA컵_결승전</t>
+  </si>
+  <si>
+    <t>아들러</t>
+  </si>
+  <si>
+    <t>프랑크푸르트</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>FA컵_8강</t>
   </si>
   <si>
     <t>피파왕초보구단주</t>
@@ -131,13 +197,7 @@
     <t>리버풀</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
+    <t>FA컵_16강</t>
   </si>
   <si>
     <t>방덕</t>
@@ -146,13 +206,7 @@
     <t>인테르</t>
   </si>
   <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
-  </si>
-  <si>
-    <t>2부리그</t>
+    <t>FA컵_32강</t>
   </si>
   <si>
     <t>은안</t>
@@ -161,60 +215,6 @@
     <t>맨체스터 시티</t>
   </si>
   <si>
-    <t>3부리그</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
-    <t>FA컵_결승전</t>
-  </si>
-  <si>
-    <t>호야국2인</t>
-  </si>
-  <si>
-    <t>SSC 나폴리</t>
-  </si>
-  <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
-    <t>FA컵_8강</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>FA컵_16강</t>
-  </si>
-  <si>
-    <t>아들러</t>
-  </si>
-  <si>
-    <t>프랑크푸르트</t>
-  </si>
-  <si>
-    <t>FA컵_32강</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
     <t>UEFA</t>
   </si>
   <si>
@@ -254,46 +254,46 @@
     <t>UEL_FINAL</t>
   </si>
   <si>
+    <t>Legend독수리</t>
+  </si>
+  <si>
+    <t>맨체스터 유나이티드</t>
+  </si>
+  <si>
+    <t>UEL_4강</t>
+  </si>
+  <si>
+    <t>suma수마</t>
+  </si>
+  <si>
+    <t>ACF 피오렌티나</t>
+  </si>
+  <si>
+    <t>UEL_8강</t>
+  </si>
+  <si>
+    <t>A지냐크</t>
+  </si>
+  <si>
+    <t>올랭피크 마르세유</t>
+  </si>
+  <si>
+    <t>UECL_FINAL</t>
+  </si>
+  <si>
+    <t>syma</t>
+  </si>
+  <si>
+    <t>RC 셀타 비고</t>
+  </si>
+  <si>
+    <t>UECL_4강</t>
+  </si>
+  <si>
     <t>여수가스</t>
   </si>
   <si>
     <t>AS 모나코</t>
-  </si>
-  <si>
-    <t>UEL_4강</t>
-  </si>
-  <si>
-    <t>Legend독수리</t>
-  </si>
-  <si>
-    <t>맨체스터 유나이티드</t>
-  </si>
-  <si>
-    <t>UEL_8강</t>
-  </si>
-  <si>
-    <t>suma수마</t>
-  </si>
-  <si>
-    <t>ACF 피오렌티나</t>
-  </si>
-  <si>
-    <t>UECL_FINAL</t>
-  </si>
-  <si>
-    <t>A지냐크</t>
-  </si>
-  <si>
-    <t>올랭피크 마르세유</t>
-  </si>
-  <si>
-    <t>UECL_4강</t>
-  </si>
-  <si>
-    <t>syma</t>
-  </si>
-  <si>
-    <t>RC 셀타 비고</t>
   </si>
   <si>
     <t>UECL_8강</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A4DD104-89F7-466C-807F-25871C27FB15}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88541D0B-1253-4E1B-A6B2-08E71476ED59}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1307.7962500000001</v>
+        <v>1309.51</v>
       </c>
       <c r="B2">
-        <v>171.67000000000007</v>
+        <v>252.03999999999996</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -735,16 +735,16 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F2">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -758,37 +758,37 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1293.1500000000001</v>
+        <v>1307.7962500000001</v>
       </c>
       <c r="B3">
-        <v>235.68000000000006</v>
+        <v>171.67000000000007</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F3">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="L3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M3" t="s">
         <v>5</v>
@@ -808,10 +808,10 @@
         <v>123.01999999999998</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4">
         <v>32</v>
@@ -826,22 +826,22 @@
         <v>9</v>
       </c>
       <c r="J4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K4">
-        <v>69.61</v>
+        <v>1.629999999999999</v>
       </c>
       <c r="L4">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="M4">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="N4">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O4">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
@@ -852,10 +852,10 @@
         <v>208.82999999999993</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5">
         <v>35</v>
@@ -870,19 +870,19 @@
         <v>10</v>
       </c>
       <c r="J5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K5">
-        <v>-23.09</v>
+        <v>43.269999999999996</v>
       </c>
       <c r="L5">
+        <v>4</v>
+      </c>
+      <c r="M5">
+        <v>2</v>
+      </c>
+      <c r="N5">
         <v>1</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
       </c>
       <c r="O5">
         <v>1</v>
@@ -896,10 +896,10 @@
         <v>240.94000000000005</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>51</v>
@@ -914,22 +914,22 @@
         <v>16</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K6">
-        <v>80.97</v>
+        <v>35.20000000000001</v>
       </c>
       <c r="L6">
         <v>12</v>
       </c>
       <c r="M6">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
@@ -940,10 +940,10 @@
         <v>182.97000000000003</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="E7">
         <v>52</v>
@@ -961,27 +961,27 @@
         <v>27</v>
       </c>
       <c r="K7">
-        <v>108.19</v>
+        <v>102.87</v>
       </c>
       <c r="L7">
+        <v>10</v>
+      </c>
+      <c r="M7">
         <v>6</v>
       </c>
-      <c r="M7">
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
         <v>4</v>
-      </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
-      <c r="O7">
-        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1115.9450000000002</v>
+        <v>1105.739</v>
       </c>
       <c r="B8">
-        <v>50.940000000000055</v>
+        <v>166.06999999999994</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -990,42 +990,42 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F8">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H8">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J8" t="s">
         <v>30</v>
       </c>
       <c r="K8">
-        <v>235.68</v>
+        <v>182.97</v>
       </c>
       <c r="L8">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="M8">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="O8">
-        <v>7</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1105.739</v>
+        <v>1093.0425</v>
       </c>
       <c r="B9">
-        <v>166.06999999999994</v>
+        <v>92.420000000000073</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1034,24 +1034,24 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F9">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G9">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1095.0862499999998</v>
+        <v>1060.77125</v>
       </c>
       <c r="B10">
-        <v>61.769999999999982</v>
+        <v>30.5</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1060,19 +1060,19 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F10">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J10" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="K10">
         <v>2</v>
@@ -1080,31 +1080,31 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1093.0425</v>
+        <v>1056.4762499999999</v>
       </c>
       <c r="B11">
-        <v>92.420000000000073</v>
+        <v>-2.1099999999999</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E11">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G11">
+        <v>7</v>
+      </c>
+      <c r="H11">
         <v>10</v>
       </c>
-      <c r="H11">
-        <v>7</v>
-      </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -1112,31 +1112,31 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1086.8699999999999</v>
+        <v>1049.76</v>
       </c>
       <c r="B12">
-        <v>36.490000000000009</v>
+        <v>-4.5699999999999363</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E12">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F12">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J12" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="K12">
         <v>0.3</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1073.0374999999999</v>
+        <v>1036.7275</v>
       </c>
       <c r="B13">
-        <v>56.189999999999941</v>
+        <v>19.879999999999995</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,7 +1156,7 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F13">
         <v>10</v>
@@ -1165,7 +1165,7 @@
         <v>4</v>
       </c>
       <c r="H13">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J13" t="s">
         <v>43</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1060.77125</v>
+        <v>1031.8049999999998</v>
       </c>
       <c r="B14">
-        <v>30.5</v>
+        <v>-14.120000000000118</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1188,16 +1188,16 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F14">
+        <v>13</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
         <v>14</v>
-      </c>
-      <c r="G14">
-        <v>3</v>
-      </c>
-      <c r="H14">
-        <v>13</v>
       </c>
       <c r="J14" t="s">
         <v>46</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1056.4762499999999</v>
+        <v>1025.3690000000001</v>
       </c>
       <c r="B15">
-        <v>-2.1099999999999</v>
+        <v>85.700000000000045</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1220,16 +1220,16 @@
         <v>48</v>
       </c>
       <c r="E15">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F15">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G15">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H15">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J15" t="s">
         <v>49</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1049.76</v>
+        <v>999.84500000000014</v>
       </c>
       <c r="B16">
-        <v>-4.5699999999999363</v>
+        <v>-65.159999999999968</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1252,16 +1252,16 @@
         <v>51</v>
       </c>
       <c r="E16">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F16">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G16">
         <v>4</v>
       </c>
       <c r="H16">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J16" t="s">
         <v>52</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>1031.8049999999998</v>
+        <v>995.08624999999984</v>
       </c>
       <c r="B17">
-        <v>-14.120000000000118</v>
+        <v>-38.230000000000018</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1287,13 +1287,13 @@
         <v>28</v>
       </c>
       <c r="F17">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>987.35900000000015</v>
+        <v>986.86999999999989</v>
       </c>
       <c r="B18">
-        <v>47.690000000000055</v>
+        <v>-63.509999999999991</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,13 +1316,13 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F18">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H18">
         <v>13</v>
@@ -1464,10 +1464,10 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>949.52900000000011</v>
+        <v>924.23124999999993</v>
       </c>
       <c r="B23">
-        <v>9.8600000000000136</v>
+        <v>-21.210000000000036</v>
       </c>
       <c r="C23" t="s">
         <v>71</v>
@@ -1476,16 +1476,16 @@
         <v>72</v>
       </c>
       <c r="E23">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F23">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H23">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="J23" t="s">
         <v>73</v>
@@ -1496,10 +1496,10 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>924.23124999999993</v>
+        <v>887.14900000000011</v>
       </c>
       <c r="B24">
-        <v>-21.210000000000036</v>
+        <v>-52.519999999999982</v>
       </c>
       <c r="C24" t="s">
         <v>74</v>
@@ -1511,13 +1511,13 @@
         <v>41</v>
       </c>
       <c r="F24">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="G24">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H24">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="J24" t="s">
         <v>76</v>
@@ -1528,10 +1528,10 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>887.14900000000011</v>
+        <v>881.87900000000013</v>
       </c>
       <c r="B25">
-        <v>-52.519999999999982</v>
+        <v>-57.789999999999964</v>
       </c>
       <c r="C25" t="s">
         <v>77</v>
@@ -1540,16 +1540,16 @@
         <v>78</v>
       </c>
       <c r="E25">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F25">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H25">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="J25" t="s">
         <v>79</v>
@@ -1560,10 +1560,10 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>881.87900000000013</v>
+        <v>878.62900000000013</v>
       </c>
       <c r="B26">
-        <v>-57.789999999999964</v>
+        <v>-61.039999999999964</v>
       </c>
       <c r="C26" t="s">
         <v>80</v>
@@ -1575,13 +1575,13 @@
         <v>42</v>
       </c>
       <c r="F26">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G26">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H26">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="J26" t="s">
         <v>82</v>
@@ -1592,10 +1592,10 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>878.62900000000013</v>
+        <v>849.52900000000011</v>
       </c>
       <c r="B27">
-        <v>-61.039999999999964</v>
+        <v>-90.139999999999986</v>
       </c>
       <c r="C27" t="s">
         <v>83</v>
@@ -1607,13 +1607,13 @@
         <v>42</v>
       </c>
       <c r="F27">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="G27">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H27">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="J27" t="s">
         <v>85</v>

</xml_diff>

<commit_message>
Update: Ranking Data (04:38:30)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D60644C-7284-4C41-9E33-3F47EC8467C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{91FE6571-A532-471C-B18D-07D4E82D07F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{A674F3CD-1D97-45A0-91EA-38392124A88B}"/>
+    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{460371F5-EBBF-4E6E-9B27-479AF86DA384}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88541D0B-1253-4E1B-A6B2-08E71476ED59}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30FAB3D7-57E5-4865-BF88-442B0077FFF3}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (06:04:38)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91FE6571-A532-471C-B18D-07D4E82D07F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{52223723-A456-414C-BF8D-800D685C31C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{460371F5-EBBF-4E6E-9B27-479AF86DA384}"/>
+    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{54557B03-EE8B-47A7-87C5-407FDEEBFCCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30FAB3D7-57E5-4865-BF88-442B0077FFF3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB793AB5-7805-4470-A678-526A90488609}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (08:55:12)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52223723-A456-414C-BF8D-800D685C31C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2B166FD-6F69-49A5-884F-E7B29C36FDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{54557B03-EE8B-47A7-87C5-407FDEEBFCCD}"/>
+    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{FEECBC2E-2D2E-4C41-84E8-7D9B6B8C83F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB793AB5-7805-4470-A678-526A90488609}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D533A24A-9D90-4F0A-85B8-3A262BC00203}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (10:06:51)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2B166FD-6F69-49A5-884F-E7B29C36FDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BF895E1-4652-4224-81FF-9B7419BB3CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{FEECBC2E-2D2E-4C41-84E8-7D9B6B8C83F4}"/>
+    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{C7F7136F-CF96-461D-985D-0745AB93D31E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,27 +65,27 @@
     <t>패</t>
   </si>
   <si>
+    <t>개포동덕배</t>
+  </si>
+  <si>
+    <t>바이에른 뮌헨</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
     <t>검정소</t>
   </si>
   <si>
     <t>AC 밀란</t>
   </si>
   <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>17시즌</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>개포동덕배</t>
-  </si>
-  <si>
-    <t>바이에른 뮌헨</t>
-  </si>
-  <si>
     <t>대회종류</t>
   </si>
   <si>
@@ -125,19 +125,28 @@
     <t>UEL</t>
   </si>
   <si>
+    <t>앙쿠</t>
+  </si>
+  <si>
+    <t>아틀레티코 마드리드</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>0708ManUtd</t>
   </si>
   <si>
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>앙쿠</t>
-  </si>
-  <si>
-    <t>아틀레티코 마드리드</t>
+    <t>오스트리아</t>
+  </si>
+  <si>
+    <t>마인츠</t>
+  </si>
+  <si>
+    <t>1부리그</t>
   </si>
   <si>
     <t>호야국2인</t>
@@ -146,15 +155,6 @@
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>오스트리아</t>
-  </si>
-  <si>
-    <t>마인츠</t>
-  </si>
-  <si>
     <t>2부리그</t>
   </si>
   <si>
@@ -173,31 +173,40 @@
     <t>FA컵_결승전</t>
   </si>
   <si>
+    <t>비주류중독</t>
+  </si>
+  <si>
+    <t>셀틱 FC</t>
+  </si>
+  <si>
+    <t>FA컵_4강</t>
+  </si>
+  <si>
     <t>아들러</t>
   </si>
   <si>
     <t>프랑크푸르트</t>
   </si>
   <si>
-    <t>FA컵_4강</t>
-  </si>
-  <si>
-    <t>비주류중독</t>
-  </si>
-  <si>
-    <t>셀틱 FC</t>
-  </si>
-  <si>
     <t>FA컵_8강</t>
   </si>
   <si>
+    <t>은안</t>
+  </si>
+  <si>
+    <t>맨체스터 시티</t>
+  </si>
+  <si>
+    <t>FA컵_16강</t>
+  </si>
+  <si>
     <t>피파왕초보구단주</t>
   </si>
   <si>
     <t>리버풀</t>
   </si>
   <si>
-    <t>FA컵_16강</t>
+    <t>FA컵_32강</t>
   </si>
   <si>
     <t>방덕</t>
@@ -206,15 +215,6 @@
     <t>인테르</t>
   </si>
   <si>
-    <t>FA컵_32강</t>
-  </si>
-  <si>
-    <t>은안</t>
-  </si>
-  <si>
-    <t>맨체스터 시티</t>
-  </si>
-  <si>
     <t>UEFA</t>
   </si>
   <si>
@@ -236,19 +236,19 @@
     <t>UCL_4강</t>
   </si>
   <si>
+    <t>경남FC가즈아</t>
+  </si>
+  <si>
+    <t>경남 FC</t>
+  </si>
+  <si>
+    <t>UCL_8강</t>
+  </si>
+  <si>
     <t>Gucci와퍼</t>
   </si>
   <si>
     <t>함부르크SV</t>
-  </si>
-  <si>
-    <t>UCL_8강</t>
-  </si>
-  <si>
-    <t>경남FC가즈아</t>
-  </si>
-  <si>
-    <t>경남 FC</t>
   </si>
   <si>
     <t>UEL_FINAL</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D533A24A-9D90-4F0A-85B8-3A262BC00203}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{556A9437-9B4F-49FF-9D71-3027033186BD}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1309.51</v>
+        <v>1339.0762500000001</v>
       </c>
       <c r="B2">
-        <v>252.03999999999996</v>
+        <v>202.95000000000005</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -738,13 +738,13 @@
         <v>31</v>
       </c>
       <c r="F2">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1307.7962500000001</v>
+        <v>1309.51</v>
       </c>
       <c r="B3">
-        <v>171.67000000000007</v>
+        <v>252.03999999999996</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,16 +770,16 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F3">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1122.6390000000001</v>
+        <v>1132.0390000000002</v>
       </c>
       <c r="B7">
-        <v>182.97000000000003</v>
+        <v>192.37000000000012</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -946,13 +946,13 @@
         <v>12</v>
       </c>
       <c r="E7">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F7">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H7">
         <v>17</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1105.739</v>
+        <v>1093.0425</v>
       </c>
       <c r="B8">
-        <v>166.06999999999994</v>
+        <v>92.420000000000073</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -990,16 +990,16 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F8">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H8">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="J8" t="s">
         <v>30</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1093.0425</v>
+        <v>1091.7190000000001</v>
       </c>
       <c r="B9">
-        <v>92.420000000000073</v>
+        <v>152.04999999999995</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1034,24 +1034,24 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F9">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G9">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1060.77125</v>
+        <v>1088.3062499999999</v>
       </c>
       <c r="B10">
-        <v>30.5</v>
+        <v>29.720000000000027</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1060,16 +1060,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="F10">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H10">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J10" t="s">
         <v>35</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1056.4762499999999</v>
+        <v>1052.1212499999999</v>
       </c>
       <c r="B11">
-        <v>-2.1099999999999</v>
+        <v>21.849999999999909</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1092,16 +1092,16 @@
         <v>37</v>
       </c>
       <c r="E11">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="F11">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G11">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J11" t="s">
         <v>38</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>1031.8049999999998</v>
+        <v>1025.3690000000001</v>
       </c>
       <c r="B14">
-        <v>-14.120000000000118</v>
+        <v>85.700000000000045</v>
       </c>
       <c r="C14" t="s">
         <v>44</v>
@@ -1188,16 +1188,16 @@
         <v>45</v>
       </c>
       <c r="E14">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F14">
+        <v>14</v>
+      </c>
+      <c r="G14">
+        <v>4</v>
+      </c>
+      <c r="H14">
         <v>13</v>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-      <c r="H14">
-        <v>14</v>
       </c>
       <c r="J14" t="s">
         <v>46</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1025.3690000000001</v>
+        <v>1014.125</v>
       </c>
       <c r="B15">
-        <v>85.700000000000045</v>
+        <v>-31.799999999999955</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1220,16 +1220,16 @@
         <v>48</v>
       </c>
       <c r="E15">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F15">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J15" t="s">
         <v>49</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>999.84500000000014</v>
+        <v>1005.3499999999999</v>
       </c>
       <c r="B16">
-        <v>-65.159999999999968</v>
+        <v>-45.029999999999973</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1272,10 +1272,10 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>995.08624999999984</v>
+        <v>999.84500000000014</v>
       </c>
       <c r="B17">
-        <v>-38.230000000000018</v>
+        <v>-65.159999999999968</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1284,16 +1284,16 @@
         <v>54</v>
       </c>
       <c r="E17">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H17">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
@@ -1304,10 +1304,10 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>986.86999999999989</v>
+        <v>995.08624999999984</v>
       </c>
       <c r="B18">
-        <v>-63.509999999999991</v>
+        <v>-38.230000000000018</v>
       </c>
       <c r="C18" t="s">
         <v>56</v>
@@ -1316,16 +1316,16 @@
         <v>57</v>
       </c>
       <c r="E18">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F18">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="J18" t="s">
         <v>58</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>972.31999999999994</v>
+        <v>969.67124999999987</v>
       </c>
       <c r="B21">
-        <v>-10.009999999999991</v>
+        <v>11.039999999999964</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="F21">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H21">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>969.67124999999987</v>
+        <v>949.86999999999989</v>
       </c>
       <c r="B22">
-        <v>11.039999999999964</v>
+        <v>-32.460000000000036</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,13 +1444,13 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F22">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="G22">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H22">
         <v>18</v>

</xml_diff>

<commit_message>
Update: Ranking Data (00:26:16)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BF895E1-4652-4224-81FF-9B7419BB3CC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C60C7DE5-3CD4-49EA-88DB-E394178E6953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2025" yWindow="1996" windowWidth="27730" windowHeight="17394" xr2:uid="{C7F7136F-CF96-461D-985D-0745AB93D31E}"/>
+    <workbookView xWindow="2367" yWindow="2338" windowWidth="27730" windowHeight="17394" xr2:uid="{890FF290-3363-4CD1-804D-E4DB9707BDD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,25 +65,25 @@
     <t>패</t>
   </si>
   <si>
+    <t>검정소</t>
+  </si>
+  <si>
+    <t>AC 밀란</t>
+  </si>
+  <si>
+    <t>셀래스틴</t>
+  </si>
+  <si>
+    <t>17시즌</t>
+  </si>
+  <si>
+    <t>바르셀로나</t>
+  </si>
+  <si>
     <t>개포동덕배</t>
   </si>
   <si>
     <t>바이에른 뮌헨</t>
-  </si>
-  <si>
-    <t>셀래스틴</t>
-  </si>
-  <si>
-    <t>17시즌</t>
-  </si>
-  <si>
-    <t>바르셀로나</t>
-  </si>
-  <si>
-    <t>검정소</t>
-  </si>
-  <si>
-    <t>AC 밀란</t>
   </si>
   <si>
     <t>대회종류</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{556A9437-9B4F-49FF-9D71-3027033186BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C488C999-3675-48A8-9ECF-2880DB74C818}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -723,10 +723,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1339.0762500000001</v>
+        <v>1415.45</v>
       </c>
       <c r="B2">
-        <v>202.95000000000005</v>
+        <v>357.98</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -735,16 +735,16 @@
         <v>9</v>
       </c>
       <c r="E2">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F2">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J2" t="s">
         <v>10</v>
@@ -758,10 +758,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1309.51</v>
+        <v>1362.7462500000001</v>
       </c>
       <c r="B3">
-        <v>252.03999999999996</v>
+        <v>226.62000000000012</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
@@ -770,16 +770,16 @@
         <v>14</v>
       </c>
       <c r="E3">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="F3">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J3" t="s">
         <v>15</v>
@@ -846,10 +846,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>1247.6299999999999</v>
+        <v>1236.75</v>
       </c>
       <c r="B5">
-        <v>208.82999999999993</v>
+        <v>197.95000000000005</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -858,7 +858,7 @@
         <v>22</v>
       </c>
       <c r="E5">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F5">
         <v>18</v>
@@ -867,7 +867,7 @@
         <v>7</v>
       </c>
       <c r="H5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J5" t="s">
         <v>23</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1132.0390000000002</v>
+        <v>1131.8690000000001</v>
       </c>
       <c r="B7">
-        <v>192.37000000000012</v>
+        <v>192.20000000000005</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1091.7190000000001</v>
+        <v>1091.269</v>
       </c>
       <c r="B9">
-        <v>152.04999999999995</v>
+        <v>151.59999999999991</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1048,10 +1048,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1088.3062499999999</v>
+        <v>1088.9362499999997</v>
       </c>
       <c r="B10">
-        <v>29.720000000000027</v>
+        <v>30.349999999999909</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1052.1212499999999</v>
+        <v>1051.9512500000001</v>
       </c>
       <c r="B11">
-        <v>21.849999999999909</v>
+        <v>21.680000000000064</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1208,10 +1208,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>1014.125</v>
+        <v>1014.145</v>
       </c>
       <c r="B15">
-        <v>-31.799999999999955</v>
+        <v>-31.779999999999973</v>
       </c>
       <c r="C15" t="s">
         <v>47</v>
@@ -1240,10 +1240,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>1005.3499999999999</v>
+        <v>1005.3699999999999</v>
       </c>
       <c r="B16">
-        <v>-45.029999999999973</v>
+        <v>-45.009999999999991</v>
       </c>
       <c r="C16" t="s">
         <v>50</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>949.86999999999989</v>
+        <v>950.49999999999989</v>
       </c>
       <c r="B22">
-        <v>-32.460000000000036</v>
+        <v>-31.830000000000041</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>

</xml_diff>

<commit_message>
Update: Ranking Data (07:33:20)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C60C7DE5-3CD4-49EA-88DB-E394178E6953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE0D91C8-6031-4578-8E71-3C515D5ED594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2367" yWindow="2338" windowWidth="27730" windowHeight="17394" xr2:uid="{890FF290-3363-4CD1-804D-E4DB9707BDD1}"/>
+    <workbookView xWindow="770" yWindow="770" windowWidth="18506" windowHeight="17394" xr2:uid="{8C7C26D9-E3AC-4390-BC6B-3759828A1956}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -125,21 +125,21 @@
     <t>UEL</t>
   </si>
   <si>
+    <t>0708ManUtd</t>
+  </si>
+  <si>
+    <t>레알 마드리드</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>앙쿠</t>
   </si>
   <si>
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
-    <t>0708ManUtd</t>
-  </si>
-  <si>
-    <t>레알 마드리드</t>
-  </si>
-  <si>
     <t>오스트리아</t>
   </si>
   <si>
@@ -149,27 +149,27 @@
     <t>1부리그</t>
   </si>
   <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>2부리그</t>
+  </si>
+  <si>
+    <t>콩콩콩룔</t>
+  </si>
+  <si>
+    <t>라치오</t>
+  </si>
+  <si>
     <t>호야국2인</t>
   </si>
   <si>
     <t>SSC 나폴리</t>
   </si>
   <si>
-    <t>2부리그</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
-  </si>
-  <si>
-    <t>콩콩콩룔</t>
-  </si>
-  <si>
-    <t>라치오</t>
-  </si>
-  <si>
     <t>FA컵_결승전</t>
   </si>
   <si>
@@ -236,19 +236,19 @@
     <t>UCL_4강</t>
   </si>
   <si>
+    <t>Gucci와퍼</t>
+  </si>
+  <si>
+    <t>함부르크SV</t>
+  </si>
+  <si>
+    <t>UCL_8강</t>
+  </si>
+  <si>
     <t>경남FC가즈아</t>
   </si>
   <si>
     <t>경남 FC</t>
-  </si>
-  <si>
-    <t>UCL_8강</t>
-  </si>
-  <si>
-    <t>Gucci와퍼</t>
-  </si>
-  <si>
-    <t>함부르크SV</t>
   </si>
   <si>
     <t>UEL_FINAL</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C488C999-3675-48A8-9ECF-2880DB74C818}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E84CD286-230A-4194-B8ED-26908CF0EC2D}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1093.0425</v>
+        <v>1094.229</v>
       </c>
       <c r="B8">
-        <v>92.420000000000073</v>
+        <v>154.55999999999995</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -993,13 +993,13 @@
         <v>45</v>
       </c>
       <c r="F8">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G8">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H8">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="J8" t="s">
         <v>30</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1091.269</v>
+        <v>1093.0425</v>
       </c>
       <c r="B9">
-        <v>151.59999999999991</v>
+        <v>92.420000000000073</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1034,16 +1034,16 @@
         <v>32</v>
       </c>
       <c r="E9">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F9">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G9">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H9">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1051.9512500000001</v>
+        <v>1049.76</v>
       </c>
       <c r="B11">
-        <v>21.680000000000064</v>
+        <v>-4.5699999999999363</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1092,7 +1092,7 @@
         <v>37</v>
       </c>
       <c r="E11">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F11">
         <v>14</v>
@@ -1101,7 +1101,7 @@
         <v>4</v>
       </c>
       <c r="H11">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="J11" t="s">
         <v>38</v>
@@ -1112,10 +1112,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>1049.76</v>
+        <v>1036.7275</v>
       </c>
       <c r="B12">
-        <v>-4.5699999999999363</v>
+        <v>19.879999999999995</v>
       </c>
       <c r="C12" t="s">
         <v>39</v>
@@ -1124,16 +1124,16 @@
         <v>40</v>
       </c>
       <c r="E12">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G12">
         <v>4</v>
       </c>
       <c r="H12">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J12" t="s">
         <v>20</v>
@@ -1144,10 +1144,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1036.7275</v>
+        <v>1028.08125</v>
       </c>
       <c r="B13">
-        <v>19.879999999999995</v>
+        <v>-2.1900000000000546</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -1156,13 +1156,13 @@
         <v>42</v>
       </c>
       <c r="E13">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F13">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13">
         <v>15</v>
@@ -1400,10 +1400,10 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>969.67124999999987</v>
+        <v>972.59999999999991</v>
       </c>
       <c r="B21">
-        <v>11.039999999999964</v>
+        <v>-9.7300000000000182</v>
       </c>
       <c r="C21" t="s">
         <v>65</v>
@@ -1412,16 +1412,16 @@
         <v>66</v>
       </c>
       <c r="E21">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F21">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G21">
         <v>5</v>
       </c>
       <c r="H21">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J21" t="s">
         <v>67</v>
@@ -1432,10 +1432,10 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>950.49999999999989</v>
+        <v>969.67124999999987</v>
       </c>
       <c r="B22">
-        <v>-31.830000000000041</v>
+        <v>11.039999999999964</v>
       </c>
       <c r="C22" t="s">
         <v>68</v>
@@ -1444,13 +1444,13 @@
         <v>69</v>
       </c>
       <c r="E22">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="F22">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22">
         <v>18</v>

</xml_diff>

<commit_message>
Update: Ranking Data (07:39:54)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE0D91C8-6031-4578-8E71-3C515D5ED594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D49145E3-4CE1-4AED-B730-09E613344EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="770" yWindow="770" windowWidth="18506" windowHeight="17394" xr2:uid="{8C7C26D9-E3AC-4390-BC6B-3759828A1956}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{8A625F5B-4E9D-4693-AC2D-BC4D62782048}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E84CD286-230A-4194-B8ED-26908CF0EC2D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A615F7EA-9D4C-40D3-81D8-9EE380B493C9}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>

</xml_diff>

<commit_message>
Update: Ranking Data (10:07:15)
</commit_message>
<xml_diff>
--- a/Ranking_Data.xlsx
+++ b/Ranking_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\원영이\Desktop\ATL AUTO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D49145E3-4CE1-4AED-B730-09E613344EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7DA75066-A487-4738-96E3-5671D1098606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="36727" windowHeight="20317" xr2:uid="{8A625F5B-4E9D-4693-AC2D-BC4D62782048}"/>
+    <workbookView xWindow="4149" yWindow="1668" windowWidth="18506" windowHeight="17394" xr2:uid="{0D9238CE-65E1-4267-A2C6-2DE6C9755778}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -125,34 +125,34 @@
     <t>UEL</t>
   </si>
   <si>
+    <t>Special블루</t>
+  </si>
+  <si>
+    <t>아스널</t>
+  </si>
+  <si>
+    <t>전체 합계</t>
+  </si>
+  <si>
     <t>0708ManUtd</t>
   </si>
   <si>
     <t>레알 마드리드</t>
   </si>
   <si>
-    <t>전체 합계</t>
-  </si>
-  <si>
     <t>앙쿠</t>
   </si>
   <si>
     <t>아틀레티코 마드리드</t>
   </si>
   <si>
+    <t>1부리그</t>
+  </si>
+  <si>
     <t>오스트리아</t>
   </si>
   <si>
     <t>마인츠</t>
-  </si>
-  <si>
-    <t>1부리그</t>
-  </si>
-  <si>
-    <t>Special블루</t>
-  </si>
-  <si>
-    <t>아스널</t>
   </si>
   <si>
     <t>2부리그</t>
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A615F7EA-9D4C-40D3-81D8-9EE380B493C9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC00202-7C98-4136-9451-EDC4E35715DB}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15.7" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -978,10 +978,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>1094.229</v>
+        <v>1119.08</v>
       </c>
       <c r="B8">
-        <v>154.55999999999995</v>
+        <v>64.75</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -990,16 +990,16 @@
         <v>29</v>
       </c>
       <c r="E8">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="F8">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G8">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J8" t="s">
         <v>30</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>1093.0425</v>
+        <v>1094.229</v>
       </c>
       <c r="B9">
-        <v>92.420000000000073</v>
+        <v>154.55999999999995</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1037,21 +1037,21 @@
         <v>45</v>
       </c>
       <c r="F9">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G9">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>1088.9362499999997</v>
+        <v>1093.0425</v>
       </c>
       <c r="B10">
-        <v>30.349999999999909</v>
+        <v>92.420000000000073</v>
       </c>
       <c r="C10" t="s">
         <v>33</v>
@@ -1060,16 +1060,16 @@
         <v>34</v>
       </c>
       <c r="E10">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F10">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G10">
+        <v>10</v>
+      </c>
+      <c r="H10">
         <v>7</v>
-      </c>
-      <c r="H10">
-        <v>10</v>
       </c>
       <c r="J10" t="s">
         <v>35</v>
@@ -1080,10 +1080,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1049.76</v>
+        <v>1042.3662499999998</v>
       </c>
       <c r="B11">
-        <v>-4.5699999999999363</v>
+        <v>-16.220000000000027</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1092,16 +1092,16 @@
         <v>37</v>
       </c>
       <c r="E11">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="F11">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H11">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J11" t="s">
         <v>38</v>

</xml_diff>